<commit_message>
Rebuild ERG Viewer v2 workflow
</commit_message>
<xml_diff>
--- a/docs/examples/demo-cko-1_FERG.xlsx
+++ b/docs/examples/demo-cko-1_FERG.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C440"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -517,7 +517,7 @@
         <v>[R_01_闪光]</v>
       </c>
       <c r="C11" t="str">
-        <v>白色光: 0.01 cd·s/m²</v>
+        <v>b白色光:0.01cd.m-2,5ms</v>
       </c>
     </row>
     <row r="12">
@@ -528,7 +528,7 @@
         <v>[R_01_闪光背景]</v>
       </c>
       <c r="C12" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="13">
@@ -539,7 +539,7 @@
         <v>[R_01_采样]</v>
       </c>
       <c r="C13" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="14">
@@ -550,7 +550,7 @@
         <v>[R_01_分析时间]</v>
       </c>
       <c r="C14" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="15">
@@ -572,7 +572,7 @@
         <v>[R_01_详细数据(uv)]</v>
       </c>
       <c r="C16" t="str">
-        <v>-2.01,-2.98,-2.43,-0.62,1.5,2.85,2.74,1.22,-0.93,-2.6,-2.93,-1.76,0.32,2.23,3,2.22,0.31,-1.77,-2.94,-2.59,-0.92,1.23,2.74,2.85,1.49,-0.64,-2.44,-2.99,-2,0.01,2.01,2.98,2.41,0.59,-1.53,-2.88,-2.76,-1.24,0.9,2.56,2.87,1.67,-0.42,-2.35,-3.13,-2.37,-0.48,1.56,2.67,2.27,0.53,-1.68,-3.26,-3.44,-2.18,-0.16,1.5,1.9,0.74,-1.46,-3.67,-4.86,-4.54,-3.01,-1.21,-0.23,-0.75,-2.71,-5.32,-7.48,-8.34,-7.75,-6.3,-5.08,-5.07,-6.64,-9.4,-12.35,-14.42,-15.03,-14.35,-13.25,-12.84,-13.87,-16.39,-19.68,-22.65,-24.37,-24.55,-23.72,-22.88,-23.07,-24.75,-27.62,-30.73,-32.98,-33.68,-32.88,-31.37,-30.25,-30.34,-31.8,-33.99,-35.84,-36.37,-35.17,-32.66,-29.82,-27.7,-26.9,-27.21,-27.77,-27.46,-25.52,-21.91,-17.34,-12.91,-9.53,-7.49,-6.26,-4.81,-2.13,2.26,8.05,14.29,19.88,24.14,27.13,29.65,32.78,37.36,43.54,50.68,57.7,63.62,68.05,71.41,74.67,78.89,84.64,91.72,99.26,106.13,111.58,115.54,118.74,122.26,127.01,133.23,140.41,147.49,153.44,157.78,160.81,163.47,166.82,171.54,177.55,184.02,189.86,194.21,196.91,198.58,200.3,203.01,207.1,212.12,217.08,220.91,223.03,223.63,223.57,223.97,225.57,228.4,231.74,234.49,235.74,235.23,233.48,231.54,230.43,230.62,231.8,233.03,233.23,231.73,228.62,224.7,221.1,218.64,217.49,217.02,216.16,213.95,210.04,204.85,199.39,194.74,191.47,189.4,187.64,185.12,181.08,175.5,169.12,163.05,158.2,154.84,152.44,149.97,146.42,141.33,135.03,128.47,122.74,118.52,115.73,113.56,110.92,106.98,101.6,95.43,89.54,84.91,81.9,80.09,78.48,76.02,72.13,67.03,61.6,56.95,53.83,52.26,51.52,50.51,48.32,44.7,40.2,35.85,32.67,31.13,30.89,31.01,30.41,28.41,25.11,21.33,18.15,16.42,16.25,17.02,17.64,17.15,15.18,12.17,9.11,7.07,6.59,7.47,8.83,9.54,8.87,6.79,4.03,1.69,0.67,1.2,2.75,4.26,4.72,3.67,1.43,-1.05,-2.69,-2.82,-1.56,0.29,1.61,1.57,0.06,-2.3,-4.43,-5.36,-4.75,-3.03,-1.21,-0.34,-0.99,-2.94,-5.31,-6.98,-7.22,-6.02,-4.1,-2.57,-2.33,-3.62,-5.88,-8.09,-9.21,-8.8,-7.19,-5.32,-4.29,-4.76,-6.6,-9.01,-10.89,-11.39,-10.42,-8.6,-7.01,-6.62,-7.78,-10.04,-12.4,-13.79,-13.67,-12.26,-10.44,-9.33,-9.65,-11.43,-13.91,-16.01,-16.82,-16.11,-14.43,-12.83,-12.33,-13.36,-15.6,-18.1,-19.76,-19.93,-18.73,-16.99,-15.79,-15.97,-17.64,-20.16,-22.44,-23.52,-23.07,-21.53,-19.91,-19.26,-20.13,-22.3,-24.87,-26.74,-27.17,-26.16,-24.45,-23.13,-23.12,-24.62,-27.09,-29.48,-30.77,-30.52,-29.07,-27.38,-26.53,-27.17,-29.17,-31.72,-33.71,-34.32,-33.43,-31.7,-30.22,-29.93,-31.17,-33.49,-35.88,-37.29,-37.16,-35.74,-33.92,-32.8,-33.1,-34.84,-37.26,-39.27,-39.97,-39.14,-37.33,-35.6,-34.96,-35.85,-37.91,-40.2,-41.64,-41.57,-40.11,-38.11,-36.65,-36.56,-37.94,-40.14,-42.08,-42.8,-41.97,-40.05,-38.04,-37,-37.47,-39.22,-41.34,-42.73,-42.68,-41.17,-38.96,-37.15,-36.63,-37.62,-39.56,-41.39,-42.11,-41.27,-39.23,-36.96,-35.53,-35.58,-36.99,-38.92,-40.27,-40.24,-38.7,-36.34,-34.22,-33.3,-33.91,-35.59,-37.32,-38.06,-37.27,-35.18,-32.71,-30.95,-30.62,-31.72,-33.5,-34.85,-34.9,-33.41,-30.97,-28.63,-27.39,-27.68,-29.15,-30.84,-31.67,-31,-28.96,-26.39,-24.39,-23.77,-24.64,-26.32,-27.74,-27.94,-26.61,-24.2,-21.73,-20.26,-20.31,-21.65,-23.36,-24.34,-23.88,-21.99,-19.43,-17.3,-16.47,-17.17,-18.82,-20.36,-20.8,-19.69,-17.42,-14.93,-13.31,-13.19,-14.44,-16.21,-17.41,-17.23,-15.57,-13.1,-10.91,-9.94,-10.51,-12.16,-13.86,-14.57,-13.76</v>
+        <v>-13.75,-13.52,-10.77,-6.58,-2.61,-0.46,-0.94,-3.74,-7.58,-10.74,-11.78,-10.17,-6.5,-2.22,0.92,1.7,-0.15,-3.76,-7.52,-9.78,-9.52,-6.78,-2.67,1.11,3.01,2.26,-0.79,-4.82,-8.11,-9.25,-7.74,-4.24,-0.21,2.62,3.03,0.83,-3.07,-7.05,-9.48,-9.35,-6.77,-2.9,0.58,2.16,1.06,-2.3,-6.56,-10,-11.22,-9.76,-6.43,-2.56,-0.02,0.2,-2.19,-6.33,-10.43,-12.84,-12.55,-10.08,-6.11,-2.79,-1.38,-2.59,-6.13,-10.61,-13.58,-14.62,-13.18,-10.41,-6.52,-4.03,-3.07,-6.03,-10.11,-14.72,-17,-17.02,-14.26,-9.33,-5.93,-6.37,-7.16,-10.05,-15.48,-18.97,-18.94,-16.34,-14.78,-11.7,-10.13,-7.9,-9.86,-13.11,-18.37,-22.82,-23.38,-16.97,-17.63,-13.61,-12.07,-12.57,-18.37,-16.61,-20.85,-24.98,-17.29,-16.52,-12.96,-6.04,-5.42,-9.01,-13.59,-11.57,-11.76,-15.6,-15.24,-3.39,-5.68,7.36,4.95,-1.65,-3.84,-6.52,-6.99,-2.88,1.54,9.31,12.12,17.2,21.72,18.05,20.6,13.71,28.89,25.62,34.24,34.14,41.74,41.76,40.45,38.67,47.91,48.53,45.62,60.52,57.35,63.12,72.2,71.68,83.08,88.07,74.14,80.08,93.58,102.39,93.53,96.24,96.73,98.51,99.34,121.88,96.73,128.77,119.87,117.57,144.5,137.99,135.14,117.67,143.21,149.01,124.85,134.26,137.32,164.24,174.43,164.95,153.39,151.04,147.94,150.86,168.56,147.51,166.48,162.92,166.54,178.19,143.71,148.75,164.18,167.04,147.56,167.34,173.04,179.77,148.72,160.95,169.71,146.91,150.47,145.61,172.5,144.39,147.9,170.91,143.14,153.61,134.68,131.39,126,151.15,146.6,143.46,132.58,143.03,117.58,115.38,101.09,123.81,119.79,114.84,106.34,110.54,99.89,104.28,95.62,82.03,75.47,89.57,75.97,94.09,89.54,90.42,70.74,68.31,70.61,66.82,59.01,59.73,63.5,64.78,62.84,62.04,48.71,47.7,38.27,38.83,39.58,36.47,40.97,45.85,37.43,38.82,32.6,23.37,25.95,22.39,21.06,23.58,27.77,29.34,28.7,22.23,18.59,11.81,9.65,14.13,14.58,17.66,20.52,21.93,18.54,13.09,7.54,5.05,6.52,8.77,12.11,14.99,17.04,15.42,12.02,7.02,3.63,2.47,3.77,6.6,11.05,13.17,12.75,11.6,6.72,2.69,0.5,-0.16,2.69,6.65,9.39,11.07,9.23,6.66,1.59,-1.73,-3.59,-0.88,2.58,5.5,7.62,6.95,3.72,0.98,-4.93,-4.97,-5.82,-2.37,0.21,3.54,4.91,4.35,0.59,-5.92,-8.51,-9.32,-9.92,-3.5,-2.28,-0.7,2.56,-1,-5.61,-12.01,-14.77,-11.07,-8.6,-4.82,-3.56,0.69,-3.81,-3.64,-13.64,-13.33,-15.86,-10.07,-8.44,-2.13,-0.19,-2.74,-3.24,-12.29,-13.57,-16.76,-16.58,-13.71,-4.97,-1.1,-1.36,-6.81,-5.82,-11.23,-15.2,-18.61,-15.48,-6.25,-3.06,-6.47,-4.09,-4.03,-16.28,-12.26,-15.53,-15.57,-10.3,-14.77,-4.47,-8.6,-7.48,-5.8,-17.41,-18.26,-21.49,-18.26,-6.53,-14.49,-9.7,-13,-6.57,-16.59,-18.27,-19.83,-22.99,-12.75,-19.13,-14.76,-6.16,-13.43,-20.49,-26.99,-27.21,-23.11,-26.06,-12.51,-11.09,-11.41,-8.02,-16.61,-26.39,-20,-19.25,-31.46,-18.83,-25.95,-16.16,-14.52,-12.13,-27.93,-31.78,-22.54,-21.89,-24.51,-13.75,-21.35,-15.26,-17.74,-21.42,-22.66,-30.42,-20.78,-29.65,-19.42,-25.64,-13.86,-11.12,-13.28,-15.52,-19.46,-21.37,-25.61,-21.43,-19.12,-11.12,-7.41,-7.66,-9.17,-19.85,-15.71,-16.75,-18.31,-16.6,-16.09,-10.97,-10.76,-5.06,-6.09,-14.73,-14.77,-19.01,-8.27,-6.21,-4.96,-2.68,-7.52,-1.21,-11.51,-14.46,-8.33,-13.99,-7.27,-6.13,-2.58,1.94,-1.23,-8.58,-8.43,-14.13,-6.97,-3.36,-5.5,4.17,3.39,-1.41,2.93,-1.53,-8.99,-9.72,-3.82,-5.26,-1.66,3.64,2.42,3.21,-0.66,-4.31,-6.05,-4.65,-5.23,2.97,1.51,3.21,3.47</v>
       </c>
     </row>
     <row r="17">
@@ -583,7 +583,7 @@
         <v>[R_01_标记]</v>
       </c>
       <c r="C17" t="str">
-        <v>a: 17.2ms -52.3uv b: 36.2ms 239.8uv</v>
+        <v>a: 15.8ms -32.3uv b: 33.5ms 104.0uv</v>
       </c>
     </row>
     <row r="18">
@@ -616,7 +616,7 @@
         <v>[L_01_闪光]</v>
       </c>
       <c r="C20" t="str">
-        <v>白色光: 0.01 cd·s/m²</v>
+        <v>b白色光:0.01cd.m-2,5ms</v>
       </c>
     </row>
     <row r="21">
@@ -627,7 +627,7 @@
         <v>[L_01_闪光背景]</v>
       </c>
       <c r="C21" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="22">
@@ -638,7 +638,7 @@
         <v>[L_01_采样]</v>
       </c>
       <c r="C22" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="23">
@@ -649,7 +649,7 @@
         <v>[L_01_分析时间]</v>
       </c>
       <c r="C23" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="24">
@@ -671,7 +671,7 @@
         <v>[L_01_详细数据(uv)]</v>
       </c>
       <c r="C25" t="str">
-        <v>-1.07,-1.99,-2.66,-2.98,-2.91,-2.46,-1.69,-0.7,0.38,1.41,2.26,2.81,3,2.79,2.22,1.36,0.33,-0.75,-1.74,-2.49,-2.92,-2.97,-2.63,-1.95,-1.02,0.05,1.11,2.03,2.68,2.98,2.89,2.42,1.64,0.64,-0.45,-1.48,-2.32,-2.86,-3.04,-2.82,-2.25,-1.39,-0.36,0.7,1.66,2.37,2.76,2.75,2.36,1.61,0.61,-0.52,-1.65,-2.63,-3.36,-3.75,-3.76,-3.42,-2.77,-1.94,-1.05,-0.25,0.33,0.58,0.42,-0.15,-1.12,-2.4,-3.88,-5.43,-6.92,-8.2,-9.19,-9.85,-10.16,-10.19,-10.01,-9.76,-9.57,-9.59,-9.92,-10.64,-11.79,-13.34,-15.23,-17.33,-19.53,-21.66,-23.58,-25.2,-26.42,-27.22,-27.63,-27.73,-27.61,-27.4,-27.23,-27.22,-27.45,-27.95,-28.72,-29.69,-30.75,-31.79,-32.63,-33.14,-33.2,-32.72,-31.66,-30.04,-27.92,-25.4,-22.62,-19.72,-16.83,-14.05,-11.45,-9.05,-6.81,-4.66,-2.49,-0.16,2.47,5.49,9.01,13.06,17.61,22.63,27.98,33.55,39.18,44.73,50.06,55.1,59.82,64.21,68.35,72.33,76.28,80.33,84.61,89.21,94.18,99.53,105.22,111.14,117.19,123.2,129.03,134.55,139.68,144.35,148.57,152.38,155.88,159.19,162.44,165.76,169.25,172.99,177,181.23,185.62,190.04,194.35,198.41,202.08,205.25,207.87,209.9,211.4,212.44,213.14,213.63,214.05,214.52,215.12,215.89,216.82,217.85,218.88,219.79,220.43,220.66,220.39,219.53,218.08,216.05,213.53,210.64,207.51,204.3,201.13,198.12,195.33,192.76,190.39,188.14,185.88,183.5,180.86,177.84,174.39,170.45,166.07,161.29,156.25,151.07,145.91,140.91,136.19,131.83,127.85,124.24,120.93,117.81,114.75,111.63,108.31,104.71,100.78,96.53,92,87.29,82.53,77.86,73.42,69.33,65.69,62.53,59.83,57.54,55.55,53.74,51.96,50.08,47.99,45.62,42.96,40.04,36.93,33.74,30.62,27.7,25.1,22.93,21.22,19.97,19.15,18.64,18.33,18.06,17.71,17.15,16.3,15.11,13.62,11.87,9.97,8.04,6.24,4.69,3.49,2.7,2.34,2.37,2.72,3.25,3.84,4.33,4.61,4.58,4.18,3.42,2.35,1.05,-0.34,-1.69,-2.86,-3.74,-4.25,-4.36,-4.09,-3.5,-2.72,-1.86,-1.07,-0.49,-0.22,-0.32,-0.81,-1.66,-2.77,-4.03,-5.31,-6.47,-7.38,-7.94,-8.13,-7.93,-7.41,-6.66,-5.8,-4.98,-4.34,-3.98,-3.99,-4.4,-5.18,-6.26,-7.54,-8.88,-10.15,-11.2,-11.94,-12.31,-12.29,-11.93,-11.3,-10.54,-9.77,-9.14,-8.76,-8.74,-9.11,-9.86,-10.95,-12.26,-13.68,-15.06,-16.27,-17.19,-17.76,-17.93,-17.74,-17.26,-16.6,-15.9,-15.28,-14.89,-14.83,-15.14,-15.85,-16.91,-18.23,-19.69,-21.15,-22.48,-23.55,-24.27,-24.6,-24.56,-24.19,-23.61,-22.93,-22.3,-21.85,-21.7,-21.91,-22.52,-23.48,-24.74,-26.17,-27.64,-29.01,-30.15,-30.97,-31.4,-31.44,-31.12,-30.55,-29.85,-29.14,-28.57,-28.26,-28.3,-28.72,-29.51,-30.61,-31.92,-33.31,-34.63,-35.76,-36.58,-37.02,-37.06,-36.73,-36.11,-35.3,-34.45,-33.69,-33.16,-32.94,-33.1,-33.63,-34.5,-35.6,-36.82,-38.01,-39.04,-39.79,-40.17,-40.16,-39.75,-39.02,-38.07,-37.03,-36.05,-35.24,-34.73,-34.58,-34.8,-35.38,-36.22,-37.22,-38.23,-39.12,-39.77,-40.07,-39.97,-39.48,-38.63,-37.54,-36.31,-35.09,-34.02,-33.22,-32.76,-32.68,-32.96,-33.55,-34.32,-35.16,-35.93,-36.48,-36.71,-36.56,-36.01,-35.1,-33.91,-32.54,-31.15,-29.87,-28.83,-28.11,-27.78,-27.82,-28.19,-28.8,-29.51,-30.19,-30.71,-30.93,-30.8,-30.27,-29.37,-28.16,-26.74,-25.27,-23.86,-22.66,-21.78,-21.27,-21.14,-21.37,-21.87,-22.53,-23.2,-23.74,-24.04,-24,-23.57,-22.76,-21.62,-20.25,-18.78,-17.34,-16.08,-15.1,-14.49,-14.27,-14.43,-14.89,-15.54,-16.26,-16.89,-17.31,-17.43,-17.16,-16.52,-15.52,-14.27,-12.87,-11.47,-10.21,-9.2,-8.55,-8.28,-8.4,-8.86</v>
+        <v>11.86,15.3,12.87,6.19,-0.59,-3.25,-0.02,7.32,14.52,17.43,14.47,7.6,1.11,-0.91,2.91,10.45,17.35,19.61,16.04,8.93,2.7,1.23,5.51,13.12,19.55,21.08,16.84,9.43,3.43,2.41,7.07,14.62,20.46,21.18,16.17,8.53,2.72,2.22,7.05,14.47,19.8,19.6,13.75,5.85,0.44,0.09,5.56,12.47,17.32,15.95,9.47,1.46,-3.63,-3.7,1.69,9.32,12.37,11.54,3.54,-3.64,-8.12,-8.51,-3.8,2.78,7.88,4.81,-3.35,-11.63,-14.77,-13.24,-6.96,-3.15,0.54,-1.26,-9.64,-16.22,-19.72,-20.36,-13.88,-4.8,-3.07,-5.89,-18.81,-21.09,-28.09,-25.5,-15.34,-6.48,-6.77,-7.9,-12.09,-26.44,-18.29,-15.03,-8.15,-5.94,7,1.02,-11.58,-12.66,-8.29,0.4,3.79,16.75,13.61,10.82,0.01,-2.93,11.03,17.71,19.24,35.97,38.55,30.48,29.74,19.89,30.41,41.08,45.3,58.97,62.56,55.15,51.86,49.16,49.54,64.93,87.2,90.31,88.57,90.4,77.5,71.49,73.89,98.67,94.71,124.26,106.3,123.94,119.26,112.03,111.04,126.9,139.92,150.55,125.83,139.24,134.17,120.6,135.7,125.14,140.61,138.72,159.81,151.48,152.51,137.17,145.76,158.02,158.82,157.75,167.21,157.66,160.98,149.1,171.44,174.38,183.64,192.75,158.03,168,144.75,166.52,159.15,156.34,187.17,158.59,160.86,172.1,142.68,146.62,136.14,165.72,164.94,179.66,161.52,136.01,138.87,137.82,131.96,146.3,137.63,148.73,143.25,133.49,135.35,114.89,134.75,139.31,135.45,128.79,122.71,106.87,94.31,88.35,99.35,111.57,100.87,104.15,101.73,79.18,85.19,79.95,88.37,87.68,86.39,85.1,72,63.91,53.68,57.45,65.59,59.19,69.88,64.44,52.26,39.6,32.4,41.68,40.37,44.67,43.67,40.64,32.96,26.18,17.91,18.97,27.32,32.07,31.57,25.05,17.68,8.64,6.5,9.17,15.28,22.19,21.12,15.19,6.81,1.54,-1.67,3.2,9.1,14.37,15.94,9.75,1.78,-4.76,-5.6,-0.34,6.56,11.4,11.38,4.97,-2.03,-7.24,-7.89,-1.64,5.44,10.94,10.23,3.73,-3.19,-8.18,-7.22,-1.38,6.87,11.92,9.54,4.33,-3.09,-6.84,-6.76,0.58,8.44,11.66,9.6,3.47,-3.69,-8.17,-3.89,2.04,8.54,12.05,9.81,3,-4.26,-8.9,-4.16,0.71,7.82,8.83,6.72,-2.13,-8.05,-11.97,-6.43,0.43,5.41,6.53,2.13,-4.96,-10.1,-14.39,-10.92,-5.17,1.63,2.94,-3.48,-7.14,-18.86,-15.4,-12.86,-9.08,-4.36,-1.97,-4.42,-13.87,-24.72,-20.71,-16.81,-7.87,-5.91,-8.18,-13.64,-17.65,-24.4,-30.48,-18.2,-11.93,-8.13,-5.82,-12.12,-21.66,-24.6,-31.29,-23.02,-17.48,-8.91,-10.64,-14.31,-28.87,-26.99,-30.9,-19.33,-18.28,-12.75,-18.22,-19.38,-26.9,-28.21,-29.03,-19.7,-11.58,-15.22,-12.53,-19.92,-29.83,-25.04,-25.4,-17.11,-9.88,-4.36,-13.45,-14.95,-25.18,-26.55,-28.73,-13.28,-18.94,-12.83,-15.67,-17.46,-27.5,-28.23,-33.79,-18.54,-10.23,-15.83,-17.08,-30.36,-31.05,-31.52,-29.78,-18,-19.22,-6.1,-14.4,-32.54,-33.14,-33.19,-22.37,-25.84,-18.08,-8.94,-19.68,-21.9,-39.75,-39.15,-26.56,-20.75,-16.47,-12.41,-19.34,-29.34,-38.17,-40.28,-24.46,-21.47,-18.33,-19.69,-32.02,-31.68,-44.01,-40.7,-28.18,-24.23,-21.04,-20.16,-26.52,-37.45,-32.53,-36.28,-32.44,-26.14,-20.06,-15,-26.72,-25.34,-33.49,-33.56,-24.74,-12.06,-15.78,-11.84,-23.78,-24.86,-34.09,-27.18,-15.62,-12.6,-10.43,-7.85,-21.68,-22.07,-30.21,-21.05,-9.93,-8.18,-7.89,-10.2,-14.1,-17.46,-20.32,-15.59,-12.16,-0.99,-3.22,-3.58,-12.5,-13.97,-17.8,-13.84,-3.94,-0.84,1.97,-2.26,-7.09,-16.45,-17.72,-9.68,-3.61,5.18,4.11,-1.27,-10.84,-15.55,-13.22,-7.16,-0.01,4.59,3.53,-4.02,-10.21,-16.26,-17.4,-12.56,-5.86,-0.85,-2.56</v>
       </c>
     </row>
     <row r="26">
@@ -682,7 +682,7 @@
         <v>[L_01_标记]</v>
       </c>
       <c r="C26" t="str">
-        <v>a: 17.2ms -49.1uv b: 36.2ms 225.5uv</v>
+        <v>a: 15.6ms -26.8uv b: 33.4ms 134.9uv</v>
       </c>
     </row>
     <row r="27">
@@ -693,7 +693,7 @@
         <v>[R_02_名字]</v>
       </c>
       <c r="C27" t="str">
-        <v>FERG(2)_dMax</v>
+        <v>FERG(2)_dRod</v>
       </c>
     </row>
     <row r="28">
@@ -715,7 +715,7 @@
         <v>[R_02_闪光]</v>
       </c>
       <c r="C29" t="str">
-        <v>白色光: 5.00 cd·s/m²</v>
+        <v>b白色光:0.03cd.m-2,5ms</v>
       </c>
     </row>
     <row r="30">
@@ -726,7 +726,7 @@
         <v>[R_02_闪光背景]</v>
       </c>
       <c r="C30" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="31">
@@ -737,7 +737,7 @@
         <v>[R_02_采样]</v>
       </c>
       <c r="C31" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="32">
@@ -748,7 +748,7 @@
         <v>[R_02_分析时间]</v>
       </c>
       <c r="C32" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="33">
@@ -770,7 +770,7 @@
         <v>[R_02_详细数据(uv)]</v>
       </c>
       <c r="C34" t="str">
-        <v>-1.07,-1.99,-2.66,-2.98,-2.91,-2.46,-1.69,-0.7,0.38,1.41,2.26,2.81,3,2.79,2.22,1.36,0.32,-0.77,-1.75,-2.51,-2.95,-3.01,-2.68,-2.01,-1.09,-0.03,1.01,1.9,2.51,2.78,2.64,2.12,1.27,0.19,-0.99,-2.13,-3.09,-3.78,-4.13,-4.11,-3.77,-3.17,-2.45,-1.73,-1.17,-0.9,-1.02,-1.59,-2.61,-4.05,-5.83,-7.82,-9.88,-11.9,-13.74,-15.34,-16.66,-17.71,-18.56,-19.31,-20.1,-21.05,-22.3,-23.96,-26.07,-28.64,-31.64,-34.97,-38.49,-42.05,-45.49,-48.67,-51.45,-53.76,-55.58,-56.92,-57.85,-58.45,-58.84,-59.12,-59.38,-59.66,-59.98,-60.29,-60.49,-60.45,-60.02,-59.04,-57.36,-54.85,-51.44,-47.11,-41.89,-35.85,-29.11,-21.82,-14.12,-6.16,1.97,10.2,18.5,26.91,35.5,44.37,53.63,63.4,73.76,84.76,96.4,108.64,121.38,134.48,147.78,161.11,174.31,187.26,199.85,212.06,223.89,235.4,246.68,257.85,269.03,280.31,291.77,303.42,315.24,327.16,339.05,350.78,362.17,373.07,383.35,392.9,401.69,409.7,417,423.68,429.85,435.63,441.14,446.48,451.68,456.75,461.64,466.26,470.48,474.15,477.15,479.33,480.61,480.96,480.38,478.94,476.74,473.92,470.63,467.03,463.24,459.35,455.41,451.41,447.31,443.01,438.41,433.39,427.84,421.69,414.91,407.51,399.56,391.18,382.51,373.72,364.97,356.41,348.14,340.24,332.71,325.52,318.59,311.81,305.06,298.21,291.17,283.88,276.33,268.56,260.64,252.71,244.89,237.34,230.19,223.54,217.45,211.92,206.91,202.32,198.04,193.92,189.81,185.59,181.18,176.52,171.62,166.53,161.36,156.21,151.23,146.54,142.25,138.42,135.06,132.13,129.56,127.22,124.98,122.69,120.2,117.44,114.32,110.86,107.09,103.1,99.01,94.96,91.09,87.51,84.31,81.52,79.13,77.08,75.26,73.55,71.8,69.89,67.7,65.17,62.28,59.08,55.63,52.05,48.48,45.07,41.95,39.2,36.88,35.01,33.51,32.32,31.3,30.31,29.21,27.9,26.29,24.34,22.08,19.56,16.89,14.21,11.65,9.35,7.41,5.89,4.81,4.14,3.8,3.66,3.58,3.43,3.08,2.43,1.44,0.1,-1.54,-3.39,-5.32,-7.19,-8.86,-10.23,-11.22,-11.8,-11.98,-11.83,-11.47,-11.03,-10.65,-10.47,-10.59,-11.07,-11.92,-13.13,-14.59,-16.21,-17.82,-19.31,-20.55,-21.44,-21.94,-22.05,-21.84,-21.39,-20.83,-20.3,-19.95,-19.88,-20.17,-20.86,-21.91,-23.27,-24.81,-26.42,-27.94,-29.25,-30.24,-30.86,-31.08,-30.96,-30.58,-30.04,-29.51,-29.1,-28.95,-29.14,-29.72,-30.68,-31.97,-33.48,-35.09,-36.66,-38.05,-39.15,-39.88,-40.22,-40.19,-39.86,-39.34,-38.77,-38.29,-38.03,-38.08,-38.51,-39.32,-40.48,-41.89,-43.43,-44.97,-46.37,-47.5,-48.27,-48.65,-48.65,-48.31,-47.75,-47.09,-46.46,-46.02,-45.85,-46.05,-46.63,-47.56,-48.78,-50.16,-51.58,-52.89,-53.96,-54.69,-55.04,-54.98,-54.57,-53.89,-53.07,-52.24,-51.55,-51.1,-51,-51.27,-51.9,-52.84,-53.98,-55.2,-56.34,-57.29,-57.92,-58.16,-58,-57.47,-56.64,-55.62,-54.55,-53.57,-52.81,-52.36,-52.29,-52.58,-53.21,-54.07,-55.04,-55.99,-56.77,-57.26,-57.4,-57.12,-56.46,-55.48,-54.27,-52.97,-51.72,-50.66,-49.88,-49.47,-49.43,-49.75,-50.33,-51.07,-51.83,-52.46,-52.85,-52.89,-52.54,-51.8,-50.71,-49.36,-47.89,-46.43,-45.12,-44.08,-43.38,-43.07,-43.12,-43.48,-44.03,-44.65,-45.2,-45.53,-45.55,-45.19,-44.44,-43.33,-41.93,-40.38,-38.79,-37.33,-36.1,-35.2,-34.69,-34.56,-34.76,-35.2,-35.75,-36.28,-36.63,-36.71,-36.43,-35.75,-34.71,-33.36,-31.81,-30.2,-28.67,-27.35,-26.34,-25.72,-25.48,-25.6,-25.99,-26.54,-27.11,-27.55,-27.75,-27.61,-27.1,-26.2,-24.97,-23.52,-21.97,-20.45,-19.11,-18.06,-17.38,-17.09,-17.18,-17.58,-18.17,-18.82,-19.39,-19.76,-19.82,-19.5,-18.8,-17.75,-16.45,-15,-13.56,-12.25,-11.2,-10.5,-10.19,-10.27,-10.68</v>
+        <v>-7.48,-5.59,-3.66,-1.84,-0.27,0.93,1.66,1.87,1.54,0.71,-0.55,-2.12,-3.88,-5.66,-7.32,-8.72,-9.74,-10.29,-10.34,-9.88,-8.97,-7.68,-6.14,-4.48,-2.87,-1.43,-0.33,0.36,0.54,0.18,-0.68,-2.01,-3.7,-5.61,-7.63,-9.58,-11.32,-12.7,-13.67,-14.1,-14.04,-13.44,-12.47,-11.06,-9.57,-8.03,-6.6,-5.32,-4.54,-4.08,-4.38,-5,-6.06,-7.73,-9.46,-11.6,-13.65,-15.71,-17.45,-18.79,-19.19,-18.86,-18.76,-18.82,-17.23,-16.84,-15.26,-13.55,-12.5,-10.75,-9.91,-10.5,-11.02,-12.31,-16.86,-18.96,-20.52,-23.87,-24.45,-26.56,-27.08,-26.58,-31.86,-29.35,-32.79,-26.46,-29.56,-27.64,-26.55,-25.69,-23.99,-19.47,-17.13,-19.59,-22.39,-16.92,-20.34,-23.3,-27.95,-28.07,-25.79,-25.63,-29.56,-28.71,-25.84,-25.03,-16.22,-12.82,-13.66,-9.49,-3.41,-1.61,-0.91,1.87,6.03,10.98,10.42,10.35,12.69,11.92,9.78,21.87,16.19,15.74,23.45,32.4,33.71,27.48,38.83,36.38,48.84,47.98,65.89,55.38,74.3,77.64,81.02,68.79,79.27,70.19,75.91,85.67,73.64,92.83,93.23,92.34,92.92,97.65,102.82,93.61,119.02,117.53,116.88,130.79,111.1,130.23,133.53,133.25,130.46,118.99,140.01,148.85,120.01,131.24,148.24,126.09,117.25,123.96,116.69,151.88,151.62,124.21,133.81,138.15,128.24,139.37,131.74,129.9,139.04,156.14,140.58,146.7,119.43,146.21,127.15,129.45,126.11,127.52,107.06,97.51,106.58,103.82,111.83,105.74,102.22,105.87,103.16,95.05,88.08,104.43,85.66,79.08,90.56,73.69,85.07,70.98,71.48,60.77,50.66,58.09,55.89,54.37,47.47,43.86,44.02,36,41.15,42.25,33.52,41.2,35.22,37.62,30.1,27.22,23.59,25.43,16.47,17.1,10.83,7.33,3.86,3.68,2.07,2.99,-1.73,1.15,0.87,1.59,3.81,2.43,4.8,3.04,4.69,3.99,2.65,0.6,-0.44,-2.27,-5.13,-7.01,-9.72,-10.93,-12.03,-13.21,-13.65,-13.1,-11.75,-10.76,-8.93,-7.44,-5.51,-4.49,-3.25,-2.32,-1.57,-2.25,-2.52,-3.65,-5.15,-7.54,-8.99,-10.85,-12.55,-14.19,-14.8,-14.89,-14.6,-14.42,-13.19,-11.16,-10.47,-8.03,-6.11,-6.06,-4.54,-4.19,-4.94,-5.86,-6.01,-7.27,-9.49,-12.94,-13.19,-14.8,-17.96,-19.81,-19.35,-21.09,-19.85,-20.23,-18.41,-15.57,-15.91,-14.12,-13.88,-10.24,-10.53,-11.87,-11.07,-11.78,-13.54,-15.52,-17.5,-18.58,-21.75,-23.86,-25.04,-25.72,-27.75,-26.09,-25.07,-26.78,-27.05,-23.62,-24.37,-17.45,-17.67,-16.65,-15.88,-18.04,-17.63,-22.69,-23.94,-22.29,-22.68,-27.85,-29.13,-29.13,-29.29,-30.43,-33.53,-32.89,-29.8,-25.24,-22.46,-25.79,-20.88,-19.77,-25.2,-22.39,-18.2,-16.63,-22.04,-26.68,-24.13,-24.35,-27.54,-25.45,-33.55,-30.45,-38.82,-38.51,-27.71,-33.28,-27.66,-25.53,-28.92,-21.04,-30.7,-18.44,-19.67,-20.23,-19.06,-21.17,-29.47,-26.96,-34.53,-36.77,-33.42,-38,-40.08,-38.36,-37.82,-41.39,-37.66,-36.01,-33.09,-29.52,-28.64,-35.83,-29.79,-25.4,-33.68,-27.14,-32.08,-36.93,-35.81,-32.7,-40.76,-41.25,-35.18,-43.58,-42.72,-38.55,-48.36,-49.44,-46.82,-45.13,-39.97,-31.87,-29.1,-36.42,-35.2,-32.77,-32.92,-28.2,-35.59,-31.12,-34.37,-33.14,-40.5,-34.64,-42.81,-37.89,-38.08,-46.58,-46.26,-39.73,-39.36,-30.21,-29.56,-35.95,-26.22,-24.67,-26.73,-28.64,-23.5,-22.18,-24.87,-24.57,-25.37,-28.79,-27.3,-32.93,-36.96,-31,-36.13,-37.05,-27.68,-26.98,-24.37,-31.06,-28.96,-22.6,-22.49,-21.29,-21.32,-19.04,-15,-20.75,-21.41,-19.59,-20.87,-24.05,-23.12,-24.12,-24.36,-27.71,-28.06,-30.08,-24.51,-26.39,-24,-24.88,-21.84,-17.64,-14.08,-16.63,-16.57,-13.95,-16.56,-18.08,-18.61,-17.15,-19.57,-22.09,-26.31,-25.48,-28.05,-25.57,-25.93,-28.56,-26.01,-24.17,-23.49,-20.01,-18.43,-18.06,-16.8,-16.13</v>
       </c>
     </row>
     <row r="35">
@@ -781,7 +781,7 @@
         <v>[R_02_标记]</v>
       </c>
       <c r="C35" t="str">
-        <v>a: 19.2ms -104.5uv b: 40.2ms 467.4uv</v>
+        <v>a: 16.2ms -17.9uv b: 37.9ms 38.0uv</v>
       </c>
     </row>
     <row r="36">
@@ -792,7 +792,7 @@
         <v>[L_02_名字]</v>
       </c>
       <c r="C36" t="str">
-        <v>FERG(2)_dMax</v>
+        <v>FERG(2)_dRod</v>
       </c>
     </row>
     <row r="37">
@@ -814,7 +814,7 @@
         <v>[L_02_闪光]</v>
       </c>
       <c r="C38" t="str">
-        <v>白色光: 5.00 cd·s/m²</v>
+        <v>b白色光:0.03cd.m-2,5ms</v>
       </c>
     </row>
     <row r="39">
@@ -825,7 +825,7 @@
         <v>[L_02_闪光背景]</v>
       </c>
       <c r="C39" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="40">
@@ -836,7 +836,7 @@
         <v>[L_02_采样]</v>
       </c>
       <c r="C40" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="41">
@@ -847,7 +847,7 @@
         <v>[L_02_分析时间]</v>
       </c>
       <c r="C41" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="42">
@@ -869,7 +869,7 @@
         <v>[L_02_详细数据(uv)]</v>
       </c>
       <c r="C43" t="str">
-        <v>0.02,0.04,0.06,0.08,0.1,0.12,0.14,0.16,0.18,0.2,0.22,0.24,0.26,0.28,0.3,0.32,0.34,0.36,0.37,0.39,0.4,0.42,0.43,0.44,0.44,0.45,0.45,0.44,0.43,0.41,0.39,0.36,0.31,0.26,0.19,0.1,0,-0.13,-0.28,-0.45,-0.66,-0.9,-1.18,-1.5,-1.87,-2.29,-2.77,-3.31,-3.92,-4.6,-5.36,-6.2,-7.13,-8.16,-9.27,-10.49,-11.81,-13.24,-14.77,-16.4,-18.14,-19.98,-21.91,-23.93,-26.03,-28.21,-30.44,-32.72,-35.02,-37.34,-39.65,-41.93,-44.16,-46.31,-48.35,-50.26,-52.01,-53.57,-54.91,-56,-56.81,-57.31,-57.47,-57.27,-56.68,-55.67,-54.24,-52.34,-49.98,-47.14,-43.8,-39.96,-35.61,-30.76,-25.4,-19.54,-13.19,-6.35,0.95,8.71,16.89,25.5,34.49,43.86,53.57,63.6,73.92,84.5,95.32,106.36,117.57,128.94,140.44,152.04,163.72,175.45,187.2,198.95,210.68,222.37,233.98,245.5,256.91,268.19,279.3,290.24,300.98,311.5,321.78,331.8,341.54,350.98,360.1,368.88,377.31,385.36,393.02,400.27,407.1,413.48,419.42,424.88,429.87,434.36,438.36,441.85,444.83,447.29,449.23,450.65,451.55,451.94,451.81,451.17,450.03,448.41,446.3,443.74,440.72,437.27,433.4,429.13,424.49,419.49,414.16,408.51,402.58,396.39,389.96,383.31,376.47,369.47,362.33,355.08,347.73,340.32,332.85,325.37,317.88,310.41,302.97,295.59,288.27,281.04,273.91,266.89,259.99,253.23,246.6,240.12,233.8,227.63,221.63,215.79,210.11,204.6,199.25,194.07,189.04,184.17,179.45,174.88,170.45,166.15,161.99,157.95,154.02,150.21,146.5,142.88,139.35,135.91,132.54,129.24,126.01,122.84,119.71,116.64,113.61,110.62,107.67,104.75,101.86,99,96.17,93.35,90.57,87.8,85.06,82.34,79.64,76.96,74.31,71.68,69.08,66.5,63.96,61.44,58.95,56.5,54.09,51.71,49.37,47.07,44.81,42.6,40.43,38.31,36.24,34.21,32.24,30.32,28.44,26.62,24.86,23.14,21.48,19.87,18.31,16.8,15.34,13.94,12.58,11.27,10.01,8.8,7.62,6.5,5.41,4.37,3.36,2.39,1.46,0.56,-0.3,-1.14,-1.95,-2.72,-3.48,-4.2,-4.91,-5.59,-6.25,-6.9,-7.53,-8.14,-8.74,-9.32,-9.89,-10.46,-11.01,-11.55,-12.09,-12.62,-13.14,-13.66,-14.17,-14.68,-15.18,-15.69,-16.19,-16.69,-17.19,-17.69,-18.18,-18.68,-19.18,-19.68,-20.18,-20.68,-21.18,-21.68,-22.18,-22.68,-23.19,-23.69,-24.2,-24.71,-25.22,-25.73,-26.24,-26.75,-27.26,-27.77,-28.28,-28.8,-29.31,-29.82,-30.33,-30.84,-31.35,-31.86,-32.37,-32.87,-33.38,-33.88,-34.38,-34.87,-35.37,-35.86,-36.34,-36.82,-37.3,-37.78,-38.25,-38.71,-39.17,-39.63,-40.07,-40.52,-40.95,-41.38,-41.81,-42.22,-42.63,-43.03,-43.42,-43.81,-44.19,-44.55,-44.91,-45.26,-45.61,-45.94,-46.26,-46.57,-46.87,-47.16,-47.44,-47.71,-47.97,-48.22,-48.46,-48.68,-48.9,-49.1,-49.29,-49.47,-49.63,-49.79,-49.93,-50.06,-50.17,-50.28,-50.37,-50.45,-50.51,-50.57,-50.61,-50.63,-50.65,-50.65,-50.64,-50.61,-50.58,-50.53,-50.47,-50.39,-50.3,-50.2,-50.09,-49.97,-49.83,-49.68,-49.52,-49.35,-49.17,-48.97,-48.76,-48.54,-48.31,-48.07,-47.82,-47.56,-47.29,-47.01,-46.72,-46.42,-46.11,-45.79,-45.46,-45.12,-44.77,-44.42,-44.06,-43.69,-43.31,-42.92,-42.53,-42.13,-41.73,-41.32,-40.9,-40.48,-40.05,-39.62,-39.18,-38.74,-38.29,-37.84,-37.39,-36.93,-36.47,-36.01,-35.54,-35.07,-34.6,-34.13,-33.66,-33.18,-32.71,-32.23,-31.76,-31.28,-30.8,-30.33,-29.85,-29.38,-28.9,-28.43,-27.96,-27.49,-27.02,-26.56,-26.1,-25.64,-25.18,-24.72,-24.27,-23.82,-23.38,-22.93,-22.5,-22.06,-21.63,-21.21,-20.78,-20.37,-19.95,-19.54,-19.14,-18.74,-18.35,-17.96,-17.58,-17.2,-16.82,-16.45,-16.09,-15.73,-15.38,-15.04,-14.7,-14.36,-14.03,-13.71,-13.39,-13.08,-12.77,-12.47</v>
+        <v>2.58,6.5,11.01,15.34,18.77,20.73,20.91,19.31,16.26,12.34,8.27,4.82,2.62,2.08,3.33,6.15,10.05,14.33,18.23,21.05,22.29,21.7,19.38,15.74,11.38,7.08,3.57,1.44,1.05,2.41,5.25,9,12.96,16.37,18.55,19.07,17.77,14.84,10.73,6.11,1.76,-1.61,-3.46,-3.52,-1.85,1.2,5.02,8.88,12.01,13.81,13.9,12.22,8.99,4.76,0.26,-3.77,-6.65,-7.92,-7.36,-5.07,-1.6,2.51,6.5,9.64,11.12,10.96,9.17,5.74,1.68,-2.52,-6.14,-8.37,-8.97,-7.61,-5.15,-1.21,2.85,6.5,10.03,10.59,9.54,7.05,3.27,-0.25,-4.51,-7.67,-10.71,-11.49,-10.52,-7.85,-4.46,-0.04,4.89,5.25,6.91,3.11,2.62,-5.3,-9.67,-11.87,-12.85,-17.69,-18.57,-18.53,-15.67,-12.52,-7.99,-3.64,-1.04,-0.34,-1.54,-9.85,-7.51,-17.43,-20.28,-24.49,-17.67,-24.43,-18.02,-15.12,-8.38,-2.21,-2.03,4.63,0.33,5.11,4.66,3.72,-0.47,0.34,-1.71,2.94,3.6,5.94,14.09,19.29,31.74,28.7,35.21,39.32,43.36,42.26,40.11,34.69,28.62,40.44,35.36,41.72,44.51,59.57,64.82,68.02,77.92,82.49,96.83,84.16,80.02,91.6,87.68,82.67,98.3,101.43,91.25,91.33,111.4,122.62,137.8,143.74,132.8,144.73,142.87,146.63,118.89,133.86,118.42,123.72,132.59,134.84,137.87,134.66,174.09,176.7,161.74,153.51,159.65,150.5,147.69,158.38,149.58,160.06,151.65,157.12,137.1,150,171.48,171.26,162.6,164.49,173.95,163.57,139.59,130.15,148.62,119.61,122.64,140.93,122.35,141.77,122.71,123.52,121.37,118.29,132.07,113.46,124.53,113.68,100.95,99.82,82.7,86.74,86.71,71.09,74.44,77.85,86,91.71,88.57,75.77,76.67,68.78,66.91,56.3,45.22,47.8,43.63,34.91,39.32,42.7,37.24,45.18,40.43,41.75,43.07,35.32,30.7,26.63,18.46,14.82,13.69,9.4,10.78,13.19,13.37,18.68,22.06,20.38,21.33,20.61,18.4,14.37,9.69,3.53,1.96,-0.37,-1.99,-0.43,2.55,6.47,10.37,13.19,15.53,16.86,14.8,12.74,7.7,3.72,-0.66,-4.12,-4.75,-4.49,-3.19,0.46,4.3,8.21,11.07,13.6,13.35,10.82,8.53,3.63,-1.42,-5.29,-7.79,-9.72,-8.62,-6.13,-3.1,0.66,4.3,6.14,8.35,7.32,5,0.28,-2.98,-8.98,-11.38,-15.54,-15.15,-15.66,-12.89,-9.09,-6.8,-3.12,0.94,-0.39,-0.54,-2.81,-7.93,-11.36,-15.95,-21.2,-23.29,-20.87,-21.5,-18.33,-14.42,-9.68,-8.46,-5.2,-5.73,-4.77,-9.35,-10.98,-15.53,-19.44,-21.32,-25.94,-24.9,-20.28,-19.68,-13.74,-9.06,-6.13,-4.29,-6.61,-9.4,-11.95,-12.38,-16.04,-20.49,-23.52,-27.27,-20.68,-20.61,-19.51,-13.58,-5.84,-4.91,-7.92,-8.39,-3.74,-11.34,-11.31,-22.69,-22.35,-21.83,-25.62,-27.16,-26.64,-20.76,-16.73,-15.99,-10.75,-3.49,-9.03,-6.25,-14.96,-19.79,-26.17,-23.8,-32.43,-25.4,-28.85,-27.53,-23.43,-22.65,-19.2,-19.56,-11.67,-20.64,-14.02,-22.55,-34.77,-35.5,-30.14,-35.74,-37.52,-41.88,-28.53,-36.28,-29.29,-19.82,-19.58,-26.31,-17.12,-32.38,-30.89,-42.01,-46.57,-48.73,-46.56,-50.02,-44.4,-37.21,-34.48,-22.57,-30.66,-27.5,-21.15,-31.23,-32.63,-30.42,-34.39,-36.62,-44.45,-41.81,-44.98,-40.51,-29.12,-33.03,-28.08,-22.07,-23.1,-28.43,-25.5,-22.22,-31.34,-33.96,-36.27,-38.16,-39.39,-33.2,-31.15,-33.19,-16.7,-12.57,-15.57,-14.29,-19.94,-13.44,-27.21,-20.58,-27.37,-25.49,-36.63,-29.92,-24.96,-24.35,-17,-17.75,-13.16,-15.17,-8.87,-15.07,-18.34,-20.44,-26.44,-25.26,-32.2,-33.53,-28.79,-29.82,-25.65,-15.62,-10.04,-7.18,-9.03,-7.02,-10.06,-12.77,-16.22,-25.52,-24.41,-33.01,-28.29,-31.84,-24.1,-20.34,-18.44,-14.73,-9.92,-11.12,-9.35,-15.71,-17.15,-21.65,-28.47,-30.43,-31.74</v>
       </c>
     </row>
     <row r="44">
@@ -880,7 +880,7 @@
         <v>[L_02_标记]</v>
       </c>
       <c r="C44" t="str">
-        <v>a: 19.2ms -98.3uv b: 40.2ms 439.4uv</v>
+        <v>a: 16.3ms -22.0uv b: 37.8ms 21.9uv</v>
       </c>
     </row>
     <row r="45">
@@ -891,7 +891,7 @@
         <v>[R_03_名字]</v>
       </c>
       <c r="C45" t="str">
-        <v>FERG(3)_dOps</v>
+        <v>FERG(3)_dRod</v>
       </c>
     </row>
     <row r="46">
@@ -913,7 +913,7 @@
         <v>[R_03_闪光]</v>
       </c>
       <c r="C47" t="str">
-        <v>白色光: 5.00 cd·s/m²</v>
+        <v>b白色光:0.10cd.m-2,5ms</v>
       </c>
     </row>
     <row r="48">
@@ -924,7 +924,7 @@
         <v>[R_03_闪光背景]</v>
       </c>
       <c r="C48" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="49">
@@ -935,7 +935,7 @@
         <v>[R_03_采样]</v>
       </c>
       <c r="C49" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="50">
@@ -946,7 +946,7 @@
         <v>[R_03_分析时间]</v>
       </c>
       <c r="C50" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="51">
@@ -968,7 +968,7 @@
         <v>[R_03_详细数据(uv)]</v>
       </c>
       <c r="C52" t="str">
-        <v>-6.13,-6.01,-5.88,-5.75,-5.62,-5.5,-5.41,-5.35,-5.32,-5.33,-5.39,-5.49,-5.64,-5.83,-6.06,-6.3,-6.54,-6.78,-6.98,-7.13,-7.22,-7.22,-7.12,-6.92,-6.62,-6.22,-5.74,-5.18,-4.59,-3.99,-3.43,-2.93,-2.54,-2.3,-2.23,-2.36,-2.71,-3.26,-4.01,-4.93,-5.98,-7.1,-8.22,-9.27,-10.19,-10.88,-11.3,-11.37,-11.07,-10.37,-9.28,-7.84,-6.09,-4.13,-2.05,0.02,1.97,3.64,4.92,5.7,5.89,5.43,4.29,2.5,0.12,-2.75,-5.96,-9.34,-12.69,-15.8,-18.47,-20.48,-21.68,-21.94,-21.17,-19.36,-16.55,-12.86,-8.44,-3.54,1.59,6.64,11.3,15.26,18.26,20.05,20.48,19.43,16.92,13.01,7.89,1.8,-4.92,-11.9,-18.72,-24.98,-30.26,-34.22,-36.56,-37.09,-35.7,-32.42,-27.38,-20.83,-13.1,-4.62,4.12,12.61,20.34,26.83,31.67,34.53,35.21,33.61,29.8,23.95,16.38,7.51,-2.15,-12.05,-21.59,-30.22,-37.42,-42.74,-45.86,-46.58,-44.84,-40.74,-34.49,-26.47,-17.14,-7.05,3.22,13.05,21.89,29.21,34.6,37.76,38.51,36.83,32.86,26.84,19.15,10.26,0.7,-8.95,-18.14,-26.33,-33.07,-37.99,-40.85,-41.52,-40.01,-36.47,-31.13,-24.38,-16.62,-8.34,-0.03,7.82,14.77,20.46,24.6,26.99,27.57,26.37,23.52,19.25,13.88,7.74,1.24,-5.24,-11.32,-16.67,-21.02,-24.15,-25.95,-26.38,-25.48,-23.37,-20.24,-16.32,-11.88,-7.2,-2.58,1.74,5.51,8.55,10.74,11.99,12.3,11.71,10.31,8.23,5.65,2.74,-0.31,-3.3,-6.07,-8.48,-10.41,-11.78,-12.57,-12.75,-12.39,-11.53,-10.26,-8.7,-6.95,-5.13,-3.36,-1.72,-0.32,0.81,1.6,2.06,2.17,1.97,1.5,0.8,-0.05,-1,-1.98,-2.94,-3.81,-4.55,-5.15,-5.56,-5.8,-5.86,-5.76,-5.52,-5.17,-4.74,-4.27,-3.78,-3.32,-2.89,-2.53,-2.25,-2.05,-1.94,-1.91,-1.96,-2.07,-2.23,-2.43,-2.65,-2.87,-3.08,-3.27,-3.43,-3.56,-3.65,-3.7,-3.72,-3.7,-3.66,-3.6,-3.52,-3.44,-3.35,-3.27,-3.2,-3.14,-3.1,-3.07,-3.05,-3.05,-3.07,-3.09,-3.12,-3.16,-3.19,-3.23,-3.27,-3.31,-3.34,-3.36,-3.38,-3.39,-3.4,-3.41,-3.41,-3.41,-3.4,-3.4,-3.4,-3.39,-3.39,-3.39,-3.39,-3.4,-3.41,-3.41,-3.42,-3.43,-3.45,-3.46,-3.47,-3.48,-3.5,-3.51,-3.52,-3.53,-3.54,-3.55,-3.56,-3.58,-3.59,-3.59,-3.6,-3.61,-3.62,-3.63,-3.65,-3.66,-3.67,-3.68,-3.69,-3.7,-3.71,-3.73,-3.74,-3.75,-3.76,-3.78,-3.79,-3.8,-3.81,-3.83,-3.84,-3.85,-3.87,-3.88,-3.89,-3.91,-3.92,-3.93,-3.95,-3.96,-3.98,-3.99,-4,-4.02,-4.03,-4.05,-4.06,-4.08,-4.09,-4.11,-4.12,-4.14,-4.15,-4.17,-4.18,-4.2,-4.21,-4.23,-4.24,-4.26,-4.28,-4.29,-4.31,-4.32,-4.34,-4.36,-4.37,-4.39,-4.41,-4.42,-4.44,-4.46,-4.47,-4.49,-4.51,-4.52,-4.54,-4.56,-4.58,-4.59,-4.61,-4.63,-4.65,-4.66,-4.68,-4.7,-4.72,-4.74,-4.75,-4.77,-4.79,-4.81,-4.83,-4.85,-4.86,-4.88,-4.9,-4.92,-4.94,-4.96,-4.98,-4.99,-5.01,-5.03,-5.05,-5.07,-5.09,-5.11,-5.13,-5.15,-5.17,-5.19,-5.21,-5.22,-5.24,-5.26,-5.28,-5.3,-5.32,-5.34,-5.36,-5.38,-5.4,-5.42,-5.44,-5.46,-5.48,-5.5,-5.52,-5.54,-5.56,-5.58,-5.6,-5.62,-5.64,-5.66,-5.68,-5.7,-5.72,-5.74,-5.76,-5.78,-5.8,-5.82,-5.84,-5.86,-5.88,-5.9,-5.93,-5.95,-5.97,-5.99,-6.01,-6.03,-6.05,-6.07,-6.09,-6.11,-6.13,-6.15,-6.17,-6.19,-6.21,-6.23,-6.25,-6.27,-6.29,-6.31,-6.33,-6.35,-6.37,-6.39,-6.42,-6.44,-6.46,-6.48,-6.5,-6.52,-6.54,-6.56,-6.58,-6.6,-6.62,-6.64,-6.66,-6.68,-6.7,-6.72,-6.74,-6.76,-6.78,-6.8,-6.82,-6.84,-6.86,-6.88,-6.9,-6.92,-6.94</v>
+        <v>-17.65,-17.35,-17.04,-16.72,-16.37,-16.01,-15.65,-15.27,-14.88,-14.49,-14.1,-13.7,-13.31,-12.92,-12.54,-12.17,-11.81,-11.46,-11.12,-10.81,-10.51,-10.23,-9.98,-9.75,-9.55,-9.37,-9.22,-9.1,-9.01,-8.95,-8.92,-8.92,-8.95,-9.01,-9.1,-9.23,-9.38,-9.55,-9.76,-9.99,-10.25,-10.53,-10.82,-11.14,-11.48,-11.83,-12.19,-12.56,-12.95,-13.34,-13.74,-14.15,-14.55,-14.94,-15.34,-15.7,-16.13,-16.46,-16.85,-17.24,-17.52,-17.86,-18.27,-18.61,-18.91,-19.01,-19.39,-19.36,-19.94,-20.18,-20.55,-20.52,-20.37,-21.07,-21.5,-21.04,-21.77,-21.48,-21.63,-21.47,-23.58,-21.84,-22.05,-24.75,-24.7,-23.45,-23.29,-25.13,-27.22,-25.67,-24.42,-28.85,-26.96,-29.78,-25.44,-31.28,-29.8,-27.22,-27.69,-31.62,-26.05,-32.15,-34.08,-28.51,-29.15,-26.34,-30.54,-25.67,-26.54,-32.72,-29.55,-31.32,-24.55,-26.56,-23.22,-27.48,-22.07,-21.27,-23.12,-18.58,-16.43,-13.58,-15.51,-10.82,-6.38,-6.6,-8.05,-0.26,-3.3,5.1,7.86,10.28,7.37,11.86,13.24,18.8,23.06,27.03,20.41,25.67,27.04,42.44,36.04,42.64,50.74,56.83,47.85,65.08,63.45,66.56,56.26,72.05,84.04,68.45,78.64,86.98,81.61,81.6,81.41,107.51,90.2,94.62,112.73,117.37,118.33,124.76,114.26,125.64,135.26,127.45,125.09,127.46,125.35,127.16,130.42,158.59,145.31,156.88,140.25,136.39,145.43,148.87,154.46,144.03,145.31,143.47,143.11,145.03,130.69,143.37,133.12,125.37,137.47,138.6,136.52,143.06,119.23,131.16,111.12,128.97,108.01,119.06,104.68,115.77,109.34,87.81,94.26,102.88,87.31,83.62,78.68,71.6,80.05,74.98,66.55,58.41,58.34,60.37,53.43,53.62,45.36,35.3,34.56,29.99,34.63,32.21,28.84,27.75,18.73,15.28,15.92,10.83,12,8.37,10.75,5.06,6,3.86,5.37,0.14,1.27,-1.51,-0.53,-1.1,-0.99,-3.13,-1.66,-2.66,-2.64,-2.33,-2.6,-2.85,-2.54,-2.49,-3.01,-1.88,-2.13,-1.64,-2.01,-1.04,-0.93,-0.55,-0.31,0.14,0.08,0.16,0.45,1.05,1.09,1.54,1.58,1.66,1.89,1.69,1.52,1.84,0.93,1.33,1.39,0.68,0.47,-0.05,-0.03,-0.92,-0.97,-2.52,-2.42,-2.8,-3.43,-3.83,-4.48,-5.34,-7.14,-7.96,-7.77,-8.33,-9.82,-11.51,-11.08,-13.07,-12,-13.43,-15.35,-15.59,-15.34,-15.87,-17.31,-16.94,-18.83,-20.38,-18.37,-21.12,-21.87,-20.08,-20.17,-21.85,-22.45,-20.87,-21.57,-23.41,-22.48,-20.24,-21.44,-23.65,-19.97,-23.37,-21.3,-20.78,-21.36,-19.77,-19.57,-19.9,-16.31,-15.66,-20.43,-19,-17.95,-19,-16.45,-16.58,-12.39,-16.05,-12.09,-12.11,-11.66,-8.91,-11.65,-13.47,-10.29,-7.5,-11.73,-9.87,-7.51,-11.95,-14.18,-6.65,-10.87,-5.98,-14.83,-14.87,-6.92,-7.81,-14.16,-10.08,-12.04,-10.21,-18.27,-14.48,-10.95,-12.42,-17.1,-23.38,-21.12,-19.07,-20.08,-24.85,-20.49,-26.56,-21.14,-31.08,-31.62,-30.37,-27.57,-34.31,-25.7,-31.78,-35.22,-28.74,-39.01,-33.98,-28.66,-33.63,-30.15,-40.39,-38.83,-37.97,-42.9,-42.74,-39.41,-40.82,-32.38,-43.45,-44.64,-34.69,-37.27,-35.56,-40.55,-40.07,-42.14,-40.71,-29.16,-31.1,-30.54,-27.71,-28.01,-25.4,-34.61,-26.13,-31.57,-32.01,-26.24,-33.71,-30.81,-25.7,-26.43,-22.05,-25.37,-25.69,-24.41,-17.27,-16.89,-13.88,-14.38,-18.51,-17.8,-13.76,-12.11,-14.49,-19.79,-14.74,-9.1,-18.95,-14.76,-8.34,-7.28,-17.01,-9.57,-9.23,-16.57,-17.26,-8.56,-16.21,-9.76,-8.29,-16.7,-16.7,-13.47,-17.59,-12.71,-12.3,-12.8,-13.64,-15.73,-17.63,-20.55,-19.2,-20.85,-22.58,-19.14,-22.08,-17.34,-21.31,-18.03,-18.34,-21.37,-21.62,-20.44,-19.8,-22.22,-22.75,-25.11,-22.62,-23.29,-23.03,-20.63,-20.97,-18.79,-20.83,-20.96,-18.65,-18.79,-19.42,-19.81,-19.06,-14.51,-14.16,-16.23,-13.9,-11.94,-13.23</v>
       </c>
     </row>
     <row r="53">
@@ -979,7 +979,7 @@
         <v>[R_03_标记]</v>
       </c>
       <c r="C53" t="str">
-        <v>80.4uv</v>
+        <v>a: 19.1ms -18.8uv b: 41.2ms 114.3uv</v>
       </c>
     </row>
     <row r="54">
@@ -990,7 +990,7 @@
         <v>[L_03_名字]</v>
       </c>
       <c r="C54" t="str">
-        <v>FERG(3)_dOps</v>
+        <v>FERG(3)_dRod</v>
       </c>
     </row>
     <row r="55">
@@ -1012,7 +1012,7 @@
         <v>[L_03_闪光]</v>
       </c>
       <c r="C56" t="str">
-        <v>白色光: 5.00 cd·s/m²</v>
+        <v>b白色光:0.10cd.m-2,5ms</v>
       </c>
     </row>
     <row r="57">
@@ -1023,7 +1023,7 @@
         <v>[L_03_闪光背景]</v>
       </c>
       <c r="C57" t="str">
-        <v>无背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="58">
@@ -1034,7 +1034,7 @@
         <v>[L_03_采样]</v>
       </c>
       <c r="C58" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="59">
@@ -1045,7 +1045,7 @@
         <v>[L_03_分析时间]</v>
       </c>
       <c r="C59" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="60">
@@ -1067,7 +1067,7 @@
         <v>[L_03_详细数据(uv)]</v>
       </c>
       <c r="C61" t="str">
-        <v>-4.68,-3.63,-2.87,-2.49,-2.52,-2.98,-3.77,-4.8,-5.91,-6.96,-7.81,-8.34,-8.5,-8.29,-7.75,-6.98,-6.11,-5.28,-4.62,-4.24,-4.19,-4.49,-5.07,-5.85,-6.69,-7.44,-7.95,-8.12,-7.86,-7.19,-6.13,-4.82,-3.41,-2.08,-1.02,-0.38,-0.31,-0.84,-1.97,-3.62,-5.63,-7.82,-9.97,-11.85,-13.27,-14.09,-14.23,-13.67,-12.46,-10.72,-8.61,-6.31,-4.02,-1.9,-0.1,1.3,2.25,2.74,2.81,2.5,1.88,1,-0.1,-1.39,-2.89,-4.59,-6.51,-8.63,-10.92,-13.31,-15.67,-17.85,-19.65,-20.84,-21.24,-20.66,-19,-16.21,-12.37,-7.65,-2.32,3.26,8.69,13.52,17.35,19.8,20.61,19.63,16.85,12.41,6.57,-0.29,-7.7,-15.15,-22.14,-28.19,-32.91,-36,-37.28,-36.69,-34.3,-30.27,-24.87,-18.42,-11.29,-3.86,3.48,10.39,16.52,21.58,25.33,27.57,28.17,27.05,24.21,19.7,13.69,6.42,-1.79,-10.55,-19.37,-27.75,-35.17,-41.12,-45.17,-46.97,-46.31,-43.14,-37.58,-29.94,-20.67,-10.34,0.36,10.72,20.04,27.7,33.19,36.17,36.48,34.15,29.39,22.6,14.29,5.03,-4.53,-13.78,-22.17,-29.25,-34.66,-38.2,-39.79,-39.46,-37.37,-33.73,-28.84,-23.01,-16.58,-9.86,-3.19,3.15,8.89,13.79,17.63,20.26,21.54,21.4,19.83,16.9,12.72,7.52,1.57,-4.77,-11.13,-17.1,-22.28,-26.35,-29.01,-30.11,-29.59,-27.51,-24.06,-19.54,-14.31,-8.8,-3.43,1.42,5.41,8.3,9.97,10.41,9.69,8.01,5.61,2.76,-0.25,-3.17,-5.79,-7.98,-9.66,-10.84,-11.54,-11.87,-11.91,-11.78,-11.54,-11.24,-10.89,-10.48,-9.96,-9.29,-8.42,-7.34,-6.06,-4.64,-3.15,-1.73,-0.5,0.39,0.83,0.76,0.14,-1,-2.54,-4.36,-6.28,-8.09,-9.62,-10.71,-11.25,-11.21,-10.62,-9.56,-8.17,-6.65,-5.17,-3.91,-3.01,-2.57,-2.6,-3.06,-3.87,-4.88,-5.94,-6.88,-7.56,-7.9,-7.86,-7.44,-6.72,-5.82,-4.89,-4.06,-3.48,-3.23,-3.37,-3.88,-4.69,-5.7,-6.76,-7.72,-8.45,-8.82,-8.8,-8.36,-7.57,-6.53,-5.38,-4.28,-3.37,-2.79,-2.62,-2.87,-3.51,-4.46,-5.59,-6.73,-7.73,-8.46,-8.81,-8.73,-8.25,-7.42,-6.37,-5.24,-4.19,-3.37,-2.89,-2.83,-3.18,-3.89,-4.88,-5.99,-7.07,-7.97,-8.56,-8.76,-8.54,-7.93,-7.02,-5.93,-4.82,-3.84,-3.14,-2.8,-2.89,-3.37,-4.2,-5.25,-6.37,-7.41,-8.23,-8.7,-8.76,-8.4,-7.68,-6.69,-5.57,-4.48,-3.58,-2.98,-2.78,-3,-3.6,-4.52,-5.61,-6.72,-7.7,-8.42,-8.76,-8.68,-8.2,-7.38,-6.33,-5.21,-4.16,-3.35,-2.87,-2.81,-3.16,-3.88,-4.86,-5.98,-7.06,-7.97,-8.57,-8.78,-8.57,-7.96,-7.05,-5.97,-4.85,-3.87,-3.15,-2.8,-2.88,-3.35,-4.17,-5.22,-6.34,-7.39,-8.21,-8.69,-8.76,-8.41,-7.7,-6.71,-5.6,-4.51,-3.6,-2.99,-2.78,-2.99,-3.59,-4.5,-5.58,-6.7,-7.68,-8.4,-8.76,-8.69,-8.22,-7.4,-6.36,-5.23,-4.19,-3.36,-2.88,-2.8,-3.14,-3.85,-4.84,-5.95,-7.04,-7.95,-8.56,-8.78,-8.58,-7.98,-7.08,-5.99,-4.88,-3.89,-3.16,-2.81,-2.87,-3.34,-4.15,-5.19,-6.32,-7.36,-8.19,-8.68,-8.76,-8.42,-7.72,-6.74,-5.62,-4.53,-3.62,-3,-2.78,-2.98,-3.57,-4.47,-5.56,-6.67,-7.66,-8.39,-8.75,-8.7,-8.23,-7.42,-6.38,-5.26,-4.21,-3.38,-2.89,-2.8,-3.13,-3.83,-4.81,-5.92,-7.02,-7.94,-8.55,-8.78,-8.59,-8,-7.1,-6.02,-4.9,-3.91,-3.18,-2.81,-2.86,-3.32,-4.13,-5.17,-6.29,-7.34,-8.18,-8.67,-8.76,-8.44,-7.74,-6.76,-5.65,-4.56,-3.64,-3.01,-2.78,-2.97,-3.55,-4.45,-5.53,-6.65,-7.64,-8.38,-8.75,-8.7,-8.25,-7.44,-6.41,-5.29,-4.23,-3.39,-2.89,-2.8,-3.12,-3.81,-4.79,-5.9,-6.99,-7.92,-8.54,-8.78,-8.6,-8.02,-7.13,-6.05</v>
+        <v>6.71,7.66,8.57,9.43,10.24,10.99,11.69,12.33,12.91,13.44,13.89,14.29,14.62,14.89,15.09,15.23,15.3,15.31,15.25,15.14,14.96,14.72,14.42,14.07,13.66,13.2,12.69,12.14,11.54,10.89,10.21,9.5,8.75,7.97,7.17,6.35,5.5,4.64,3.77,2.9,2.01,1.12,0.24,-0.64,-1.51,-2.37,-3.21,-4.05,-4.85,-5.64,-6.4,-7.13,-7.84,-8.52,-9.15,-9.76,-10.32,-10.86,-11.34,-11.81,-12.22,-12.6,-12.92,-13.25,-13.48,-13.7,-13.85,-13.96,-14.14,-14.25,-14.21,-14.18,-14.25,-14.22,-14.09,-13.97,-13.8,-13.82,-13.98,-13.8,-13.41,-13.35,-13.03,-13.01,-12.57,-12.56,-13.37,-12.87,-13.47,-13.08,-13.27,-12.16,-13.38,-12.47,-13.17,-11.71,-14.33,-13.03,-13.76,-15.14,-15.27,-15.44,-12.53,-17.64,-15.68,-16.32,-13.42,-18.65,-13.35,-19.22,-15.09,-19.63,-15.1,-16.79,-15.53,-19.05,-18.03,-17.32,-14.56,-13.43,-10.01,-10.23,-10.98,-13.7,-11.39,-14.36,-7.59,-4.03,-3.02,0.95,2.16,0.88,5.51,3.96,4.66,5.75,11.93,15.06,24.19,21.33,22.5,25.2,32.36,31.17,38.95,41.08,36.13,49.96,53.55,57.91,52.01,58.75,65.43,61.32,78.13,80.84,79.43,85.55,90.23,86.74,94.91,81.16,100.71,104.29,110,115.42,100.92,108.89,112.39,110.56,108.23,116.72,111.77,113.74,120.34,120.44,119.75,143.44,149.8,152.63,153.39,132.77,151.93,139.16,146.55,157.54,140.84,134.62,140.47,154.2,135.33,129.41,157.9,131.44,148.78,152.25,139.69,152.59,139.67,133.07,144.86,151.88,137.18,148.79,136.05,134.59,135.37,126.9,131.96,131.25,116.96,117.34,114.47,124.71,117.04,104.94,106.25,100.19,100.85,102.81,105.72,92.52,88.37,81.51,81.23,90.14,88.89,72.07,84.7,83.78,67.88,68.14,69.56,64.6,68.86,62.16,57.23,55.69,58.4,58.54,60.37,54.62,52.74,48.84,48.09,53.59,47.24,48.54,46.79,46.8,44.4,40.17,40.58,40.52,39.38,38.92,36.28,34.68,35.38,33.81,32.28,30.98,30.2,30.16,29.18,26.55,26.51,24.76,23.45,21.52,20.24,19.11,17.71,17.09,15.32,13.86,13.06,12.09,10.24,8.99,7.32,6.36,5.16,4.06,2.33,0.42,-0.27,-2.01,-2.75,-4.48,-5.65,-6.71,-7.54,-8.21,-9.62,-11,-12.17,-12.6,-13.41,-14.85,-14.28,-15.87,-15.78,-16.87,-17.4,-16.76,-17.78,-17.61,-17.54,-18.7,-18.94,-19.08,-17.35,-18.33,-18.25,-17.29,-17.53,-16.72,-16.22,-16.42,-15.84,-12.62,-11.54,-12.32,-11.03,-10.15,-8.62,-6.79,-5.86,-7.06,-3.57,-6.17,-1.76,-0.85,-2.73,2.35,1.78,3.41,2.01,4.77,3.02,4.62,5.88,8.2,9.31,7.27,10.2,8.94,12.18,13.47,14.73,13.81,12.68,14.6,17.21,16.9,16.56,13.48,13.15,15.73,11.53,17.12,17.33,16.29,13.31,14.25,8.61,9.58,11.24,10.83,4.05,5.16,3.04,2.07,0.72,4.37,-3.73,-0.19,-2.64,0.24,-7.69,-3.19,-3.94,-12.28,-14.18,-7.73,-14.78,-14.94,-14.25,-17.98,-20.39,-23.3,-19.99,-25.75,-29.44,-22.99,-22.86,-27.5,-29.19,-32.64,-36.91,-28.06,-36.91,-32.28,-40.37,-30.11,-33.06,-40.99,-40.94,-34.35,-42.1,-37.84,-36.46,-38.51,-42.6,-29.04,-35.7,-27.85,-33.38,-35.55,-37.99,-26.07,-31.37,-35.34,-31.45,-25.86,-32.71,-27.48,-28.3,-29.16,-24.5,-19.4,-18.19,-23.41,-13.2,-14.3,-22.67,-14.99,-17.09,-18.53,-5.79,-5.55,-15.59,-8.65,-12.64,-3.24,1.05,-4.43,-9.51,-2.95,2.35,2.97,1.67,-0.58,5.19,-3,0.07,9.09,1.36,2.01,9.29,5.67,7.35,8.57,2.9,3.77,6.46,9.07,2.34,6.73,5.96,3.5,10.88,6.3,6.65,2.98,9.22,7.32,7.91,1.88,4.06,6.03,4.07,2.93,5.95,2.05,2.98,0.53,-2.32,2.31,-2,1.29,0.86,0.22,-2.69,-3.86,-1.31,-5.73,-5.17,-4.42</v>
       </c>
     </row>
     <row r="62">
@@ -1078,7 +1078,7 @@
         <v>[L_03_标记]</v>
       </c>
       <c r="C62" t="str">
-        <v>76.9uv</v>
+        <v>a: 19.2ms -17.7uv b: 41.2ms 114.9uv</v>
       </c>
     </row>
     <row r="63">
@@ -1089,7 +1089,7 @@
         <v>[R_04_名字]</v>
       </c>
       <c r="C63" t="str">
-        <v>FERG(4)_lCone</v>
+        <v>FERG(4)_dRod</v>
       </c>
     </row>
     <row r="64">
@@ -1111,7 +1111,7 @@
         <v>[R_04_闪光]</v>
       </c>
       <c r="C65" t="str">
-        <v>白色光: 3.00 cd·s/m²</v>
+        <v>b白色光:0.30cd.m-2,5ms</v>
       </c>
     </row>
     <row r="66">
@@ -1122,7 +1122,7 @@
         <v>[R_04_闪光背景]</v>
       </c>
       <c r="C66" t="str">
-        <v>白色背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="67">
@@ -1133,7 +1133,7 @@
         <v>[R_04_采样]</v>
       </c>
       <c r="C67" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="68">
@@ -1144,7 +1144,7 @@
         <v>[R_04_分析时间]</v>
       </c>
       <c r="C68" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="69">
@@ -1166,7 +1166,7 @@
         <v>[R_04_详细数据(uv)]</v>
       </c>
       <c r="C70" t="str">
-        <v>1.1,2.05,2.71,2.99,2.85,2.31,1.45,0.38,-0.74,-1.76,-2.53,-2.95,-2.95,-2.54,-1.77,-0.75,0.37,1.44,2.31,2.85,2.99,2.72,2.06,1.12,0.01,-1.09,-2.04,-2.71,-2.99,-2.86,-2.32,-1.46,-0.4,0.72,1.74,2.52,2.93,2.94,2.53,1.76,0.74,-0.39,-1.47,-2.35,-2.91,-3.08,-2.83,-2.21,-1.29,-0.23,0.83,1.73,2.33,2.54,2.32,1.68,0.7,-0.51,-1.81,-3.02,-4.03,-4.71,-5.01,-4.94,-4.55,-3.96,-3.3,-2.74,-2.43,-2.5,-3.03,-4.04,-5.48,-7.28,-9.3,-11.39,-13.37,-15.13,-16.55,-17.59,-18.27,-18.64,-18.82,-18.94,-19.16,-19.61,-20.38,-21.51,-23,-24.78,-26.73,-28.68,-30.48,-31.94,-32.95,-33.41,-33.28,-32.6,-31.44,-29.94,-28.23,-26.48,-24.81,-23.33,-22.07,-21.03,-20.12,-19.25,-18.27,-17.03,-15.39,-13.25,-10.57,-7.36,-3.66,0.38,4.64,8.93,13.1,17.02,20.59,23.8,26.66,29.26,31.73,34.22,36.88,39.84,43.2,46.99,51.19,55.73,60.5,65.33,70.07,74.57,78.72,82.46,85.77,88.71,91.38,93.92,96.47,99.19,102.18,105.53,109.25,113.29,117.57,121.94,126.23,130.3,133.98,137.18,139.85,141.99,143.66,144.99,146.1,147.15,148.27,149.58,151.12,152.89,154.85,156.87,158.81,160.52,161.84,162.64,162.84,162.43,161.42,159.92,158.06,155.99,153.87,151.85,150.02,148.43,147.08,145.9,144.77,143.57,142.13,140.33,138.05,135.26,131.94,128.17,124.05,119.74,115.4,111.2,107.27,103.69,100.51,97.7,95.19,92.84,90.51,88.06,85.35,82.31,78.88,75.1,71.03,66.8,62.57,58.49,54.72,51.37,48.51,46.14,44.22,42.64,41.27,39.95,38.54,36.89,34.94,32.65,30.07,27.27,24.39,21.57,18.97,16.73,14.94,13.65,12.83,12.42,12.3,12.31,12.3,12.12,11.64,10.82,9.63,8.12,6.4,4.6,2.88,1.39,0.24,-0.47,-0.74,-0.58,-0.1,0.58,1.31,1.92,2.27,2.27,1.87,1.08,-0.04,-1.36,-2.74,-4.03,-5.07,-5.77,-6.04,-5.9,-5.39,-4.6,-3.69,-2.82,-2.12,-1.74,-1.74,-2.17,-2.99,-4.11,-5.4,-6.72,-7.9,-8.81,-9.35,-9.47,-9.2,-8.58,-7.75,-6.85,-6.03,-5.45,-5.21,-5.38,-5.98,-6.94,-8.18,-9.54,-10.87,-12.02,-12.87,-13.32,-13.36,-13.01,-12.36,-11.54,-10.7,-9.99,-9.56,-9.5,-9.86,-10.63,-11.74,-13.08,-14.49,-15.82,-16.92,-17.69,-18.04,-17.98,-17.55,-16.86,-16.04,-15.25,-14.65,-14.35,-14.44,-14.96,-15.86,-17.07,-18.45,-19.86,-21.13,-22.13,-22.76,-22.97,-22.77,-22.23,-21.47,-20.62,-19.85,-19.3,-19.09,-19.29,-19.9,-20.87,-22.1,-23.46,-24.79,-25.94,-26.77,-27.2,-27.21,-26.82,-26.11,-25.23,-24.31,-23.51,-22.98,-22.81,-23.05,-23.69,-24.66,-25.85,-27.11,-28.29,-29.23,-29.83,-30.01,-29.76,-29.14,-28.24,-27.2,-26.18,-25.32,-24.77,-24.6,-24.84,-25.46,-26.38,-27.48,-28.59,-29.57,-30.27,-30.59,-30.49,-29.97,-29.1,-27.99,-26.8,-25.67,-24.76,-24.18,-24,-24.23,-24.82,-25.67,-26.65,-27.6,-28.36,-28.81,-28.87,-28.49,-27.72,-26.63,-25.35,-24.04,-22.84,-21.91,-21.34,-21.18,-21.42,-22,-22.8,-23.68,-24.48,-25.06,-25.29,-25.11,-24.51,-23.54,-22.29,-20.9,-19.53,-18.33,-17.44,-16.93,-16.84,-17.14,-17.75,-18.55,-19.37,-20.06,-20.5,-20.56,-20.21,-19.45,-18.34,-17,-15.58,-14.24,-13.11,-12.32,-11.94,-11.98,-12.39,-13.08,-13.9,-14.71,-15.34,-15.67,-15.62,-15.15,-14.28,-13.11,-11.76,-10.37,-9.11,-8.12,-7.49,-7.29,-7.49,-8.05,-8.84,-9.72,-10.53,-11.13,-11.39,-11.25,-10.7,-9.78,-8.59,-7.26,-5.95,-4.83,-4,-3.57,-3.56,-3.95,-4.66,-5.56,-6.5,-7.32,-7.88,-8.08,-7.87,-7.25,-6.29,-5.11,-3.83,-2.63,-1.65,-1.01,-0.78,-0.97,-1.54,-2.39,-3.38,-4.36,-5.17,-5.68,-5.81,-5.52,-4.84,-3.85,-2.67</v>
+        <v>13.02,14.93,14.83,12.66,8.8,3.92,-1.08,-5.3,-7.96,-8.63,-7.25,-4.14,-0.01,4.28,7.81,9.82,9.85,7.84,4.12,-0.63,-5.54,-9.68,-12.28,-12.89,-11.41,-8.18,-3.85,0.69,4.54,6.91,7.34,5.71,2.35,-2.06,-6.68,-10.59,-12.97,-13.38,-11.75,-8.28,-3.69,1.05,5.24,7.99,8.76,7.34,4.3,-0.12,-4.38,-8.37,-10.59,-11.48,-9.83,-6.56,-1.82,2.82,7.2,9.05,9.78,8.15,5.43,-0.08,-3.74,-9.39,-10.8,-13.89,-12.49,-10.38,-5.18,-0.02,2.45,5.36,5.67,3.96,-3.46,-8.13,-10.33,-15.39,-24.08,-19.81,-24.12,-20.97,-16.91,-15.79,-6.85,-5.69,-3.66,-8.06,-14.35,-16.09,-23.76,-24.11,-28.69,-37.47,-31.14,-24.01,-22.27,-16,-11.03,-9.67,-5.16,-7.58,-11.94,-10.5,-18.63,-12.55,-21.67,-19.45,-17.11,-9.44,-0.04,4.11,4.89,11.98,17.1,20.34,21.88,16.42,25.63,16.23,25.32,24.17,21.49,27.48,37.64,51.02,51.46,61.38,59.9,75.37,69.62,76.24,72.08,61.42,81.66,73.22,84.05,76,97.33,98.78,106.88,123.01,112.8,118.31,115.86,139.55,116.37,110.19,125.4,125.52,114.78,137.48,134.44,134.92,151.09,154.12,176.62,177.8,160.45,171.71,154.77,168.63,161.76,153.18,138.46,164.52,170.28,164.49,164.77,191.07,193.5,160.18,161.45,171.84,147.31,137.4,143.87,135.24,138.29,156.51,159.06,146.92,149.44,152.04,164.12,149.01,135.62,145.25,125.98,115.64,126.07,117.03,118.3,100.62,94.09,112.42,103.23,109.96,104.05,114.99,96.1,99.45,80.35,76.17,76.23,70.99,62.84,51.73,68.82,65.37,60.28,70.93,69.29,65.75,58.19,49.4,37.14,38.28,30.13,27.67,23.08,26.74,22.82,26.07,29.49,32.06,35.09,34.75,32.45,25.03,21.06,12.25,6.33,4.93,2.18,3.2,8.59,9.9,17.05,19.25,18.94,17.93,15.46,12.2,7.53,2.61,-3.37,-6.21,-6.32,-4.27,-1.86,2.52,6.29,10.17,11.87,11.14,8.78,4.64,-0.5,-5.55,-10.49,-12.74,-13.17,-12.39,-9.02,-5.13,-0.46,2.18,3.59,3.88,0.93,-3.07,-8.19,-12.79,-17.95,-20.7,-20.28,-20.2,-16.92,-12.82,-9.43,-4.36,-3.32,-3.27,-4.92,-8.67,-14.55,-18.35,-23.45,-25.27,-27.68,-25.76,-23.51,-17.39,-12.94,-10.02,-9.35,-8.55,-10.07,-11.43,-16.63,-21.69,-26.45,-29.48,-27.33,-28.63,-22.73,-20.24,-14.07,-9.56,-8.32,-7.08,-9.25,-14.36,-19.03,-23.91,-27.84,-29.96,-28.98,-29.57,-21.43,-18.98,-17.38,-8.96,-9.62,-5.08,-6.46,-9.9,-17.57,-22.82,-28.03,-29.64,-31.73,-29.12,-21.49,-20.09,-16.33,-15.42,-9.23,-13.23,-10.42,-16.96,-19.31,-28.4,-30.54,-27.8,-33.57,-32.06,-29.19,-22.24,-21.12,-21.22,-11.64,-19.12,-15.1,-24.13,-28.99,-33.86,-31.26,-39.55,-44.62,-47.22,-35.64,-38.93,-35,-27.29,-31.76,-25.13,-25.73,-28.98,-29.61,-44,-42.1,-48.04,-44.19,-46.53,-47.66,-46.42,-36.19,-31.51,-31.16,-26.98,-34.06,-32.84,-32.36,-43.85,-42.51,-45.14,-59.29,-57.55,-54.54,-46.16,-44.15,-40,-33.93,-35.92,-37.01,-34.66,-31.56,-41.46,-46.16,-54.73,-55.83,-51.43,-44.18,-39.72,-34.6,-35.43,-22.4,-33.6,-19.68,-33.2,-35.21,-35.93,-36.93,-42.86,-37.68,-46.65,-37.61,-38.18,-37.38,-21.39,-26.99,-19.76,-15.22,-29.68,-27.96,-31.24,-40.97,-36.08,-39.26,-46.24,-36.49,-29.73,-27.15,-22.12,-18.86,-20.64,-20.32,-20.46,-23.53,-34.72,-32.8,-42.65,-43.14,-46.03,-42.53,-29.84,-32.69,-29.52,-23.32,-18.15,-19.15,-24.78,-28.2,-32.21,-37.97,-37.54,-39.88,-45.16,-42.88,-38.28,-30.48,-25.46,-18.86,-23.34,-21.44,-21.29,-29.82,-32.63,-37.84,-38.3,-39.06,-41.71,-39.05,-32.53,-26.12,-21.06,-19.92,-16.58,-19.15,-19.22,-23.02,-28.24,-32.65,-32.92,-34.27,-36.61,-31.52,-29.96,-22.56,-20.75,-14.74,-11.21,-13.99,-13.44,-16.1,-19.76,-27.93,-27.98</v>
       </c>
     </row>
     <row r="71">
@@ -1177,7 +1177,7 @@
         <v>[R_04_标记]</v>
       </c>
       <c r="C71" t="str">
-        <v>a: 23.2ms -36.9uv b: 48.2ms 159.9uv</v>
+        <v>a: 19.9ms -7.9uv b: 44.7ms 118.6uv</v>
       </c>
     </row>
     <row r="72">
@@ -1188,7 +1188,7 @@
         <v>[L_04_名字]</v>
       </c>
       <c r="C72" t="str">
-        <v>FERG(4)_lCone</v>
+        <v>FERG(4)_dRod</v>
       </c>
     </row>
     <row r="73">
@@ -1210,7 +1210,7 @@
         <v>[L_04_闪光]</v>
       </c>
       <c r="C74" t="str">
-        <v>白色光: 3.00 cd·s/m²</v>
+        <v>b白色光:0.30cd.m-2,5ms</v>
       </c>
     </row>
     <row r="75">
@@ -1221,7 +1221,7 @@
         <v>[L_04_闪光背景]</v>
       </c>
       <c r="C75" t="str">
-        <v>白色背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="76">
@@ -1232,7 +1232,7 @@
         <v>[L_04_采样]</v>
       </c>
       <c r="C76" t="str">
-        <v>刺激间隔: 15.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="77">
@@ -1243,7 +1243,7 @@
         <v>[L_04_分析时间]</v>
       </c>
       <c r="C77" t="str">
-        <v>200 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="78">
@@ -1265,7 +1265,7 @@
         <v>[L_04_详细数据(uv)]</v>
       </c>
       <c r="C79" t="str">
-        <v>2.04,2.99,2.35,0.46,-1.68,-2.92,-2.61,-0.91,1.27,2.78,2.81,1.34,-0.84,-2.57,-2.94,-1.74,0.39,2.31,3,2.09,0.07,-1.98,-2.98,-2.4,-0.53,1.61,2.9,2.65,0.98,-1.21,-2.75,-2.83,-1.41,0.76,2.53,2.94,1.79,-0.32,-2.27,-3.02,-2.17,-0.18,1.89,2.92,2.38,0.53,-1.65,-3.01,-2.84,-1.24,0.9,2.43,2.51,1.05,-1.2,-3.1,-3.69,-2.72,-0.79,1,1.58,0.54,-1.71,-4.11,-5.56,-5.47,-4.1,-2.42,-1.58,-2.31,-4.54,-7.43,-9.8,-10.8,-10.32,-9.08,-8.22,-8.71,-10.83,-14.01,-17.13,-19.12,-19.54,-18.77,-17.83,-17.84,-19.39,-22.25,-25.45,-27.83,-28.61,-27.84,-26.33,-25.23,-25.41,-26.99,-29.26,-31.09,-31.46,-30.06,-27.44,-24.68,-22.86,-22.45,-23.07,-23.72,-23.26,-21.07,-17.35,-13.04,-9.3,-6.93,-5.9,-5.43,-4.36,-1.8,2.4,7.56,12.54,16.32,18.57,19.78,21.03,23.42,27.43,32.7,38.24,42.9,46.02,47.76,49.04,51.02,54.48,59.45,65.12,70.33,74.18,76.45,77.81,79.36,82.14,86.49,91.92,97.35,101.69,104.4,105.79,106.85,108.71,112.06,116.72,121.82,126.18,128.97,130.14,130.46,131.08,132.91,136.17,140.24,143.98,146.35,146.97,146.28,145.34,145.26,146.58,149.01,151.57,153.11,152.93,151.13,148.6,146.48,145.64,146.13,147.22,147.75,146.79,144.08,140.23,136.36,133.53,132.16,131.81,131.46,129.99,126.83,122.26,117.24,112.95,110.11,108.64,107.72,106.17,103.16,98.6,93.2,88.14,84.39,82.23,81.1,79.89,77.56,73.67,68.64,63.5,59.38,56.9,55.82,55.19,53.88,51.12,46.98,42.3,38.23,35.66,34.71,34.69,34.45,33,30.06,26.15,22.38,19.81,18.92,19.32,19.99,19.79,18.1,15.12,11.77,9.21,8.22,8.76,10.01,10.83,10.29,8.26,5.39,2.83,1.57,1.95,3.43,4.93,5.37,4.24,1.9,-0.64,-2.25,-2.29,-0.92,0.94,2.12,1.84,0.07,-2.37,-4.35,-4.93,-3.94,-2.04,-0.35,0.1,-1.03,-3.26,-5.5,-6.68,-6.27,-4.58,-2.63,-1.55,-2.02,-3.88,-6.26,-7.98,-8.23,-6.98,-4.99,-3.44,-3.24,-4.61,-6.93,-9.07,-10,-9.33,-7.54,-5.69,-4.87,-5.65,-7.72,-10.1,-11.65,-11.66,-10.25,-8.3,-6.97,-7.1,-8.75,-11.17,-13.21,-13.91,-13.04,-11.2,-9.5,-8.99,-10.08,-12.33,-14.69,-16.04,-15.81,-14.26,-12.38,-11.29,-11.74,-13.63,-16.09,-17.98,-18.43,-17.35,-15.46,-13.93,-13.7,-15.06,-17.43,-19.68,-20.78,-20.28,-18.59,-16.76,-15.91,-16.63,-18.68,-21.11,-22.77,-22.91,-21.59,-19.65,-18.26,-18.28,-19.83,-22.22,-24.3,-25.08,-24.27,-22.41,-20.62,-19.96,-20.88,-23.01,-25.31,-26.67,-26.45,-24.87,-22.85,-21.57,-21.78,-23.46,-25.78,-27.59,-27.99,-26.84,-24.8,-23.03,-22.52,-23.59,-25.71,-27.81,-28.8,-28.18,-26.32,-24.23,-23.04,-23.41,-25.14,-27.33,-28.81,-28.79,-27.28,-25.07,-23.33,-22.95,-24.13,-26.2,-28.04,-28.62,-27.61,-25.48,-23.34,-22.27,-22.77,-24.53,-26.55,-27.67,-27.24,-25.41,-23.07,-21.38,-21.17,-22.45,-24.44,-26,-26.19,-24.81,-22.49,-20.35,-19.43,-20.1,-21.88,-23.72,-24.51,-23.7,-21.61,-19.21,-17.66,-17.64,-19.04,-20.97,-22.27,-22.11,-20.43,-17.99,-15.94,-15.24,-16.1,-17.93,-19.61,-20.09,-18.98,-16.71,-14.35,-13,-13.24,-14.78,-16.66,-17.73,-17.27,-15.38,-12.92,-11.04,-10.61,-11.71,-13.6,-15.14,-15.36,-14,-11.65,-9.41,-8.34,-8.87,-10.58,-12.42,-13.29,-12.58,-10.54,-8.13,-6.5,-6.39,-7.74,-9.7,-11.11,-11.09,-9.55,-7.18,-5.13,-4.37,-5.21,-7.08,-8.88,-9.55,-8.63,-6.5,-4.2,-2.86,-3.09,-4.68,-6.69,-7.95,-7.72,-6.02,-3.68,-1.86,-1.45,-2.59,-4.59,-6.32,-6.78,-5.66,-3.48,-1.33,-0.3,-0.87,-2.67,-4.68,-5.78,-5.32,-3.49,-1.21,0.36,0.43,-0.98</v>
+        <v>7.76,11.4,14.19,15.82,16.1,14.97,12.49,8.87,4.43,-0.45,-5.33,-9.79,-13.41,-15.91,-17.07,-16.84,-15.27,-12.56,-9.03,-5.05,-1.06,2.51,5.28,6.93,7.28,6.26,3.93,0.49,-3.74,-8.37,-12.97,-17.11,-20.4,-22.53,-23.32,-22.65,-20.66,-17.45,-13.43,-8.93,-4.46,-0.32,3.03,5.25,6.13,5.78,3.84,1,-2.79,-6.92,-10.91,-14.83,-17.43,-19.4,-20.08,-18.77,-16.42,-12.86,-8.9,-4.4,0.62,4.9,7.67,10.18,10.64,10.58,8.82,5.73,1.41,-3,-7.88,-13.64,-14.45,-18.44,-20.19,-20.02,-16.72,-14.43,-10.19,-6.34,-4.12,-1.11,0,1.28,6.21,3.7,1.17,-4.89,-5.23,-13.02,-19.17,-19.98,-24.31,-33.76,-31.71,-28.66,-26.68,-32.71,-26.94,-16.04,-17.98,-15.52,-3.77,-2.66,1.12,-8.56,-8.63,-5.81,-11.56,-7.01,-20.64,-17.07,-16.9,-24.3,-16.8,-20.21,-15.41,-11.2,-3.52,9.05,8.57,21.13,18.38,33.75,33.47,32.71,41.85,39.56,35.75,32.06,31.31,28.79,41.5,31.72,30.94,48.11,62.43,47.72,63.84,76.68,81.73,100.92,89.73,108.07,99.19,111.24,123.76,106.54,112.45,122.95,123.7,122.65,108.7,122.19,121.47,117.89,122.38,143.91,125.01,140.17,157.61,166.88,149.07,173.97,163.13,180.46,159.05,174.91,162.03,147.75,149.3,142.71,152.72,134.82,151.92,134.39,171.03,170.71,176.61,168.35,152.06,153.11,172.92,170.51,174.66,163.49,160.08,152.03,176.39,155,156.01,151.9,127.91,112.74,121.87,107.58,123.54,117.73,114.86,115.43,121.84,142.33,131.02,116.06,128.73,121.75,132.2,112.76,101.82,93.77,99.58,75.26,86.01,85.87,60.26,66.3,59.04,70.17,75.25,65.89,82.89,70.49,79.73,81.09,73.1,76.47,67.32,57.04,51.14,55.46,45.74,40.32,33.55,30.39,27.62,23.48,29.45,27.31,31.38,31.44,31.24,37.66,38.2,43.54,37.06,37.26,34.68,28.51,25.44,18.86,16.67,9.56,4.86,1.01,-0.8,-0.36,-0.49,3.6,4.98,9.97,13.88,14.08,18.1,20.35,18.8,18.88,16.32,11.93,6.17,1.44,-3.43,-8.13,-13.22,-16.74,-18.97,-18.57,-17.07,-15.32,-12.14,-9,-5.18,-1.61,1.03,2.18,2.88,1.19,-0.55,-4.74,-9.19,-14.21,-19.5,-24.47,-28.38,-31.28,-32.27,-32.44,-29.59,-28.63,-23.92,-20.89,-17.28,-13.21,-7.61,-7.84,-6.51,-7.43,-8.85,-12.1,-16.59,-20.55,-25.45,-28.5,-30.56,-32.82,-34.64,-34.88,-31.92,-27.25,-23.92,-18.9,-15.53,-11.66,-7.88,-6.81,-1.33,-6.47,-7.16,-5.67,-10.5,-14.01,-22.84,-27.72,-29.24,-31.33,-33.34,-28.67,-28.8,-28.24,-20.4,-17.15,-10.3,-11.06,-5.81,-3.61,-3.11,-6.02,-8.46,-12.43,-11.12,-15.6,-27.6,-32.72,-32.94,-36.09,-33.27,-40.44,-32.42,-31.62,-32.4,-29.89,-25.69,-22.87,-21.74,-15.02,-19.59,-11.06,-16.55,-22.84,-25.84,-35.07,-33.15,-38.04,-48.25,-51.19,-53.18,-56.46,-51.65,-47.45,-51.69,-46.47,-35.52,-34.34,-27.15,-31,-29.48,-24.09,-36.17,-27.27,-39.22,-36.35,-44.58,-54.77,-60.07,-51.06,-57.88,-63.53,-51.48,-51.25,-45.9,-38.12,-39.01,-37.68,-25.52,-27.15,-34.75,-23.85,-27.37,-30.76,-26.77,-39.75,-47.66,-52.07,-48.92,-43.74,-47.16,-43.46,-46.65,-48.99,-44.3,-39.91,-33.31,-21.66,-26.78,-13.04,-15.81,-22.95,-16.51,-28.46,-22.16,-33.86,-37.11,-42.83,-40.49,-41.07,-38.14,-44.41,-47.82,-45.58,-33.39,-35.93,-27.29,-20.54,-15.2,-22.16,-19.73,-10.14,-21.17,-15.15,-23.2,-28.49,-31.96,-39.4,-37.53,-44.68,-42.28,-43.29,-43.5,-37.59,-43.32,-32.27,-26.42,-28.31,-18.98,-15.22,-14.23,-20.76,-19.41,-25.07,-23.99,-28.04,-37.22,-44.19,-42.22,-44.98,-50.2,-49.11,-44.69,-41.69,-35.44,-32.84,-27.75,-25.95,-17.17,-15.31,-12.75,-16.64,-13.7,-18.39,-22.6,-25.29,-27.45,-34.2,-38.44,-38.43,-38.57,-36.15,-34.92,-30.55,-28.42,-21.91</v>
       </c>
     </row>
     <row r="80">
@@ -1276,7 +1276,7 @@
         <v>[L_04_标记]</v>
       </c>
       <c r="C80" t="str">
-        <v>a: 23.2ms -34.7uv b: 48.2ms 150.3uv</v>
+        <v>a: 19.8ms -12.6uv b: 44.8ms 113.0uv</v>
       </c>
     </row>
     <row r="81">
@@ -1287,7 +1287,7 @@
         <v>[R_05_名字]</v>
       </c>
       <c r="C81" t="str">
-        <v>FERG(5)_Flicker</v>
+        <v>FERG(5)_dRod</v>
       </c>
     </row>
     <row r="82">
@@ -1298,7 +1298,7 @@
         <v>[R_05_放大器]</v>
       </c>
       <c r="C82" t="str">
-        <v>1-300 Hz</v>
+        <v>1-75 Hz</v>
       </c>
     </row>
     <row r="83">
@@ -1309,7 +1309,7 @@
         <v>[R_05_闪光]</v>
       </c>
       <c r="C83" t="str">
-        <v>白色光: 3.00 cd·s/m²</v>
+        <v>b白色光:1.0cd.m-2,5ms</v>
       </c>
     </row>
     <row r="84">
@@ -1320,7 +1320,7 @@
         <v>[R_05_闪光背景]</v>
       </c>
       <c r="C84" t="str">
-        <v>白色背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="85">
@@ -1331,7 +1331,7 @@
         <v>[R_05_采样]</v>
       </c>
       <c r="C85" t="str">
-        <v>刺激间隔: 50.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="86">
@@ -1342,7 +1342,7 @@
         <v>[R_05_分析时间]</v>
       </c>
       <c r="C86" t="str">
-        <v>500 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="87">
@@ -1364,7 +1364,7 @@
         <v>[R_05_详细数据(uv)]</v>
       </c>
       <c r="C88" t="str">
-        <v>-0.12,0.1,-1.28,-3.92,-6.82,-8.84,-9.34,-8.48,-7.17,-6.57,-7.5,-9.97,-13.19,-16.02,-17.52,-17.51,-16.62,-15.97,-16.59,-18.84,-22.22,-25.66,-28.07,-28.88,-28.41,-27.65,-27.72,-29.29,-32.23,-35.64,-38.33,-39.48,-39.03,-37.73,-36.72,-36.95,-38.61,-41.08,-43.24,-44.03,-43.07,-40.8,-38.28,-36.6,-36.33,-37.18,-38.18,-38.17,-36.45,-33.14,-29.11,-25.52,-23.24,-22.33,-22.08,-21.34,-19.18,-15.34,-10.43,-5.59,-1.88,0.27,1.26,2.14,4,7.4,12.08,17.06,21.17,23.66,24.61,24.84,25.51,27.47,30.81,34.81,38.31,40.33,40.59,39.65,38.61,38.54,39.87,42.22,44.54,45.73,45.16,43.09,40.46,38.43,37.77,38.44,39.62,40.16,39.19,36.59,33.06,29.75,27.68,27.15,27.64,28.06,27.35,25.05,21.54,17.86,15.13,13.99,14.27,15.03,15.11,13.76,10.98,7.59,4.74,3.35,3.56,4.71,5.65,5.39,3.57,0.7,-2.12,-3.84,-3.94,-2.78,-1.39,-0.89,-1.97,-4.44,-7.41,-9.72,-10.58,-9.99,-8.73,-7.97,-8.63,-10.9,-14.13,-17.2,-19.07,-19.4,-18.66,-17.93,-18.28,-20.25,-23.51,-27.06,-29.74,-30.87,-30.57,-29.73,-29.51,-30.7,-33.33,-36.64,-39.44,-40.8,-40.48,-39.1,-37.77,-37.51,-38.7,-40.88,-42.96,-43.85,-42.99,-40.66,-37.83,-35.66,-34.84,-35.27,-36.08,-36.1,-34.5,-31.22,-27.01,-23.03,-20.25,-18.92,-18.46,-17.75,-15.79,-12.14,-7.28,-2.26,1.78,4.26,5.41,6.2,7.74,10.76,15.16,20.06,24.29,26.98,28.02,28.11,28.4,29.85,32.72,36.43,39.87,41.98,42.31,41.26,39.88,39.28,40.07,42.02,44.19,45.42,44.98,42.92,40.08,37.65,36.5,36.77,37.78,38.39,37.63,35.21,31.68,28.16,25.73,24.86,25.2,25.72,25.3,23.33,20.03,16.32,13.37,11.97,12.08,12.91,13.29,12.32,9.87,6.59,3.63,1.98,1.98,3.1,4.24,4.32,2.85,0.16,-2.73,-4.71,-5.12,-4.14,-2.7,-1.97,-2.73,-5.01,-8.01,-10.59,-11.82,-11.53,-10.38,-9.5,-9.9,-11.94,-15.13,-18.39,-20.62,-21.31,-20.76,-19.97,-20.08,-21.75,-24.83,-28.42,-31.34,-32.77,-32.66,-31.78,-31.28,-32.07,-34.35,-37.49,-40.35,-41.89,-41.72,-40.28,-38.65,-37.91,-38.6,-40.43,-42.39,-43.34,-42.58,-40.22,-37.14,-34.5,-33.13,-33.11,-33.68,-33.7,-32.22,-29.02,-24.7,-20.38,-17.13,-15.37,-14.66,-13.98,-12.21,-8.81,-4.06,1.07,5.4,8.19,9.52,10.23,11.47,14.08,18.13,22.89,27.18,30.04,31.18,31.17,31.11,32.05,34.41,37.78,41.11,43.28,43.69,42.57,40.89,39.8,40.04,41.56,43.54,44.8,44.48,42.48,39.51,36.72,35.1,34.97,35.77,36.43,35.89,33.69,30.23,26.56,23.81,22.61,22.76,23.35,23.21,21.59,18.54,14.86,11.74,10.07,10,10.85,11.49,10.92,8.81,5.69,2.65,0.76,0.52,1.55,2.84,3.25,2.12,-0.36,-3.28,-5.5,-6.24,-5.49,-4.06,-3.13,-3.6,-5.66,-8.65,-11.45,-13.06,-13.11,-12.11,-11.15,-11.31,-13.1,-16.21,-19.61,-22.17,-23.21,-22.89,-22.09,-21.96,-23.32,-26.17,-29.73,-32.84,-34.55,-34.66,-33.77,-33.01,-33.39,-35.28,-38.19,-41.04,-42.73,-42.7,-41.25,-39.35,-38.14,-38.31,-39.73,-41.51,-42.49,-41.83,-39.48,-36.19,-33.12,-31.21,-30.71,-31.01,-31,-29.64,-26.55,-22.18,-17.59,-13.91,-11.71,-10.75,-10.05,-8.49,-5.36,-0.78,4.38,8.93,12.02,13.54,14.21,15.15,17.33,20.99,25.53,29.83,32.83,34.08,34,33.61,34.04,35.87,38.84,42.01,44.22,44.72,43.58,41.66,40.1,39.8,40.87,42.6,43.87,43.7,41.8,38.75,35.66,33.61,33.06,33.63,34.31,33.99,32.05,28.72,24.96,21.93,20.4,20.35,20.97,21.09,19.84,17.08,13.5,10.25,8.32,8.04,8.87,9.73,9.53,7.79,4.88,1.8,-0.32,-0.83,0.07,1.45,2.15,1.37,-0.87</v>
+        <v>-4.59,0.82,0.63,-5.22,-13.18,-18.39,-17.69,-11.65,-4.2,-0.16,-2.16,-9.03,-16.5,-19.9,-17.14,-9.98,-2.96,-0.52,-4.17,-11.6,-18.06,-19.44,-14.78,-6.96,-0.81,-0.13,-5.21,-12.74,-17.81,-17.09,-10.88,-2.93,1.9,0.74,-5.5,-12.7,-16.12,-13.42,-6.1,1.4,4.53,1.52,-5.56,-12.04,-13.67,-9.23,-1.36,5.12,6.29,1.54,-6,-11.43,-11.23,-5.41,2.43,7.43,6.48,0.23,-7.33,-11.43,-9.45,-2.7,4.57,7.72,4.66,-2.68,-9.89,-12.35,-8.75,-1.56,4.66,5.58,0.8,-7.25,-13.72,-14.34,-9.84,-2.19,2.36,0.79,-5.19,-13.69,-19.39,-17.7,-11.71,-5.78,-2.34,-6.85,-14.01,-21.55,-26.7,-22.21,-18.31,-11.77,-10.15,-16.47,-24.8,-30.9,-35.97,-32.18,-25.04,-17.32,-20.45,-27.29,-36.64,-44.17,-37.03,-36.21,-26.31,-29.06,-22.91,-32.6,-39.91,-46.91,-43.79,-36.79,-30.87,-28.67,-28.33,-33.08,-43.67,-45.09,-34.35,-27.35,-15.51,-17.55,-15.56,-20.73,-30.08,-27.48,-12.97,-9.74,7.12,1.76,0.32,-0.66,-4.51,1.1,9.93,23.08,26.89,27.88,20.22,23.51,23,29.91,36.95,48.5,60.94,59.38,49.08,44.58,53.9,66.45,76.29,74.22,87.06,76.1,76.22,85.59,77.56,86.06,98.12,121.41,120.95,112.36,111.45,98.67,114.74,129.42,131.93,136.17,145.22,125.57,137.33,134.72,144.95,125.07,164.08,154.63,152.61,119.82,139.38,150.76,136.15,135.9,157.9,163.77,145.68,146.12,148.7,125.31,152.32,159.23,158.23,152.01,138.81,138.35,132.57,134.76,132.73,138.55,133.48,129.64,129.07,105.79,104.05,108.69,112.77,109.5,115.88,112.69,91.01,80,96.86,100.44,91.07,101.01,94.22,76.21,63.84,58.58,72.64,69.05,77.11,67.54,70.07,58.51,42.42,46,45.45,53.62,57.49,50.02,40.65,30.41,23.8,26.35,28.25,36.17,38.56,28.74,22.22,11.26,12.38,14.39,19.35,25.05,22.35,15.84,7.67,0.73,-0.86,4.4,10.51,12.38,9.93,2.8,-6.35,-9.74,-9.34,-2.25,3.82,5.33,1.83,-6.75,-14.23,-16.42,-13.16,-5.93,-0.39,0.39,-5.44,-13.63,-19.27,-19.63,-14.51,-6.88,-2.43,-3.22,-10.04,-17.72,-22.14,-20.25,-13.29,-5.62,-2.71,-5.86,-13.23,-19.94,-22.4,-18.52,-10.81,-4.72,-2.36,-7.16,-14.52,-20.92,-20.91,-14.57,-7.82,-1.4,-2.14,-7.87,-16.37,-20.71,-18.27,-10.95,-4.59,1.27,-2.77,-8.08,-16.32,-18.51,-15.6,-9.31,-2.05,1.76,-5.13,-11.11,-17.89,-18.01,-12.11,-4.95,-0.39,-0.95,-5.23,-14.57,-20.78,-18.2,-11.89,-6.66,-2.23,-3.03,-11.61,-19.93,-24.31,-22.84,-14.99,-6.02,-8.4,-10.24,-15.28,-22.19,-29.96,-19.74,-13.77,-9.31,-7.52,-19.18,-28.31,-31.01,-30.78,-26.91,-15.73,-12.12,-17.97,-25.36,-33.85,-35.98,-33.33,-25.07,-16.24,-18.86,-18.68,-27.89,-38.52,-38.74,-34.93,-27.85,-20.78,-20.87,-27.16,-36.38,-35.31,-37.65,-36.08,-30.11,-16.3,-17.62,-34.29,-34.81,-35.91,-37.24,-30.21,-22.98,-15.39,-24.23,-33.07,-37.75,-35.88,-38.81,-25.13,-22.07,-14.71,-21.75,-30.09,-39.16,-40.7,-32.59,-27.88,-23.36,-27.57,-20.68,-28.5,-43.67,-43.01,-27.71,-22.99,-26.35,-26.48,-27.05,-29.75,-35.15,-36.12,-33.06,-19.58,-13.97,-22.24,-26.67,-34.79,-35.14,-30.02,-29.75,-26.42,-24.12,-35.18,-38.26,-46.8,-46.08,-35.61,-30.27,-20.33,-25.94,-38.92,-35.13,-40.58,-45.65,-34.28,-31.52,-23.75,-33.2,-41.36,-37.88,-37.17,-35.76,-34.19,-24.89,-20.74,-26.72,-32.33,-44.8,-38.7,-39.96,-27.26,-29.3,-28.7,-32.3,-40.27,-39.86,-42.72,-31.97,-29.66,-18.1,-22.05,-29.8,-41.45,-40.98,-33.69,-24.57,-17.28,-19.33,-25.83,-27.67,-34.8,-31.21,-24.94,-22.72,-10.13,-13.45,-23.99,-31.18,-27.81,-30.34,-18.31,-12.21,-7.67,-11.42,-19.46,-23.88,-24.72,-20.81,-15.99,-10.18,-5.84,-12.43,-17.29,-22.07,-22.44,-15.21</v>
       </c>
     </row>
     <row r="89">
@@ -1375,7 +1375,7 @@
         <v>[R_05_标记]</v>
       </c>
       <c r="C89" t="str">
-        <v>幅值: 35.7uv 相位: 48.5°</v>
+        <v>a: 22.8ms -20.9uv b: 47.8ms 161.4uv</v>
       </c>
     </row>
     <row r="90">
@@ -1386,7 +1386,7 @@
         <v>[L_05_名字]</v>
       </c>
       <c r="C90" t="str">
-        <v>FERG(5)_Flicker</v>
+        <v>FERG(5)_dRod</v>
       </c>
     </row>
     <row r="91">
@@ -1397,7 +1397,7 @@
         <v>[L_05_放大器]</v>
       </c>
       <c r="C91" t="str">
-        <v>1-300 Hz</v>
+        <v>1-75 Hz</v>
       </c>
     </row>
     <row r="92">
@@ -1408,7 +1408,7 @@
         <v>[L_05_闪光]</v>
       </c>
       <c r="C92" t="str">
-        <v>白色光: 3.00 cd·s/m²</v>
+        <v>b白色光:1.0cd.m-2,5ms</v>
       </c>
     </row>
     <row r="93">
@@ -1419,7 +1419,7 @@
         <v>[L_05_闪光背景]</v>
       </c>
       <c r="C93" t="str">
-        <v>白色背景光</v>
+        <v>b背景光_关:0.0cd.m-2</v>
       </c>
     </row>
     <row r="94">
@@ -1430,7 +1430,7 @@
         <v>[L_05_采样]</v>
       </c>
       <c r="C94" t="str">
-        <v>刺激间隔: 50.0S</v>
+        <v>刺激间隔:10.0S</v>
       </c>
     </row>
     <row r="95">
@@ -1441,7 +1441,7 @@
         <v>[L_05_分析时间]</v>
       </c>
       <c r="C95" t="str">
-        <v>500 ms</v>
+        <v>200ms</v>
       </c>
     </row>
     <row r="96">
@@ -1463,7 +1463,7 @@
         <v>[L_05_详细数据(uv)]</v>
       </c>
       <c r="C97" t="str">
-        <v>-6.17,-7.13,-10.73,-13.62,-13.25,-10.7,-9.53,-11.74,-15.56,-17.42,-15.98,-13.64,-13.83,-17.18,-20.81,-21.55,-19.53,-17.99,-19.68,-23.73,-26.67,-26.27,-24.07,-23.65,-26.57,-30.64,-32.35,-30.82,-28.76,-29.42,-32.95,-36.19,-36.24,-33.67,-31.91,-33.34,-36.66,-38.3,-36.43,-33.03,-31.63,-33.36,-35.66,-35.17,-31.49,-27.62,-26.6,-28.11,-28.8,-26.09,-21.05,-17.21,-16.62,-17.53,-16.38,-11.81,-6.2,-3,-2.88,-2.99,-0.17,5.47,10.68,12.68,12.28,12.95,16.9,22.6,26.46,26.86,25.96,27.23,31.59,36.32,38.12,36.83,35.54,37.19,41.2,44.14,43.6,40.84,39.44,41.23,44.26,44.99,42.28,38.65,37.49,39.23,40.9,39.45,35.19,31.46,30.9,32.47,32.66,29.43,24.52,21.5,21.79,23.07,21.88,17.56,12.96,11.27,12.44,13.26,10.95,6.31,2.81,2.72,4.54,4.71,1.58,-2.69,-4.61,-3.25,-1.27,-1.98,-5.59,-9,-9.27,-6.95,-5.44,-7.2,-10.99,-13.26,-12.15,-9.6,-9.14,-11.98,-15.63,-16.69,-14.71,-12.67,-13.64,-17.35,-20.49,-20.41,-18.13,-17.16,-19.59,-23.7,-25.93,-24.84,-22.74,-23.08,-26.58,-30.4,-31.33,-29.39,-27.78,-29.29,-33.16,-35.91,-35.24,-32.61,-31.59,-33.82,-37.19,-38.18,-35.8,-32.71,-32.21,-34.54,-36.59,-35.41,-31.5,-28.25,-28.14,-29.95,-30.13,-26.79,-21.83,-18.81,-18.96,-19.8,-17.95,-12.91,-7.67,-5.33,-5.64,-5.33,-1.73,4.14,8.77,10.03,9.58,10.97,15.65,21.31,24.48,24.39,23.82,26,30.9,35.33,36.45,34.98,34.37,36.92,41.19,43.62,42.5,39.92,39.4,41.93,44.9,44.97,41.89,38.73,38.49,40.7,41.97,39.81,35.44,32.42,32.66,34.31,33.84,30,25.26,23.05,23.89,24.86,22.87,18.14,13.97,13.06,14.45,14.66,11.55,6.78,3.92,4.47,6.15,5.51,1.75,-2.32,-3.5,-1.73,-0.2,-1.76,-5.72,-8.62,-8.15,-5.71,-4.88,-7.38,-11.16,-12.7,-10.98,-8.61,-8.95,-12.28,-15.56,-15.8,-13.45,-11.88,-13.62,-17.51,-20,-19.16,-16.82,-16.55,-19.61,-23.56,-25,-23.36,-21.55,-22.7,-26.61,-29.99,-30.14,-27.96,-26.96,-29.27,-33.27,-35.38,-34.09,-31.6,-31.41,-34.3,-37.52,-37.79,-35.05,-32.47,-32.88,-35.63,-37.26,-35.41,-31.47,-28.99,-29.71,-31.62,-31.17,-27.32,-22.65,-20.53,-21.27,-21.86,-19.28,-13.96,-9.28,-7.78,-8.35,-7.46,-3.15,2.75,6.66,7.26,6.96,9.15,14.42,19.84,22.26,21.83,21.79,24.85,30.12,34.08,34.55,33.09,33.29,36.66,41,42.8,41.23,39.02,39.43,42.57,45.28,44.67,41.4,38.9,39.56,42.03,42.76,39.99,35.72,33.51,34.46,36,34.79,30.49,26.13,24.75,25.98,26.49,23.71,18.76,15.19,15,16.42,15.89,12.08,7.39,5.26,6.31,7.66,6.16,1.94,-1.76,-2.18,-0.19,0.72,-1.65,-5.76,-8.03,-6.89,-4.55,-4.5,-7.62,-11.18,-11.94,-9.76,-7.79,-8.93,-12.58,-15.33,-14.77,-12.24,-11.29,-13.74,-17.6,-19.34,-17.84,-15.65,-16.14,-19.69,-23.3,-23.91,-21.88,-20.54,-22.47,-26.6,-29.39,-28.8,-26.58,-26.3,-29.31,-33.24,-34.63,-32.82,-30.68,-31.36,-34.75,-37.61,-37.18,-34.25,-32.33,-33.61,-36.58,-37.65,-35.22,-31.44,-29.83,-31.27,-33.07,-31.94,-27.73,-23.55,-22.34,-23.52,-23.68,-20.4,-14.99,-11.02,-10.32,-10.94,-9.37,-4.46,1.25,4.36,4.44,4.47,7.5,13.18,18.17,19.85,19.24,19.88,23.77,29.19,32.55,32.45,31.23,32.31,36.37,40.56,41.7,39.83,38.18,39.54,43.09,45.38,44.14,40.88,39.17,40.66,43.19,43.29,40.01,36.06,34.73,36.24,37.48,35.53,30.94,27.14,26.58,28.02,27.91,24.41,19.46,16.6,17.04,18.28,16.95,12.58,8.18,6.81,8.21,9.05,6.7,2.19,-0.96,-0.68,1.32,1.49,-1.61,-5.66,-7.21,-5.54,-3.5,-4.28,-7.86,-11.04,-11.01</v>
+        <v>-35.24,-32.97,-27.18,-20.61,-16.33,-16.39,-20.88,-27.89,-34.37,-37.51,-35.98,-30.57,-23.77,-18.73,-17.76,-21.36,-27.95,-34.59,-38.33,-37.49,-32.46,-25.48,-19.69,-17.65,-20.24,-26.25,-32.92,-37.17,-37.02,-32.44,-25.39,-18.95,-15.89,-17.46,-22.84,-29.46,-34.21,-34.8,-30.82,-23.9,-16.99,-13.05,-13.67,-18.43,-25,-30.28,-31.72,-28.52,-21.95,-14.82,-10.18,-9.97,-14.15,-20.7,-26.54,-28.94,-26.69,-20.72,-13.6,-8.46,-7.52,-11.17,-17.71,-24.15,-27.55,-26.38,-21.16,-14.24,-8.83,-7.31,-10.33,-16.81,-23.78,-28.4,-28.25,-24.15,-17.5,-11.79,-9.81,-12.36,-18.69,-26.03,-31.66,-32.87,-29.34,-24.39,-18.8,-15.97,-18.19,-23.91,-32.97,-38.3,-41.19,-39.89,-32.38,-26.25,-26.07,-27.29,-32.27,-38.43,-49.12,-50.26,-51.63,-46.63,-35.47,-32.86,-35.61,-38.69,-50.93,-55.09,-61.16,-53.87,-52,-41.79,-42.69,-39.32,-45.05,-47.63,-52.25,-61.05,-55.59,-51.77,-43.06,-30.68,-29.65,-33.31,-39.62,-43.76,-45.2,-44.53,-38.78,-26.71,-15.2,-10.06,-7.78,-15.54,-15.07,-16.35,-11.84,-10.93,-3.78,10.37,23.98,20.15,18.32,21.17,15.33,20.32,23.44,35.74,48.72,43.92,54.97,63.66,47.6,51.33,57.16,62.18,67.89,82.99,76.01,78.94,82.03,90.5,80.27,71.06,80.65,103.44,95.41,117.42,107.43,125.45,107.53,98.27,100.63,104.85,122.58,119.3,144.98,140.37,148.44,119.38,116.63,124.29,136.7,128.47,119.61,129.22,134.23,147.81,156.79,146.47,128.42,134.83,119.47,138.62,137.5,134.41,159.08,152.93,138.68,104.83,103.7,131.4,135.65,133.92,126.13,140.26,121.26,117.11,103.25,107.05,98.97,82.77,102.53,94.44,88.57,100.84,75.9,68.2,67.35,61.54,76.91,76.41,76.62,82.37,77.91,64.9,58.47,40.02,33.74,46.24,51.34,46.11,46.35,50.34,35.44,29.52,25.37,19.02,16.24,22.56,30.2,26.93,27.52,19.82,10.72,6.6,-1,3.44,4.96,13.1,14.07,12.07,7.82,-0.14,-7.14,-10.43,-11.74,-7.77,-0.5,4.1,3.06,-0.34,-7.65,-16.16,-20.12,-20.4,-16.58,-9.62,-5.11,-3.07,-6.51,-13,-19.82,-25.16,-26.27,-22.29,-15.7,-9.73,-7.29,-9.11,-14.72,-22.53,-27.6,-28.51,-25.72,-18.9,-12.58,-9.21,-10.08,-14.44,-20.98,-27.18,-28.49,-25.61,-19.68,-12.68,-8.29,-8.76,-11.44,-18.06,-24.8,-27.22,-24.82,-18.82,-12.62,-5.95,-5.76,-9.35,-15.13,-20.99,-24.5,-25.13,-18.41,-12.95,-5.91,-3.64,-5.46,-12.37,-19.39,-22.95,-22.39,-18.55,-10.43,-5.58,-3.6,-6.57,-10.42,-18,-24.42,-25.87,-22.83,-14.31,-8.29,-4.95,-7.75,-9.81,-20.68,-24.9,-28.36,-27.41,-19.17,-15.22,-10.54,-10.1,-11.59,-22.71,-27.8,-30.36,-29.23,-24.11,-20.11,-16.04,-17.57,-19.79,-23.31,-31.42,-32.82,-36.95,-29.45,-23.08,-18.69,-15.53,-24.19,-32.49,-38.97,-43.14,-41.33,-33.01,-30.24,-21.26,-21.73,-25.39,-29.68,-38.47,-39.16,-39.48,-42.11,-32.25,-30.97,-22.97,-22.15,-28.17,-34.46,-47.62,-47.36,-39.17,-39.37,-30.89,-20.45,-30.29,-29.33,-37.55,-47.35,-43.1,-34.98,-32.16,-26.14,-16.18,-18.22,-30.5,-32.38,-40.53,-47.96,-43.38,-29.83,-33.23,-16.25,-14.8,-20.85,-24.87,-30.91,-39.53,-34.28,-32.19,-33.08,-21.45,-19.88,-28.52,-29.58,-34.78,-40.14,-40.19,-36.9,-35.7,-24.24,-24.96,-24.63,-24.06,-28.59,-36.16,-38.68,-43.26,-26.77,-18.36,-24.29,-18.48,-28.56,-37.14,-45.64,-44.81,-40.52,-34.91,-30,-23.81,-27.37,-25.65,-27.14,-39.1,-47.07,-44.83,-40.33,-34.15,-16.52,-22.17,-31.1,-37.1,-41.61,-35.79,-36.22,-34.88,-26.24,-23.88,-22.48,-25.23,-24.3,-31.19,-35.54,-41.6,-27.98,-29.04,-18.62,-15.24,-15.35,-20.01,-25.98,-29.7,-31.78,-28.67,-18.75,-17.47,-10.4,-10.96,-16.49,-21.23,-30.08,-25.68,-21.51,-19.89,-11.72,-5.7,-7.5,-8.85,-14.96,-23.46,-19.88,-20.1,-15.79,-3.38</v>
       </c>
     </row>
     <row r="98">
@@ -1474,12 +1474,3774 @@
         <v>[L_05_标记]</v>
       </c>
       <c r="C98" t="str">
-        <v>幅值: 33.5uv 相位: 48.5°</v>
+        <v>a: 22.8ms -20.1uv b: 47.9ms 142.8uv</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B99" t="str">
+        <v>[R_06_名字]</v>
+      </c>
+      <c r="C99" t="str">
+        <v>FERG(6)_dRod</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B100" t="str">
+        <v>[R_06_放大器]</v>
+      </c>
+      <c r="C100" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B101" t="str">
+        <v>[R_06_闪光]</v>
+      </c>
+      <c r="C101" t="str">
+        <v>b白色光:3.0cd.m-2,4ms</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B102" t="str">
+        <v>[R_06_闪光背景]</v>
+      </c>
+      <c r="C102" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B103" t="str">
+        <v>[R_06_采样]</v>
+      </c>
+      <c r="C103" t="str">
+        <v>刺激间隔:2.0S</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B104" t="str">
+        <v>[R_06_分析时间]</v>
+      </c>
+      <c r="C104" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B105" t="str">
+        <v>[R_06_数据长度]</v>
+      </c>
+      <c r="C105" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B106" t="str">
+        <v>[R_06_详细数据(uv)]</v>
+      </c>
+      <c r="C106" t="str">
+        <v>-2.34,4.63,13.19,12.63,3.65,-2.46,2,11.53,14.32,7,-1.12,0.3,9.66,15.47,10.68,1.53,-0.28,7.79,15.92,14.23,5.13,0.33,6.13,15.61,17.22,9.26,2.02,4.87,14.55,19.26,13.4,4.59,4.13,12.87,20.11,17.03,7.69,3.98,10.71,19.59,19.68,10.9,4.37,8.33,17.8,20.94,13.83,5.24,5.82,14.77,20.65,16.11,6.37,3.51,10.92,18.55,16.99,7.64,1.42,6.04,15.17,16.95,8.07,-0.29,1.32,10.21,14.41,8.95,-1.22,-3.7,4.77,11.29,7.3,-3.67,-6.55,-2.8,6.17,4.47,-4.98,-11.92,-7.79,-0.59,2.8,-6.42,-14.76,-13.27,-8.3,-2.89,-6.39,-16.01,-22.64,-9.93,-8.06,-1.95,-14.43,-19.99,-13.72,-5.42,-1.73,-12.91,-17.02,-13.07,-10.63,-4.06,-7.93,-14.13,-16.73,-9.12,0.39,0.34,-9.77,-10.05,0.83,7.88,10.68,4.19,2.05,6.88,24.94,24.31,17.9,11.77,16.16,26.14,38.74,39.54,35.56,33.74,49.12,56.03,50.04,46.22,52.28,62.97,74.64,80.6,72.69,66.16,69.66,84.15,85.73,92.52,84.78,91.22,96.81,109.46,114.63,112.5,97.54,99.66,139.4,142.3,130.07,106.59,137.45,132.85,139.16,134.33,138.88,120.91,134.52,168.66,147.97,154.05,164.54,162.63,171.75,164.39,166.35,140.31,162.16,158.08,191.94,174.43,146.46,158.52,177.17,160.45,159.18,176.03,156.3,150.12,196.9,172,176,155.21,167.05,187.71,188.64,152.5,171.87,146.63,169.27,159.42,175.82,158.82,155.34,141.8,145.87,139.23,144.63,122.97,142.04,156.38,136.34,123.16,121.58,134.43,140.19,129.69,130.9,107.39,109.96,125.54,117.93,104.83,99.1,85.08,97.26,94.42,104.05,89.35,74.77,88.89,88.65,86.04,83.8,61.55,71.22,69.04,69.29,65.38,60.41,49.28,59.48,59.1,52.53,44.01,41.68,42.69,45.11,47.88,39.58,28.01,26.39,37.64,37.46,29.42,18.98,19.65,27.69,30.96,24.94,15.74,12.08,14.71,23.38,21.99,12.31,4.95,7.71,16.37,19.15,10.46,2.71,2.42,10.39,15.82,11.42,1.69,-1.6,5.76,12.82,11.77,1.85,-3.98,1.19,9.53,11.97,3.9,-3.51,-2.13,7.7,12.28,6.73,-3.03,-4.02,4.54,12.69,9.75,-0.58,-4.39,1.76,10.37,11.67,4.06,-4.44,0.29,9.06,12.73,6.22,-3.26,-2.65,5.44,11.7,8.89,-1.08,-4.09,2.86,9.86,8.7,0.57,-6,-2.49,7.34,11.59,0.89,-5.12,-2.85,3.17,10.47,4.44,-4.07,-10.15,-1.21,5.88,1.63,-4.43,-10.25,-6.72,3.59,3.88,-8.84,-14.02,-9.15,-3.54,-1.21,-3.43,-18.33,-15.42,-5.25,0.88,-3.5,-13.39,-23.34,-11.78,-7.51,-2.09,-14.66,-23.72,-15.55,-13.88,-7.91,-17.42,-24.09,-25.98,-10.64,-9.07,-16.34,-19.74,-24.72,-13.12,-10.55,-11.34,-25.39,-29.25,-17.98,-11.45,-4.53,-14.58,-20.85,-19.13,-11.29,-5.62,-18.76,-25.05,-32.52,-18.38,-12.13,-11.27,-27.56,-33.59,-20.84,-7.45,-4.13,-20.13,-24.45,-25.08,-18.61,-3.51,-14.32,-19.4,-18.03,-13.27,-6.47,-20.64,-16.36,-26.22,-13.28,-13.99,-12.55,-14.05,-23.66,-24.94,-15.08,-11.59,-16.8,-29.42,-29.26,-16.4,-17.04,-20.77,-19.98,-32.26,-15.12,-6.01,-21.12,-21.86,-24.43,-16.77,-21.23,-21.27,-30.68,-34.53,-21.67,-13.42,-17.1,-20.12,-31.16,-26.96,-26.08,-13.38,-24.4,-28.73,-28.48,-18.74,-22.25,-20.36,-21.34,-29.18,-24.37,-13.65,-10.56,-22.6,-23.4,-30.22,-17.37,-16.18,-22.71,-32.23,-24.92,-14.89,-7.62,-9.64,-17.24,-22.54,-19.36,-14.9,-10.29,-17.28,-27.78,-18.27,-15.52,-5.68,-13.39,-15.47,-22.37,-6.94,-3.51,-4.74,-15.67,-19.84,-9.1,1.37,-1.64,-10.73,-14.13,-13.36,-4.56,5.56,-4.46,-9.44,-11.41,-4.15,1.72,0.44,-11.13,-11.66,-1.81,3.49,6.56,-4.14,-8.18,-5.56,3.23,5.46,0.06,-9.1,-5.35,2.28</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B107" t="str">
+        <v>[R_06_标记]</v>
+      </c>
+      <c r="C107" t="str">
+        <v>a: 24.6ms -28.0uv b: 52.7ms 138.7uv</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B108" t="str">
+        <v>[L_06_名字]</v>
+      </c>
+      <c r="C108" t="str">
+        <v>FERG(6)_dRod</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B109" t="str">
+        <v>[L_06_放大器]</v>
+      </c>
+      <c r="C109" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B110" t="str">
+        <v>[L_06_闪光]</v>
+      </c>
+      <c r="C110" t="str">
+        <v>b白色光:3.0cd.m-2,4ms</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B111" t="str">
+        <v>[L_06_闪光背景]</v>
+      </c>
+      <c r="C111" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B112" t="str">
+        <v>[L_06_采样]</v>
+      </c>
+      <c r="C112" t="str">
+        <v>刺激间隔:2.0S</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B113" t="str">
+        <v>[L_06_分析时间]</v>
+      </c>
+      <c r="C113" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B114" t="str">
+        <v>[L_06_数据长度]</v>
+      </c>
+      <c r="C114" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B115" t="str">
+        <v>[L_06_详细数据(uv)]</v>
+      </c>
+      <c r="C115" t="str">
+        <v>14.35,11.36,13.73,18.97,21.71,19.11,13.75,11.01,13.64,18.96,21.59,18.87,13.58,11.1,13.98,19.36,21.87,19.03,13.81,11.58,14.69,20.11,22.46,19.49,14.32,12.32,15.63,21.05,23.22,20.09,14.96,13.15,16.64,22.02,23.97,20.65,15.51,13.86,17.48,22.74,24.47,20.91,15.71,14.19,17.82,22.99,24.38,20.68,15.42,13.92,17.74,22.51,23.47,19.44,13.96,12.44,16.2,20.6,21.52,16.62,11.97,9.93,14.22,18.47,18.8,13.91,6.73,6.39,10.27,14.11,14.26,8.31,2.88,0.96,3.85,8.95,8.02,-0.53,-2.06,-5.88,-4.68,4.63,2.02,-7.76,-7.19,-11.01,-9.42,-4.29,-6.64,-8.22,-9.7,-13.95,-10.41,-6.55,-10.3,-6.23,-15.94,-14.35,-13.88,0.74,1.13,-3.43,-12.32,-10.82,4.08,6.44,9.96,4.38,7.51,2.54,12.62,21.55,21.72,15.97,13.98,21.69,27.55,34.68,40.98,41.65,40.45,47.64,53.21,64.13,67.01,55.48,61.94,67.61,69.51,90.2,92.37,78.83,89.01,96.95,95.91,104.06,117.81,111,108.48,104.85,117.76,141.3,136.92,135.61,114.64,139.68,147.18,141.35,139.32,143.32,160.5,159.89,168.73,181.78,167,170.73,148.75,165.7,166.64,193.63,189.86,174.67,160.99,154.69,165.88,172.38,180.56,186.6,163.96,171.37,197.92,173.73,180.5,172.27,167.65,178.23,157.99,179.24,190.45,170.66,160.58,147.85,153.86,156.12,172.48,160.17,142.04,164.88,141.36,150.79,159.99,122.49,140.24,135.11,123.44,123.41,133.63,105.64,105.82,103.18,118.74,120.89,103.21,91.66,92.49,89.16,99.16,88.11,83.37,88.7,82.68,84.53,83.64,77.53,68.31,65.58,62.24,58.61,64.38,63.92,55.18,48.41,50.82,48.11,49.56,49.21,44.41,35.79,33.67,40.06,42.35,40.93,37.11,29.28,27.95,29.84,31.72,31.53,26.78,19.64,19.01,23.81,26.3,26.99,19.92,15.18,13.93,18.84,22.4,21.78,15.23,10.78,9.92,14.9,18.14,17.73,11.78,7.01,6.96,12,15.27,14.21,8.5,4.56,5,9.68,13.47,12.34,6.57,2.92,3.37,8.67,11.48,10.26,5.93,1.26,3.24,7.6,11.49,9.45,4.57,0.54,2.53,8.25,10.75,8.64,4.42,0.09,2.9,6.42,10.27,8.67,4.95,1.17,2.66,7.47,9.58,9.52,3.77,-0.26,1.36,8.11,9.58,6.78,4.55,0.66,2.78,8.16,10.41,8.12,2.72,-0.13,3.06,6.36,7.46,8.06,0.7,-4.6,0.47,6.92,4.1,4.86,0.98,-2.31,0.92,1.76,7.52,3.25,-4.51,-5.18,-3.62,-2.81,2.14,-5.08,-9.26,-13.09,-10.34,-0.91,1.61,-6.13,-7.77,-8.55,-9.49,-9.54,-6.95,-7.58,-9.9,-13.51,-17.25,-9.41,-8.03,-10.01,-20.02,-16.13,-16.81,-15.32,-13.33,-12.19,-22.8,-14.91,-22.69,-14.08,-9.61,-19.72,-18.99,-16.24,-23.1,-19.32,-17.48,-16.58,-20.17,-16.59,-21.33,-11.59,-12.46,-12.58,-27.86,-23.59,-22.34,-20.56,-8.26,-19.71,-20.1,-19.3,-19.41,-16.71,-6.61,-19.52,-18.25,-18.44,-15.85,-14.02,-10.79,-14.84,-29.65,-16.58,-13.51,-19.94,-8.44,-23.67,-30.03,-24.2,-21.52,-19.01,-9.71,-24.01,-27.97,-23.78,-18.09,-13.5,-19.82,-19.35,-29.4,-23.18,-22.18,-6.82,-14.74,-25.37,-28.58,-26.53,-15.17,-18.78,-17.79,-13.63,-16.9,-15.24,-21.1,-18.72,-10.44,-14.09,-17.76,-20.62,-12.54,-18.68,-13.05,-18.6,-28.39,-26.31,-11.07,-9.75,-8.63,-20.8,-20.99,-20.7,-18.75,-6.56,-10.46,-21.42,-19.07,-16.41,-12.01,-4.73,-10.07,-12.35,-19.11,-13.21,-13.35,-5.36,-12.3,-14.54,-13.95,-18.02,-10.1,-5.3,-10.51,-8.63,-13.83,-12.17,-7.13,-0.7,-5.38,-7.81,-9.87,-6.65,-4.1,-1.75,-1.82,-7.24,-8.28,-5.25,-0.48,2.29,-1.63,-4.56,-8.92,-3.34,2.86,2.85,1.57,-2.21,-6.71,-1.98,1.73,4.54,1.28,-5.5,-7.84,-2.27,3.54,6.33</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B116" t="str">
+        <v>[L_06_标记]</v>
+      </c>
+      <c r="C116" t="str">
+        <v>a: 24.4ms -29.5uv b: 52.8ms 186.9uv</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B117" t="str">
+        <v>[R_07_名字]</v>
+      </c>
+      <c r="C117" t="str">
+        <v>FERG(7)_dMax</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B118" t="str">
+        <v>[R_07_放大器]</v>
+      </c>
+      <c r="C118" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B119" t="str">
+        <v>[R_07_闪光]</v>
+      </c>
+      <c r="C119" t="str">
+        <v>b白色光:3.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B120" t="str">
+        <v>[R_07_闪光背景]</v>
+      </c>
+      <c r="C120" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B121" t="str">
+        <v>[R_07_采样]</v>
+      </c>
+      <c r="C121" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B122" t="str">
+        <v>[R_07_分析时间]</v>
+      </c>
+      <c r="C122" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B123" t="str">
+        <v>[R_07_数据长度]</v>
+      </c>
+      <c r="C123" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B124" t="str">
+        <v>[R_07_详细数据(uv)]</v>
+      </c>
+      <c r="C124" t="str">
+        <v>-8.28,-24.43,-14.17,3.05,-5.92,-22.53,-13.15,4.61,-3.39,-20.45,-12.01,6.21,-0.82,-18.32,-10.87,7.71,1.63,-16.28,-9.88,8.98,3.84,-14.46,-9.16,9.9,5.69,-12.97,-8.81,10.37,7.08,-11.9,-8.9,10.34,7.97,-11.28,-9.46,9.77,8.33,-11.13,-10.48,8.68,8.19,-11.41,-11.94,7.13,7.6,-12.08,-13.76,5.17,6.6,-13.04,-15.86,2.86,5.32,-14.28,-18.23,0.3,3.58,-15.84,-20.93,-2.69,1.8,-17.42,-23.88,-6.34,-0.71,-20.24,-26.77,-10.03,-4.86,-22.43,-32.75,-16.32,-9.1,-27.98,-37.41,-22.44,-12.06,-33.48,-44.71,-32.14,-23.53,-43.25,-51.88,-36.34,-32.28,-43.1,-60.05,-49.58,-31.22,-47.79,-65.93,-45.39,-35.42,-55.09,-67.44,-65.33,-36.97,-64.76,-69.98,-58.77,-47.25,-60,-66.42,-53.44,-34.24,-42.02,-61.83,-42.06,-19.22,-14.63,-25.82,-9.41,15.1,-3,-9.64,4.38,33.02,26.8,21.92,38.67,49.69,60.97,42.2,62.32,84.34,95.6,86.78,93.03,117.5,121.48,110.49,109.62,161.77,142.32,152.27,153.23,174.77,174.73,171.35,169.15,235.33,240.3,194.3,195.77,237.08,251.42,216.6,223.85,235.43,250.34,243.8,258.98,267.29,273.86,253.93,263.5,329.8,314.87,286.18,247.97,281.43,282.62,271.99,261.68,335.66,277.49,292.38,296.62,269.91,316.94,262.75,286.65,281.94,248.5,255.41,223.99,273.21,284.36,216.45,203.52,220.8,225,224.28,198.37,189.11,221.91,180.06,184.96,171.74,194.21,174.44,161.87,143.28,169.31,146.17,134.21,149.03,152.11,116.83,96.85,110.04,134.45,115.48,81.24,118.7,117.88,110.02,69.82,95.23,107.69,88.89,63.27,88.17,101.51,84.42,57.22,78.06,75.51,71.65,64.97,74.89,88.73,73.42,53.08,64.81,71.21,60.66,36.82,63.45,80.61,66.92,50.01,51.95,53.82,41.44,33.66,52.67,49.2,42.15,27.84,26.89,54.55,31.95,27.79,18.8,46.29,39.46,9.17,18.71,35.73,31.74,16.4,8.5,32.32,32.46,5.26,10.3,30.49,20.68,-2.72,6.76,22.02,18.1,1.54,-2.81,17.59,14.94,-2.35,-5.41,16.91,12.75,-3.13,-6.7,14.25,16,-4.83,-6.25,13.92,12.17,-6.77,-6.81,9.28,11.01,-6.89,-10.55,9.79,10.98,-4.81,-10.72,6.98,13.83,-6.37,-12.95,7.23,12.47,-6.71,-13.58,3.95,12.97,-4.79,-16.7,1.9,10.31,-8.43,-16.21,0.05,5.15,-11.56,-21.54,-0.91,2.86,-10.07,-25.65,-10.36,2,-16.99,-25.21,-7.57,0.8,-15.46,-27.84,-17.81,-4.72,-20.2,-31.01,-20.99,-9.11,-19.64,-31.92,-17.99,-6.37,-24.87,-34.2,-21.9,-11.42,-25.58,-39.02,-27.05,-13.91,-20.69,-38.57,-34.62,-9.26,-28.6,-37.29,-27.63,-13.5,-19.69,-38.36,-31.63,-18.56,-23.79,-47.33,-27.78,-16.19,-18.73,-41.44,-27.38,-17.64,-20.22,-34.13,-37.77,-9.13,-24.22,-40.4,-30.68,-8.15,-16.37,-38.33,-39.9,-17.48,-18.17,-42.37,-25.91,-17.09,-10.08,-36.7,-26.8,-12.24,-21.88,-32.37,-31.5,-6.81,-18.41,-36.84,-42.34,-11.8,-17.32,-33.98,-41.77,-20.35,-11.12,-33.29,-38.62,-19.51,-19.45,-31.15,-44.06,-27.84,-18.31,-31.56,-48.09,-15.86,-24.97,-28.68,-48.07,-29.36,-25.35,-37.15,-40.2,-25.1,-19.53,-42.73,-42.09,-22.88,-18.99,-40.02,-46.95,-22.35,-21.43,-45.78,-41.27,-27.55,-23.28,-35.73,-41.24,-24.17,-27.21,-37.86,-46.02,-35.25,-23.04,-37.1,-42.08,-29.88,-10.06,-35.2,-41.87,-31.65,-12.81,-24.28,-42.39,-24.18,-17.27,-19.38,-41.19,-20.93,-4.2,-20.21,-38.19,-25.1,-2.69,-17.66,-34.09,-17.85,1.78,-19.78,-29.07,-21.1,1.5,-7.13,-28.31,-14.61,6.77,-9.18,-25.5,-17.52,-0.69,-8.44,-16.87,-15.32,3.66,2.09,-23.03,-9.64,7.05,-3.25,-17.18,-13.97,7.04,2.96,-18.07,-14.89,8.62,-0.08,-17.13,-14.5,6.36,3.83,-14.07,-11.77,5.45,2.67,-15.95,-16.65,4.64,5.89,-17.86,-14.68,2.77</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B125" t="str">
+        <v>[R_07_标记]</v>
+      </c>
+      <c r="C125" t="str">
+        <v>a: 26.0ms -52.3uv b: 55.1ms 200.4uv</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B126" t="str">
+        <v>[L_07_名字]</v>
+      </c>
+      <c r="C126" t="str">
+        <v>FERG(7)_dMax</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B127" t="str">
+        <v>[L_07_放大器]</v>
+      </c>
+      <c r="C127" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B128" t="str">
+        <v>[L_07_闪光]</v>
+      </c>
+      <c r="C128" t="str">
+        <v>b白色光:3.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B129" t="str">
+        <v>[L_07_闪光背景]</v>
+      </c>
+      <c r="C129" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B130" t="str">
+        <v>[L_07_采样]</v>
+      </c>
+      <c r="C130" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B131" t="str">
+        <v>[L_07_分析时间]</v>
+      </c>
+      <c r="C131" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B132" t="str">
+        <v>[L_07_数据长度]</v>
+      </c>
+      <c r="C132" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B133" t="str">
+        <v>[L_07_详细数据(uv)]</v>
+      </c>
+      <c r="C133" t="str">
+        <v>-16.59,-20.52,-6.67,1.69,-9.32,-20.46,-12.25,1.78,-1.8,-16.35,-16.47,-1.38,3.74,-9.25,-17.57,-6.41,5.78,-1.21,-14.86,-11.28,3.98,5.42,-8.89,-14,-0.75,8.75,-1.42,-13.42,-6.57,7.75,5.28,-9.52,-11.47,2.92,9.14,-3.62,-13.67,-3.84,8.29,2.09,-13.16,-11.15,3.36,4.41,-9.79,-17.37,-6.57,2.67,-5.87,-21.13,-16.22,-2.12,-3.78,-22.12,-28.25,-14.84,-5.35,-19.91,-34.9,-24.95,-14.59,-21.23,-41.54,-41.04,-22.93,-28.39,-43.76,-54.46,-43.49,-31.76,-41.19,-52.25,-47.18,-35.59,-35.96,-56.49,-68.36,-37.82,-38.15,-44.26,-54.59,-48.31,-43.33,-43.1,-50.55,-56.37,-38.85,-35.17,-34.15,-45.16,-25.77,-5.88,-6.68,-22.21,-4.25,15.5,13.16,3.07,9.48,23.12,43.02,47.43,43.08,38.6,84.4,59.15,60.71,80.74,82.43,107.99,109.68,121.7,110.55,140.75,135.59,139.31,163.31,194.07,204.19,157.76,193.66,197.35,227.81,237.48,230.59,242.24,231.88,233.55,237.97,215.92,238.46,296.5,295.24,227.87,251.52,263.97,280.12,265.52,249.94,313.41,279.11,262.94,309.65,284.96,302.83,320.28,307.82,256.63,271.07,333.08,307.38,315.1,277.43,288.38,287.44,305.4,265.69,300.93,279.35,288.73,265.5,264.99,244.42,249.24,225.34,231.79,270.88,243.21,231.11,213.39,203.44,246.19,194.47,212.42,192.03,192.73,186.31,185.26,177.2,198.22,177.03,142.69,159.64,159.1,159.55,168.41,131.8,138.56,166.24,153.82,132.7,133.4,126.61,144,124.53,106.59,105.97,113.58,102.82,87.78,84.13,117.42,99.42,81.55,78.49,92.51,104.85,86.95,87.01,70,95.97,76.05,57.15,73.15,70.36,76.58,52.36,57.64,60.35,58.54,68.87,40.04,35.27,55.18,52.2,47.48,35.11,45.23,54.98,47.82,24.62,35.06,39.88,40.39,18.09,20.51,28.89,27.48,23.97,9.21,9.43,26.85,22.71,-1.05,3.88,12.07,12.84,5.18,-4.14,0.56,14.03,3.05,-15.97,-10.6,3.99,2.85,-12.89,-13.46,-2.87,3.63,-11.26,-19.27,-12.86,-2.08,-7.26,-22.3,-21.25,-4.78,-4.14,-15.17,-24.42,-11.1,-3.75,-12.13,-25.57,-18.89,-6.68,-5.17,-22.42,-24.77,-11.33,-5.46,-16.28,-28.07,-17.44,-2.14,-10.36,-23.14,-24.27,-10.89,-2.32,-19.6,-23.76,-13.97,-5.11,-9.2,-25.62,-21.57,-9.24,-9.63,-21.06,-25.48,-16.52,-3.75,-18.37,-33.52,-21.4,-8.53,-8.89,-29.98,-27.07,-16.37,-7.9,-23.66,-35.15,-24.33,-16.24,-17.56,-37.01,-35.68,-18.62,-19.41,-35.02,-39.85,-33.9,-22.13,-30.22,-40.13,-41.28,-28.33,-23.22,-40.71,-43.43,-27.97,-22.22,-42.53,-51.03,-46.31,-27.29,-38.62,-50.75,-49.53,-32.43,-30.58,-38.66,-59.45,-35.14,-28.44,-40.95,-53.51,-48.61,-29.55,-31.48,-50.41,-57.06,-37.24,-32.72,-37.68,-62.27,-47.4,-40.92,-34.41,-57.5,-53.17,-40.11,-23.89,-43.52,-53.87,-45.3,-24.75,-38.1,-58.58,-40.05,-27.77,-31.82,-40.26,-57.9,-29.62,-24.67,-41.76,-56.38,-50.63,-25.26,-27.82,-42.79,-45.03,-38.84,-30.07,-37.21,-45.41,-41.25,-35.17,-36.79,-38.96,-39.72,-27.33,-25.27,-46.47,-51.41,-43.19,-33.89,-40.43,-48.8,-47.98,-23.1,-31.95,-49.23,-43.05,-34.57,-27.56,-42.6,-50.66,-44.67,-28.94,-29.56,-45.81,-45.3,-36.04,-35.2,-40.39,-47.83,-41.05,-33.71,-38.46,-49.65,-46.53,-33.81,-28,-49.27,-45.06,-41.61,-31.21,-45.54,-54.3,-42.61,-29.98,-33.56,-48.95,-41.74,-34.77,-29.39,-43.97,-52.66,-34.09,-26.17,-35.53,-47.36,-45.9,-29.25,-19.47,-41.61,-39.18,-32.47,-21.19,-28.98,-37.44,-29.79,-17.41,-19.93,-33.61,-33.12,-23.94,-13.29,-24.19,-30.92,-27.46,-7.21,-17.77,-29.23,-30.71,-11.49,-6.56,-20.5,-30.99,-18.27,-4.24,-16.39,-28.73,-23.74,-7.95,-4.38,-23.75,-24.15,-8.95,-3.8,-13.62,-26.17,-19.52,-4.02,-6.35,-22.63,-23.72,-6.68,-2.52,-19.56,-28.01,-13.96,-5.31,-12.39,-27.62</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B134" t="str">
+        <v>[L_07_标记]</v>
+      </c>
+      <c r="C134" t="str">
+        <v>a: 25.8ms -58.1uv b: 55.1ms 266.5uv</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B135" t="str">
+        <v>[R_08_名字]</v>
+      </c>
+      <c r="C135" t="str">
+        <v>FERG(8)_dOps</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B136" t="str">
+        <v>[R_08_放大器]</v>
+      </c>
+      <c r="C136" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B137" t="str">
+        <v>[R_08_闪光]</v>
+      </c>
+      <c r="C137" t="str">
+        <v>b白色光:3.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B138" t="str">
+        <v>[R_08_闪光背景]</v>
+      </c>
+      <c r="C138" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B139" t="str">
+        <v>[R_08_采样]</v>
+      </c>
+      <c r="C139" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B140" t="str">
+        <v>[R_08_分析时间]</v>
+      </c>
+      <c r="C140" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B141" t="str">
+        <v>[R_08_数据长度]</v>
+      </c>
+      <c r="C141" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B142" t="str">
+        <v>[R_08_详细数据(uv)]</v>
+      </c>
+      <c r="C142" t="str">
+        <v>-5.82,7.05,7.49,-5.13,3.74,10.7,-2.59,0.18,11.92,1.36,-2.69,11.02,5.82,-3.98,8.27,9.67,-3.5,4.32,11.96,-1.34,0.01,11.98,1.75,-3.66,9.65,5.18,-5.67,5.72,7.83,-5.8,1.04,9.36,-3.64,-3.34,9.23,-0.02,-6.24,7.4,3.99,-7.22,3.65,6.87,-6.78,-1.53,7.36,-5.39,-6.89,5.39,-3.75,-11.69,0.75,-1.75,-14.73,-4.86,0.01,-14.8,-9.01,0.88,-10.45,-11.67,2.63,-4.05,-10.76,3,3.61,-9.22,2.8,8.15,-5.5,-2.83,9.17,-3.63,-8.21,3.95,-4.33,-14.78,-3.32,-4.95,-17.75,-11.19,-3.64,-19.45,-15.46,-3.07,-11.2,-11.92,4.4,1.51,-4.9,10.91,15.49,4.96,13.2,24.25,10.02,8.54,19.03,8.55,1.34,10.72,1.82,-12.13,-6.25,-8.54,-25.16,-17.46,-7.43,-23.44,-24.1,-6,-13.02,-14.44,3.02,4.36,-2.24,15.18,23.1,12.29,22.7,27.46,15.78,14.95,23.26,11.88,0.16,8.09,0.18,-18.05,-12.69,-14.7,-32.64,-30.17,-21.71,-31.35,-33.16,-20.04,-22.71,-27.9,-7.15,-2.73,-8.75,8.62,15.23,4.78,14.36,23.23,19.35,8.57,24.36,8.81,-3.65,3.42,-2.28,-21.33,-19.44,-14.11,-37.47,-37.7,-28.13,-38.46,-40.18,-21.66,-21.85,-27.72,-8.51,-2.91,-11.13,2.26,14.21,7.05,13.01,20.9,15.09,10.87,21.47,9.78,-2.1,5.38,3.72,-13.25,-9.33,-5.2,-19.71,-22.34,-8.51,-19.41,-24.78,-8.7,-9.52,-17.44,-3.26,2.52,-8.04,1.21,11.39,2.66,1.57,15.93,7.62,1.24,12.25,6.84,-6.3,3.38,4.79,-10.83,-7.27,0.77,-13.41,-15.27,-1.89,-10.85,-19.17,-5.6,-5.72,-17.26,-6.69,-0.63,-13.37,-8.17,2.84,-8.42,-10.63,2.54,-4.65,-12.99,-1.06,-2.83,-16.05,-7.14,-2.12,-16.39,-13.62,-2.94,-14.97,-18.47,-5.27,-11.34,-20.58,-8.09,-6.91,-19.86,-10.84,-3.56,-16.64,-14,-1.85,-12.25,-16.44,-2.64,-7.5,-17.4,-5.28,-3.57,-16.66,-8.96,-0.98,-14.04,-12.68,-0.27,-9.88,-15.19,-1.3,-5.14,-15.74,-3.86,-0.9,-14.14,-7.15,1.84,-10.74,-10.37,2.53,-6.34,-12.58,1.03,-1.88,-13.21,-2.21,1.58,-11.99,-6.26,3.29,-9.16,-10.15,2.83,-5.45,-12.9,0.28,-1.79,-13.9,-3.79,0.81,-13,-8.49,1.61,-10.54,-12.8,0.26,-7.29,-15.81,-3.06,-4.2,-16.94,-7.71,-2.22,-16.08,-12.71,-2,-13.64,-17.01,-3.79,-10.4,-19.74,-7.32,-7.32,-20.39,-11.88,-5.32,-18.94,-16.5,-5.04,-15.89,-20.14,-6.64,-12.07,-22,-9.81,-8.51,-21.68,-13.81,-6.1,-19.26,-17.66,-5.44,-15.34,-20.39,-6.65,-10.84,-21.27,-9.38,-6.78,-19.99,-12.85,-4.08,-16.77,-16.11,-3.28,-12.28,-18.21,-4.45,-7.5,-18.52,-7.17,-3.47,-16.81,-10.63,-1.05,-13.38,-13.86,-0.72,-8.97,-15.95,-2.46,-4.57,-16.3,-5.77,-1.19,-14.77,-9.77,0.37,-11.7,-13.47,-0.27,-7.86,-15.97,-2.97,-4.23,-16.7,-7.13,-1.77,-15.56,-11.83,-1.21,-12.95,-16.01,-2.8,-9.65,-18.8,-6.31,-6.63,-19.67,-11.04,-4.82,-18.59,-16.01,-4.84,-16.01,-20.17,-6.87,-12.75,-22.69,-10.59,-9.78,-23.1,-15.25,-8,-21.47,-19.84,-7.98,-18.32,-23.35,-9.85,-14.53,-25.01,-13.21,-11.11,-24.47,-17.3,-8.93,-21.88,-21.11,-8.54,-17.88,-23.69,-10,-13.41,-24.34,-12.9,-9.51,-22.84,-16.43,-7.04,-19.45,-19.6,-6.49,-14.88,-21.53,-7.88,-10.14,-21.59,-10.73,-6.24,-19.63,-14.2,-4.04,-16.02,-17.31,-3.94,-11.53,-19.18,-5.87,-7.15,-19.26,-9.26,-3.91,-17.47,-13.24,-2.56,-14.22,-16.79,-3.41,-10.3,-19.05,-6.28,-6.72,-19.5,-10.52,-4.42,-18.12,-15.17,-4.07,-15.34,-19.19,-5.88,-12,-21.75,-9.56,-9.07,-22.37,-14.37,-7.44,-21.07,-19.29,-7.7,-18.37,-23.31,-9.98,-15.11,-25.61,-13.88,-12.26,-25.79,-18.62,-10.71,-23.98,-23.17,-10.96,-20.74,-26.54</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B143" t="str">
+        <v>[R_08_标记]</v>
+      </c>
+      <c r="C143" t="str">
+        <v>59.7uv</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B144" t="str">
+        <v>[L_08_名字]</v>
+      </c>
+      <c r="C144" t="str">
+        <v>FERG(8)_dOps</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B145" t="str">
+        <v>[L_08_放大器]</v>
+      </c>
+      <c r="C145" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B146" t="str">
+        <v>[L_08_闪光]</v>
+      </c>
+      <c r="C146" t="str">
+        <v>b白色光:3.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B147" t="str">
+        <v>[L_08_闪光背景]</v>
+      </c>
+      <c r="C147" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B148" t="str">
+        <v>[L_08_采样]</v>
+      </c>
+      <c r="C148" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B149" t="str">
+        <v>[L_08_分析时间]</v>
+      </c>
+      <c r="C149" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B150" t="str">
+        <v>[L_08_数据长度]</v>
+      </c>
+      <c r="C150" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B151" t="str">
+        <v>[L_08_详细数据(uv)]</v>
+      </c>
+      <c r="C151" t="str">
+        <v>11.39,-7.53,-7.63,12.44,4.91,-10.7,4.84,14.65,-4.5,-5,15.02,7.16,-8.9,6.22,15.74,-3.64,-4.72,15,7.34,-9.14,6.1,15.87,-3.4,-4.67,15.39,8.14,-7.98,7.17,17.26,-1.48,-2.56,17.37,9.98,-6.8,7.24,17.05,-2.9,-5.21,13.39,4.97,-12.78,0.26,9.3,-11.45,-13.36,5.61,-3.18,-19.24,-4.94,5.32,-13.65,-14.62,6.44,0.4,-14.71,0.33,11.89,-5.64,-8.53,10.84,4.34,-11.52,-0.34,9.55,-11.87,-15.85,1.54,-6.84,-27.37,-15.1,-6.34,-26.91,-28.36,-7.95,-11.73,-29.03,-11.76,0.88,-14.03,-12.69,10.45,8.57,-7.32,12.74,25.02,4.41,0.97,21.44,15.64,-3.94,5.93,13.54,-9.17,-16.99,-1.02,-10.59,-28.02,-19.02,-6.72,-23.02,-26.46,-2.4,-7.82,-19.7,-0.02,16.73,2.67,4.89,27.67,31.46,16.92,27.51,44.24,17.04,15.12,27.6,16.88,-5.23,1.64,6.91,-17.06,-26.85,-13.85,-14.92,-42.84,-22.85,-17.42,-27.25,-27.67,-1.48,-1.67,-14.54,5.23,20.79,6.64,4.84,34.37,22.28,10.91,21.59,27.82,6.93,-2.32,10.75,-1.55,-26.81,-18.89,-10.53,-31.92,-38.56,-19.6,-23.28,-46.18,-28.95,-10.47,-27.89,-26.67,-0.55,0.56,-12.07,3.44,21.81,4.87,3.16,17.86,19.39,-3.69,5.48,15.46,-6.57,-15.33,0.69,-6.23,-29.1,-16.71,-6.07,-25.48,-30.56,-10.05,-9.74,-26.4,-10.63,5.96,-8.36,-10.5,12.05,12,-5.07,9.11,24.84,5.79,1.75,19.34,14.76,-5.45,3.5,15.05,-4.56,-11.87,6.91,0.92,-16.64,-5.99,5.95,-9.5,-16.58,5,2.59,-14.67,-2.24,12.39,-3.93,-9.8,10.47,7.93,-10.12,0.25,12.8,-4.63,-11.63,6.67,2.86,-16.93,-6.95,5.75,-12.17,-19.36,-0.27,-3.05,-22.34,-11.92,1.97,-15,-21.29,-1.4,-3.68,-22.45,-11.63,2.67,-14.39,-21.06,-1.07,-3.41,-22.41,-11.79,2.08,-14.92,-21.7,-1.99,-4.04,-23.08,-12.64,1.94,-14.72,-21.55,-1.43,-2.95,-21.68,-11,3.96,-12.31,-18.97,1.32,0.1,-18.56,-8,7.03,-9.15,-16.07,4.09,3.01,-15.83,-5.53,9.53,-6.68,-13.85,6.21,5.15,-13.82,-3.8,11.28,-4.92,-12.39,7.52,6.5,-12.67,-2.97,12.06,-4.22,-12.04,7.63,6.6,-12.84,-3.5,11.43,-4.95,-13.14,6.29,5.25,-14.42,-5.42,9.47,-6.96,-15.46,3.82,2.83,-16.99,-8.24,6.69,-9.7,-18.42,0.78,-0.05,-19.92,-11.33,3.72,-12.53,-21.37,-2.15,-2.73,-22.57,-14.04,1.24,-14.79,-23.66,-4.33,-4.59,-24.3,-15.77,-0.21,-15.94,-24.78,-5.3,-5.18,-24.74,-16.16,-0.28,-15.7,-24.5,-4.87,-4.38,-23.78,-15.18,0.98,-14.15,-22.95,-3.21,-2.39,-21.7,-13.14,3.24,-11.67,-20.55,-0.78,0.29,-19.01,-10.59,5.92,-8.87,-17.92,1.78,2.98,-16.4,-8.21,8.33,-6.44,-15.75,3.79,5.04,-14.51,-6.64,9.84,-4.97,-14.61,4.69,5.94,-13.84,-6.32,10.06,-4.83,-14.83,4.22,5.44,-14.56,-7.4,8.89,-6.07,-16.4,2.42,3.66,-16.52,-9.68,6.58,-8.38,-18.99,-0.32,1.01,-19.27,-12.67,3.64,-11.23,-22.01,-3.4,-1.89,-22.18,-15.7,0.76,-13.93,-24.79,-6.15,-4.35,-24.55,-18.12,-1.42,-15.84,-26.69,-7.95,-5.8,-25.84,-19.39,-2.41,-16.5,-27.31,-8.42,-5.9,-25.75,-19.27,-2,-15.77,-26.53,-7.53,-4.64,-24.34,-17.86,-0.34,-13.83,-24.6,-5.53,-2.35,-21.95,-15.56,2.14,-11.16,-22.03,-2.98,0.41,-19.2,-12.98,4.78,-8.41,-19.47,-0.55,2.94,-16.77,-10.82,6.92,-6.26,-17.61,1.1,4.62,-15.27,-9.66,7.99,-5.24,-16.92,1.52,5.02,-15.07,-9.84,7.69,-5.6,-17.63,0.55,4.02,-16.26,-11.39,6.06,-7.27,-19.6,-1.65,1.86,-18.56,-13.98,3.44,-9.85,-22.41,-4.6,-0.97,-21.44,-17.06,0.43,-12.73,-25.41,-7.65,-3.8,-24.21,-19.94,-2.29,-15.21,-27.93</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B152" t="str">
+        <v>[L_08_标记]</v>
+      </c>
+      <c r="C152" t="str">
+        <v>57.6uv</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B153" t="str">
+        <v>[R_09_名字]</v>
+      </c>
+      <c r="C153" t="str">
+        <v>FERG(9)_dMax</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B154" t="str">
+        <v>[R_09_放大器]</v>
+      </c>
+      <c r="C154" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B155" t="str">
+        <v>[R_09_闪光]</v>
+      </c>
+      <c r="C155" t="str">
+        <v>b白色光:20.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B156" t="str">
+        <v>[R_09_闪光背景]</v>
+      </c>
+      <c r="C156" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B157" t="str">
+        <v>[R_09_采样]</v>
+      </c>
+      <c r="C157" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B158" t="str">
+        <v>[R_09_分析时间]</v>
+      </c>
+      <c r="C158" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B159" t="str">
+        <v>[R_09_数据长度]</v>
+      </c>
+      <c r="C159" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B160" t="str">
+        <v>[R_09_详细数据(uv)]</v>
+      </c>
+      <c r="C160" t="str">
+        <v>2.77,-6.18,-1.08,1.08,-6.94,1.47,-1.8,-6.03,2.66,-4.89,-3.83,2,-7.14,-1.2,-0.36,-7.87,0.8,-3.7,-6.91,1.3,-6.95,-4.81,-0.04,-9.15,-2.41,-2.9,-9.73,-0.97,-6.59,-8.61,-0.94,-9.7,-6.47,-2.83,-11.99,-4.49,-6.32,-12.22,-3.36,-10.25,-11.38,-4.2,-14.13,-9.92,-7.01,-15.25,-7.6,-11.72,-16.25,-7.32,-14.59,-16.6,-11.67,-20.13,-14.63,-15.28,-24.24,-13.34,-21.39,-24.75,-16.81,-28.7,-23.63,-21.16,-29.72,-23.12,-25.07,-29.53,-29.23,-36.06,-31.67,-23.13,-33.9,-39.46,-35.56,-33.35,-30.94,-37.1,-38.46,-36.66,-31.17,-36.55,-33.3,-43.54,-30.35,-23.17,-40.36,-20.07,-23.09,-20.05,-11.71,-15.52,-28.07,1.66,-15.9,12.1,15.11,13.09,15.87,27.92,12.03,33.13,28.73,39.58,60.73,43.59,69.01,77.11,69.74,84.8,100.99,94.74,104.81,96.2,120.15,145.75,151.2,162.83,157.77,174.33,198.69,177.11,166.81,203.05,182.08,239.7,221.8,207.63,222.1,233.59,262.55,239.2,262.57,272.02,307.63,252.51,288.16,305.71,276.96,278.16,294.01,277.88,278.91,318.34,311.46,358.51,292.56,327.51,297.55,357.16,342.57,292.7,292.94,317,343.7,350.15,331.68,292.01,325.31,330.25,327.04,353.24,311.16,321.31,348.66,303.39,321.57,281.31,308.48,318.06,316.17,289.91,260.25,257.9,295.29,276.68,262.89,280.11,277.94,271.36,240.1,227.19,264.29,235.59,248.51,229.92,211.56,187.39,222.77,198.3,186.78,198.23,192.9,192.25,166.52,179.78,167.31,166.3,159.84,136.69,148.03,132.92,157.18,150.29,120.37,152.22,138.96,115.4,134.97,120.31,101.33,99.15,89.43,96.38,105.93,98.43,88.6,97.01,92.04,83.9,62.52,77.39,75.38,68.94,76.39,58.86,55.41,69.22,55.89,61.92,65.46,54.16,51.47,37.63,40.9,40.13,33.29,42.19,44.27,38.32,31.11,38.45,25.04,26.39,26.66,16.46,26.3,15.41,19.86,14.27,6.58,17.48,15.35,9.07,16.98,3.62,6.51,6.88,-0.96,1.49,6.2,-7.56,3.02,1.46,-10.06,0.93,-6.96,-7.17,-2.6,-10.19,-5.76,-4.76,-12.95,-7.19,-8.97,-15.87,-8.28,-16.15,-15.35,-10.88,-17.4,-14.81,-12.16,-22.96,-13.89,-18.64,-22.78,-15.37,-21.25,-20.21,-16.97,-26.32,-18.57,-17.95,-29.71,-17.52,-21.41,-24.93,-17.65,-31.82,-29.13,-22.59,-34.38,-28.51,-24.37,-30.36,-26.11,-30.08,-35.2,-29.29,-35.8,-30.14,-28.92,-33.26,-34.03,-27.1,-40.33,-25.91,-36.4,-35.92,-33.74,-40.15,-39.52,-28.56,-40.82,-28.63,-32.73,-45.45,-34.44,-37.08,-43.93,-33.02,-43.92,-32.51,-35.12,-39.85,-36.53,-35.12,-47.26,-29.41,-37.5,-44.14,-34.05,-48.02,-32.31,-43.8,-51.67,-31.83,-38.84,-42.92,-31.77,-44.92,-46.38,-37.37,-46.6,-41.94,-40.81,-48,-38.55,-39.31,-41.57,-43.19,-40.89,-44.36,-34.69,-46.59,-40.28,-45.81,-53.34,-44.31,-50.86,-46.38,-45.64,-54.19,-57.2,-41.6,-62.1,-50.51,-52.3,-46.54,-48.14,-60.04,-58.56,-54.52,-53.49,-41.96,-56.26,-59.68,-46.5,-44.46,-59.36,-53.5,-48.02,-57.92,-51.87,-64.61,-42.08,-44.54,-66.73,-40.01,-64,-58.32,-51.79,-53.37,-48.65,-40.51,-60.02,-49.44,-47.42,-60.14,-55.4,-54.1,-60.61,-54.17,-47.11,-54.6,-49.49,-62.08,-47.24,-45.62,-53.18,-42.97,-45.85,-48.85,-39.29,-43.94,-51.22,-41.01,-57.05,-37.45,-41.07,-47.84,-45.17,-39.59,-50.88,-44.83,-45.62,-36.4,-43.12,-46.7,-39.79,-40.14,-44.47,-36.31,-48.59,-37.59,-31.77,-37.65,-37.7,-30.75,-35.96,-31.34,-43.06,-37.72,-36.5,-41.2,-33.56,-29.35,-41.97,-31.52,-29.7,-40.14,-26.76,-39.7,-35.44,-31.16,-39.46,-36.12,-29.65,-36.93,-27.38,-35.33,-38.8,-28.04,-31.35,-31.48,-27.26,-38.56,-27.73,-32.67,-38.57,-25.48,-34.1,-31.75,-27.17,-33.51,-32.33,-28.89,-32.56,-25.87,-27.25,-33.44,-22.55,-30.48,-31.98,-23.62,-32.65,-26.3,-25.56,-30.95</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B161" t="str">
+        <v>[R_09_标记]</v>
+      </c>
+      <c r="C161" t="str">
+        <v>a: 29.5ms -75.6uv b: 62.0ms 254.6uv</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B162" t="str">
+        <v>[L_09_名字]</v>
+      </c>
+      <c r="C162" t="str">
+        <v>FERG(9)_dMax</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B163" t="str">
+        <v>[L_09_放大器]</v>
+      </c>
+      <c r="C163" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B164" t="str">
+        <v>[L_09_闪光]</v>
+      </c>
+      <c r="C164" t="str">
+        <v>b白色光:20.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B165" t="str">
+        <v>[L_09_闪光背景]</v>
+      </c>
+      <c r="C165" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B166" t="str">
+        <v>[L_09_采样]</v>
+      </c>
+      <c r="C166" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B167" t="str">
+        <v>[L_09_分析时间]</v>
+      </c>
+      <c r="C167" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B168" t="str">
+        <v>[L_09_数据长度]</v>
+      </c>
+      <c r="C168" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B169" t="str">
+        <v>[L_09_详细数据(uv)]</v>
+      </c>
+      <c r="C169" t="str">
+        <v>-3.85,-3.04,-16.22,-1.83,-4.33,-15.58,-0.22,-5.92,-14.75,0.92,-7.73,-13.75,1.54,-9.68,-12.64,1.63,-11.69,-11.45,1.16,-13.66,-10.24,0.18,-15.51,-9.05,-1.28,-17.15,-7.93,-3.14,-18.52,-6.93,-5.34,-19.54,-6.1,-7.76,-20.17,-5.45,-10.3,-20.38,-5.03,-12.86,-20.18,-4.85,-15.33,-19.59,-4.93,-17.62,-18.58,-5.33,-19.62,-17.31,-5.98,-21.28,-15.88,-7.05,-22.69,-14.43,-8.59,-24.16,-12.84,-9.89,-25.2,-12.44,-12.93,-26,-11.59,-14.96,-27.48,-12.23,-20.02,-29.2,-12.9,-23.24,-30.63,-17.47,-25.98,-29.51,-17.67,-35.05,-31.18,-25.77,-36.27,-37.92,-27.94,-50.72,-37.89,-33.56,-57.87,-38.67,-48.11,-56.71,-50.8,-39.48,-57.97,-48.87,-43.23,-61.43,-50.82,-47,-55.73,-44.45,-64.55,-64.42,-43.05,-51.83,-51.74,-27.97,-40.46,-39.12,-19.31,-21.3,-25.26,-7.63,-24.37,-13.28,10.7,-0.69,20.93,29.11,25.59,44.22,45.9,46.65,55.92,76.03,83.77,109.98,86.22,91.21,140.09,125.01,114.15,169.93,150.7,142.09,184.91,191.35,196.24,189.6,207.97,223.29,209.88,239.52,220.76,259.12,236.73,285.95,249.95,244.39,256.7,289.33,281.29,281.81,277.47,316.8,341.21,338.37,336.48,354.23,309.81,298.92,369.66,294.25,320.89,363.12,330.39,328.38,321.32,299.34,310.29,373.72,283.77,304.26,361.62,315.23,298.92,335.58,285.59,283.32,285.35,264.72,306.22,255.82,244.51,265.63,266.99,263.41,255.96,258.23,233.4,236,216.98,192.49,203.4,210.68,202.9,178.98,178.66,172.64,190.19,161.7,135.99,164.27,142.31,146.26,157.42,137.48,124.3,128.88,120.42,121.48,103.5,91.47,120.43,118.83,72.43,110.18,77.83,78.45,90.36,91.66,86.97,73.28,79.13,71,90.32,70.95,50.76,77.1,73.17,71.11,60.47,64.14,68.02,60.7,54.57,38.56,67.55,43.69,49.17,41.73,24.42,52.74,45.49,32.07,33.48,43.16,22.65,32.6,27.32,15.93,44.21,33.25,19.24,31.53,14.77,10.06,24.51,20.76,18.7,26.97,12.18,11.35,18.94,3.1,17.07,19.39,5.71,12.88,19.17,2.11,14.25,11.93,0.53,9.7,8.37,-9.3,11.06,3.46,-7.09,7.35,-1.17,-12.82,6.34,-8.2,-13.57,2.24,-9.28,-9.43,-0.1,-14.66,-10.26,0.91,-18.69,-12.46,-3.41,-21.59,-11.74,-7.01,-23.09,-15.7,-13.55,-26.56,-16.59,-14.94,-25.45,-12.6,-16.98,-30.58,-17.44,-19.08,-31.08,-13.53,-23.58,-27.05,-17.51,-26.77,-30.46,-14.76,-32.26,-32.81,-17.69,-34.72,-28.23,-16.13,-32.27,-27.7,-23.43,-35.97,-28.29,-23.62,-39.33,-25.88,-29.61,-36.87,-23.33,-21.47,-39.58,-23.37,-30.78,-42.17,-17.65,-31.26,-42.59,-26.63,-30.54,-35.8,-24.15,-35.16,-29,-23.34,-37.42,-27.26,-15.84,-34.81,-32.07,-30.06,-42.27,-35.78,-29.78,-48.64,-22.34,-20.52,-34.83,-31.25,-37.83,-38.64,-21.44,-36.76,-41.41,-35.21,-38.82,-42.46,-23.9,-34.62,-50.37,-33.49,-43.68,-46.94,-33.24,-43.47,-50.88,-39.56,-53.43,-50.91,-27.84,-50.4,-49.2,-35.84,-58.83,-36.09,-33.33,-62.07,-37.45,-32.46,-50.32,-43.9,-50.64,-56.72,-42.36,-42.83,-59.86,-34.59,-45.33,-50.95,-32.83,-46.59,-61.75,-45.47,-48.13,-50.3,-28.85,-51.76,-44.22,-36.63,-49.35,-48.51,-35.06,-48.75,-45.2,-36.26,-46.89,-37.87,-43.89,-57,-32.14,-37.61,-54.55,-26.66,-38.41,-54.36,-37.17,-44.73,-45.67,-23.28,-34.4,-40.29,-20.87,-46.08,-35.54,-22.94,-40.03,-39.45,-30.37,-33.64,-31.66,-24.42,-35.21,-25.67,-20.67,-39.1,-28.04,-25.26,-30.59,-26.37,-28.19,-30.55,-19.94,-24.48,-29.57,-14.99,-26.69,-33.7,-21.17,-21.59,-32.23,-18.49,-30.25,-26.25,-20.3,-32.54,-29.27,-13.13,-29.16,-23.62,-12.29,-30.77,-18.67,-14.51,-35.45,-19.29,-14.25,-30.82,-17.98,-18.83,-34,-18.17,-22.1,-31.05,-14.34,-17.38,-27.12,-15.76,-20.1,-30.72,-13.45,-24.59,-22.82,-8.76,-20.83,-24.48</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B170" t="str">
+        <v>[L_09_标记]</v>
+      </c>
+      <c r="C170" t="str">
+        <v>a: 29.7ms -80.8uv b: 61.9ms 249.8uv</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B171" t="str">
+        <v>[R_10_名字]</v>
+      </c>
+      <c r="C171" t="str">
+        <v>FERG(10)_dOps</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B172" t="str">
+        <v>[R_10_放大器]</v>
+      </c>
+      <c r="C172" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B173" t="str">
+        <v>[R_10_闪光]</v>
+      </c>
+      <c r="C173" t="str">
+        <v>b白色光:20.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B174" t="str">
+        <v>[R_10_闪光背景]</v>
+      </c>
+      <c r="C174" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B175" t="str">
+        <v>[R_10_采样]</v>
+      </c>
+      <c r="C175" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B176" t="str">
+        <v>[R_10_分析时间]</v>
+      </c>
+      <c r="C176" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B177" t="str">
+        <v>[R_10_数据长度]</v>
+      </c>
+      <c r="C177" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B178" t="str">
+        <v>[R_10_详细数据(uv)]</v>
+      </c>
+      <c r="C178" t="str">
+        <v>23.63,6.92,16.34,15.38,6.88,21.97,2.09,20.37,5.61,11.36,13.56,1.64,18.23,-2.13,15.34,2.9,6.11,11.94,-2.52,16.44,-2.82,13.21,5.1,4.88,14.66,-0.89,18.65,-0.11,13.81,8.2,4.02,16.25,-2.4,16.38,-1.71,7.82,4.92,-3.83,10.56,-9.48,9.51,-4.8,1.77,4.68,-5.98,12.31,-5.88,14.06,3.7,10.17,16.83,6.06,26.16,7.89,23.33,15.39,16.36,22.73,6.66,24.06,3.97,15.69,6.84,1.45,9.85,-6.67,9.27,-6.98,4.62,1.93,-3.31,13.77,-1.89,20.24,8.45,21.13,25.05,17.84,39.58,18.15,37.94,28.31,27.81,33.26,17.46,31.65,8.02,19.49,4.14,-0.68,5.55,-15.56,0.65,-21.99,-5.89,-10.91,-13.67,1.83,-11.15,13.18,0.87,19.35,21.85,20.58,35.34,17.53,44.27,22.37,38.74,31.47,20.33,30.55,3.64,14.91,-4.67,-7.98,-7.06,-24.22,-12.17,-34.63,-20.92,-28.46,-23.04,-12.88,-21.85,5.37,-6.85,15.03,14.19,22.38,36.98,22.36,39.79,26.36,40.37,33.5,25.19,33.19,5.98,19.46,-4.11,0.87,-8.35,-18.11,-3.31,-28,-8.88,-20.05,-14.78,-8.36,-13.96,12.57,-2.84,21.85,17.7,26.56,36.22,24.1,45.8,23.29,39.13,31.62,27.14,34.03,12.03,26.77,2.74,12.67,-0.47,-8.16,2.83,-15.74,2.17,-12.7,-2.01,-3.22,-5.22,13.5,-2.66,21.08,9.73,19.28,24.86,13.58,31.98,11.52,32.18,18.53,21.26,21.46,4.57,20.72,-2.61,10.22,-2.41,-4.47,2.51,-14.24,3.81,-15.37,1.65,-4.58,-4.61,8.02,-7.68,13.6,-2.01,10.98,8.74,4.91,18.28,0.59,18.32,2.77,11.16,10.28,-0.03,14.95,-5.76,11.7,-2.38,2.19,5.14,-6.09,10.73,-7.6,9.43,-0.43,2.35,11.11,-2.99,17.26,-0.82,14.95,8.49,7.3,18.39,2.1,21.97,3.83,16.24,12.22,6.89,19.88,1.19,20.56,4.15,13.44,12.85,4.28,20.03,1.05,19.66,5.92,12.38,15.41,4.16,21.85,2.26,19.81,8.47,11.19,17.43,3.14,21.72,2.18,17.51,8.81,7.72,16.96,0.15,19.33,0.54,13.35,7.89,3.37,15.58,-2.91,16.46,-0.69,9.34,7.51,-0.33,14.45,-5,13.83,-1.17,5.78,7.52,-3.42,13.45,-6.41,11.31,-1.06,2.6,7.93,-5.68,12.8,-6.78,9.36,0.12,0.41,9.22,-6.55,12.98,-5.64,8.4,2.58,-0.49,11.48,-5.99,13.94,-3.17,8.27,6.01,-0.38,14.31,-4.34,15.27,0.17,8.58,9.89,0.33,17.21,-2.09,16.52,3.85,8.9,13.68,1.19,19.65,0.27,17.21,7.32,8.78,16.81,1.73,21.12,2.22,16.9,10.05,7.83,18.82,1.6,21.26,3.43,15.34,11.74,5.91,19.48,0.68,19.99,3.79,12.57,12.36,3.11,18.86,-0.89,17.47,3.48,8.89,12.1,-0.21,17.27,-2.75,14.13,2.86,4.78,11.39,-3.53,15.17,-4.39,10.54,2.41,0.84,10.7,-6.27,13.12,-5.3,7.25,2.59,-2.35,10.49,-7.94,11.56,-5.08,4.73,3.72,-4.4,11.03,-8.24,10.76,-3.54,3.21,5.89,-5.15,12.37,-7.13,10.74,-0.78,2.68,8.93,-4.71,14.31,-4.84,11.28,2.85,2.86,12.43,-3.43,16.4,-1.84,11.96,6.83,3.32,15.83,-1.81,18.14,1.33,12.28,10.55,3.57,18.55,-0.35,19,4.11,11.81,13.48,3.2,20.13,0.52,18.63,6.09,10.26,15.27,2,20.32,0.63,16.89,7.12,7.63,15.81,0,19.13,0.02,13.94,7.28,4.15,15.28,-2.53,16.85,-1.02,10.17,6.89,0.28,14.06,-5.1,13.96,-2.02,6.14,6.42,-3.39,12.66,-7.17,11.03,-2.49,2.44,6.33,-6.31,11.56,-8.24,8.55,-2.01,-0.42,6.99,-8.03,11.12,-8,6.88,-0.37,-2.16,8.55,-8.35,11.45,-6.36,6.12,2.39,-2.73,10.91,-7.37,12.43,-3.54,6.09,5.98,-2.36,13.71,-5.4,13.69,0.02,6.44</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B179" t="str">
+        <v>[R_10_标记]</v>
+      </c>
+      <c r="C179" t="str">
+        <v>62.1uv</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B180" t="str">
+        <v>[L_10_名字]</v>
+      </c>
+      <c r="C180" t="str">
+        <v>FERG(10)_dOps</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B181" t="str">
+        <v>[L_10_放大器]</v>
+      </c>
+      <c r="C181" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B182" t="str">
+        <v>[L_10_闪光]</v>
+      </c>
+      <c r="C182" t="str">
+        <v>b白色光:20.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B183" t="str">
+        <v>[L_10_闪光背景]</v>
+      </c>
+      <c r="C183" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B184" t="str">
+        <v>[L_10_采样]</v>
+      </c>
+      <c r="C184" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B185" t="str">
+        <v>[L_10_分析时间]</v>
+      </c>
+      <c r="C185" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B186" t="str">
+        <v>[L_10_数据长度]</v>
+      </c>
+      <c r="C186" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B187" t="str">
+        <v>[L_10_详细数据(uv)]</v>
+      </c>
+      <c r="C187" t="str">
+        <v>-14.33,-19.75,-5.16,-24.09,-8.05,-15.94,-19.55,-6.37,-25.16,-8.32,-18.09,-19.94,-8.35,-26.85,-9.43,-20.97,-20.91,-10.94,-28.88,-10.85,-23.77,-21.85,-13.32,-30.15,-11.7,-25.71,-21.47,-14.49,-30.08,-11.14,-26.44,-19.84,-14.79,-29.61,-10.78,-27.21,-19.14,-16.52,-30.02,-12.05,-29.73,-20.49,-19.55,-32.32,-14.42,-32.17,-21.83,-21.41,-32.31,-13.51,-31.33,-17.7,-19.04,-26.15,-8.26,-25.17,-9.27,-13.71,-19.42,-3.13,-20.77,-5.82,-10.84,-17.94,-3.48,-24.19,-9.25,-19.26,-23.66,-12.25,-33,-15.68,-27.73,-27.61,-16.88,-31.48,-12.76,-21.21,-18.22,-4.75,-18.36,2.28,-8.18,0.12,9.52,-8.04,14.4,-3.14,0.96,5.29,-13.11,0.79,-19.38,-17.33,-18.32,-36.11,-20.2,-39.15,-36.6,-33.53,-41.92,-22.27,-41.07,-22.96,-19.73,-25.35,-1.34,-16.3,-0.26,3.49,0.16,16.75,-0.07,10.4,3.92,-4.37,5.41,-19.22,-12.74,-24.12,-36.31,-29.1,-52.78,-45.35,-47.14,-52.32,-40.46,-52.4,-37.35,-39,-33.16,-14.18,-25.97,-1.81,-7.47,-0.83,15.36,0.85,17.99,9.22,0.62,9.1,-14.72,2.14,-19.09,-21.87,-18.42,-42.28,-29.91,-46.74,-38.26,-31.14,-50.61,-30.33,-39.3,-26.64,-18.08,-26,-1.38,-13.31,0.29,4.85,-4.17,14.94,3.4,8.69,10.13,-4.28,12.5,-12.53,-3.5,-9.71,-22.48,-10.61,-29.72,-18.02,-26.44,-33.16,-14.35,-32.17,-17.29,-19.95,-24.09,-6.04,-21.87,-3.79,-7.77,-9.95,3.61,-14.51,1.82,-6.64,-11.07,0.9,-19.82,-4.74,-17.11,-19.25,-10.41,-29.32,-12.95,-26.59,-26.22,-15.48,-32.86,-14.07,-28.16,-22.88,-14.53,-29.78,-9.98,-24.04,-17.6,-11.06,-25.85,-6.53,-22.43,-15.71,-11.56,-25.42,-7.77,-25.02,-16,-14.52,-27.12,-9.15,-26.62,-16.12,-16.06,-26.55,-8.5,-26.05,-13.43,-14.87,-23.35,-5.9,-24.02,-9.74,-13.13,-20.04,-3.58,-22.17,-6.74,-12.21,-17.56,-2.46,-21.12,-4.85,-12.27,-15.78,-2.1,-20.55,-3.41,-12.62,-14.18,-1.95,-19.98,-2.15,-13.01,-12.69,-2.06,-19.64,-1.31,-13.79,-11.67,-2.82,-19.73,-1.17,-15.19,-11.25,-4.3,-20.35,-1.74,-17.09,-11.39,-6.34,-21.31,-2.79,-19.27,-11.79,-8.67,-22.36,-4.09,-21.48,-12.28,-11.07,-23.31,-5.46,-23.55,-12.68,-13.38,-24.01,-6.73,-25.3,-12.86,-15.43,-24.31,-7.76,-26.58,-12.68,-17.06,-24.07,-8.41,-27.27,-12.03,-18.17,-23.23,-8.6,-27.29,-10.88,-18.72,-21.77,-8.35,-26.68,-9.29,-18.74,-19.78,-7.73,-25.53,-7.35,-18.36,-17.38,-6.86,-23.97,-5.24,-17.7,-14.77,-5.92,-22.18,-3.13,-16.96,-12.13,-5.08,-20.36,-1.23,-16.31,-9.68,-4.53,-18.71,0.27,-15.93,-7.58,-4.43,-17.37,1.23,-15.94,-5.99,-4.87,-16.46,1.56,-16.41,-4.97,-5.91,-16.01,1.23,-17.34,-4.53,-7.51,-16.01,0.28,-18.67,-4.61,-9.57,-16.36,-1.16,-20.28,-5.08,-11.94,-16.92,-2.95,-21.99,-5.79,-14.44,-17.52,-4.89,-23.62,-6.54,-16.86,-17.97,-6.77,-24.95,-7.15,-19,-18.09,-8.43,-25.83,-7.48,-20.7,-17.76,-9.7,-26.13,-7.39,-21.83,-16.88,-10.51,-25.78,-6.86,-22.36,-15.45,-10.83,-24.79,-5.88,-22.29,-13.51,-10.71,-23.22,-4.56,-21.72,-11.18,-10.26,-21.21,-3.02,-20.78,-8.64,-9.62,-18.94,-1.45,-19.65,-6.06,-8.99,-16.61,-0.03,-18.53,-3.67,-8.54,-14.42,1.03,-17.58,-1.65,-8.44,-12.53,1.6,-16.97,-0.15,-8.81,-11.09,1.56,-16.77,0.75,-9.7,-10.15,0.87,-17.02,1.01,-11.1,-9.72,-0.42,-17.68,0.68,-12.95,-9.73,-2.24,-18.66,-0.12,-15.11,-10.04,-4.41,-19.78,-1.25,-17.39,-10.51,-6.76,-20.88,-2.51,-19.6,-10.94,-9.07,-21.77,-3.71,-21.54,-11.15,-11.16,-22.25,-4.68,-23.03,-11,-12.85,-22.21,-5.29,-23.94,-10.38,-14.05,-21.56,-5.46,-24.21,-9.27,-14.71,-20.29,-5.19,-23.83,-7.68,-14.85,-18.45,-4.52,-22.89,-5.71,-14.56,-16.17,-3.59,-21.52</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B188" t="str">
+        <v>[L_10_标记]</v>
+      </c>
+      <c r="C188" t="str">
+        <v>61.8uv</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B189" t="str">
+        <v>[R_11_名字]</v>
+      </c>
+      <c r="C189" t="str">
+        <v>FERG(11)_dMax</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B190" t="str">
+        <v>[R_11_放大器]</v>
+      </c>
+      <c r="C190" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B191" t="str">
+        <v>[R_11_闪光]</v>
+      </c>
+      <c r="C191" t="str">
+        <v>b白色光:200.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B192" t="str">
+        <v>[R_11_闪光背景]</v>
+      </c>
+      <c r="C192" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B193" t="str">
+        <v>[R_11_采样]</v>
+      </c>
+      <c r="C193" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B194" t="str">
+        <v>[R_11_分析时间]</v>
+      </c>
+      <c r="C194" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B195" t="str">
+        <v>[R_11_数据长度]</v>
+      </c>
+      <c r="C195" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B196" t="str">
+        <v>[R_11_详细数据(uv)]</v>
+      </c>
+      <c r="C196" t="str">
+        <v>-10.83,-8.96,-12.07,-8.22,-13.22,-7.56,-14.24,-7.01,-15.07,-6.6,-15.7,-6.35,-16.09,-6.27,-16.22,-6.36,-16.1,-6.62,-15.72,-7.05,-15.11,-7.61,-14.28,-8.28,-13.27,-9.03,-12.12,-9.82,-10.87,-10.61,-9.57,-11.35,-8.27,-12.02,-7.03,-12.58,-5.88,-12.98,-4.88,-13.22,-4.07,-13.3,-3.46,-13.11,-3.13,-12.8,-2.94,-12.46,-3.24,-11.81,-3.63,-10.96,-4.54,-10.59,-5.65,-9.89,-7.02,-8.83,-7.99,-9.04,-9.34,-8.31,-11.36,-9.44,-15.18,-10.36,-17.76,-11.21,-19.2,-10.34,-22.66,-14.65,-23.38,-19.58,-31.41,-18.38,-31.64,-26.64,-31.87,-25.75,-33.23,-36.21,-43.93,-33.04,-42.21,-42.5,-43.64,-50.77,-49.18,-48.73,-50.6,-44.6,-45.31,-52.91,-52.48,-61.98,-36.38,-46.23,-41.63,-44.14,-36.75,-54.43,-33.86,-43.53,-22.59,-31.92,-13.64,-19.92,-13.28,-13.64,-13.47,4.94,-3.81,-2,20.63,32.18,25.06,38.3,55.32,64.98,74.07,60.96,63.23,94.41,107.23,109.93,125.22,125.62,118.72,166.56,152.09,174.02,159.57,197.09,200.04,193.29,183.81,233.61,244.14,263.82,235.58,246.18,270.58,283.41,293.85,305.29,252.98,315.44,306.09,332.76,277.3,275.74,308.32,314.38,306.71,346.43,313.5,361.6,311.3,373.29,330.26,349.64,312.43,355.9,376.37,300.13,353.14,326.03,327.87,359.62,372.97,327.24,346.62,286.76,292.33,314.01,338.23,305.32,314.66,303.28,271.95,301.35,270.61,282.13,247.03,280.42,261.66,269.35,249.35,234.46,225.97,241.96,236.1,204.43,224.31,208.12,191.02,223.42,185.75,205.87,169.13,184.11,159.83,186.78,176.24,163.13,144.7,161.53,144.06,140.96,143.42,141.21,131.25,134.71,129.31,124.7,138.11,115.11,121.04,95.16,109.36,89.99,112.45,100.25,83.17,81.1,104.73,97.1,94.49,83.01,83,64.89,78.51,59.1,88.84,61.74,76.75,52.81,53.72,66.71,64.89,46.66,43.42,60.87,54.02,53.35,54.74,59.27,30.99,37.91,37.21,34.19,23.31,41.09,27.53,32.66,24.8,25.51,17.57,30.95,13.21,25.92,19.75,21.6,13.17,16.08,13.94,14.94,13.48,9.35,11.13,5.3,10.85,2.31,9.92,3.42,4.28,-3.75,5.84,-7.27,4.7,-7.61,3.98,-7.72,0.61,-8.88,-1.95,-7.87,1.25,-8.94,-2.38,-10.41,-6.01,-9.94,-4.04,-13.73,-5.88,-10,-8.35,-9.32,-9.53,-7.5,-11.34,-11.52,-10.57,-7.16,-11.92,-6.2,-14.06,-9.46,-14.57,-9.44,-16.28,-10.18,-18.09,-7.37,-19.06,-9.01,-16.65,-11.5,-16.15,-6.78,-17.46,-7.53,-19.93,-9.83,-18.34,-10.87,-21.01,-18.2,-12.8,-13.36,-18.74,-20.54,-20.74,-26.3,-10.5,-25.51,-12.69,-26.28,-12.12,-29.12,-11.52,-31.54,-19.84,-32.97,-24.77,-30.07,-18.48,-35.34,-18.16,-25.11,-22.63,-34.26,-22.06,-24.31,-19.79,-29.58,-25.65,-36.05,-23.66,-27.46,-39.66,-34.47,-30.44,-32.87,-30.26,-30.77,-43.36,-26.31,-43.44,-26.32,-43.37,-26.21,-37.85,-21.91,-40.24,-31.94,-44.44,-40.48,-34.76,-24.23,-44.67,-26.95,-34.81,-42.82,-47.19,-32.22,-38.02,-36.31,-41.5,-36.29,-30.38,-39.15,-37.17,-35.36,-37.66,-46.94,-29.2,-29.44,-38.85,-41.58,-25.31,-29.91,-26.93,-35.16,-22.49,-43.3,-30.17,-41.17,-32.45,-29.63,-30.12,-35.06,-36.39,-26.34,-23.59,-25.71,-31.55,-31.81,-23.66,-38.55,-36.06,-22.95,-33.84,-34.15,-32.41,-25.67,-28.3,-23.25,-26.18,-17.8,-37.71,-26.93,-28.36,-28.09,-26.9,-31.34,-28.48,-19.49,-34.48,-24.39,-24.81,-25.81,-33.93,-31.34,-33.28,-30.44,-30.43,-28.02,-18.54,-25.48,-29.28,-31.24,-16.89,-31.9,-25.67,-32.21,-13.37,-23.67,-23.9,-22.2,-21.33,-29.48,-13.07,-20.94,-10.37,-28.41,-12.56,-27.81,-17.86,-17,-9.63,-24.04,-11.5,-13.06,-13.29,-13.32,-13.52,-15.04,-17.22,-9.15,-8.39,-5.33,-9.27,-4.12,-8.95,-1.77,-8.77,-5.87,-12.4,-5.29,-12.93,-1.73,-7.11,-0.66,-7.48,-1.51,-10.09,-1.29</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B197" t="str">
+        <v>[R_11_标记]</v>
+      </c>
+      <c r="C197" t="str">
+        <v>a: 32.5ms -86.9uv b: 70.9ms 407.5uv</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B198" t="str">
+        <v>[L_11_名字]</v>
+      </c>
+      <c r="C198" t="str">
+        <v>FERG(11)_dMax</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B199" t="str">
+        <v>[L_11_放大器]</v>
+      </c>
+      <c r="C199" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B200" t="str">
+        <v>[L_11_闪光]</v>
+      </c>
+      <c r="C200" t="str">
+        <v>b白色光:200.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B201" t="str">
+        <v>[L_11_闪光背景]</v>
+      </c>
+      <c r="C201" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B202" t="str">
+        <v>[L_11_采样]</v>
+      </c>
+      <c r="C202" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B203" t="str">
+        <v>[L_11_分析时间]</v>
+      </c>
+      <c r="C203" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B204" t="str">
+        <v>[L_11_数据长度]</v>
+      </c>
+      <c r="C204" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B205" t="str">
+        <v>[L_11_详细数据(uv)]</v>
+      </c>
+      <c r="C205" t="str">
+        <v>-13.37,-23.86,-14.49,-22.76,-16.61,-20.85,-19.3,-18.61,-22.03,-16.58,-24.24,-15.27,-25.5,-15.01,-25.55,-15.9,-24.45,-17.79,-22.45,-20.26,-20.03,-22.82,-17.74,-24.91,-16.12,-26.07,-15.5,-26.05,-16.11,-24.81,-17.67,-22.79,-19.94,-20.21,-22.31,-17.81,-24.77,-16.24,-26.12,-15.66,-26.12,-16.01,-25.7,-18.32,-24.07,-20.5,-22.48,-24.78,-20.25,-28.19,-19.25,-29.44,-19.93,-31.52,-24.81,-36.2,-28.59,-32.83,-29.16,-31.65,-38.78,-31.42,-39.3,-36.82,-47.44,-43.52,-52.75,-43.05,-55.71,-51.9,-54.7,-49.22,-48.47,-50.45,-51.52,-56.1,-47.74,-72.04,-55.44,-68.94,-60.04,-69.65,-61.75,-61.12,-61.39,-50.16,-54.9,-44.99,-53.73,-33.4,-51.01,-27.24,-23.13,-24.26,-21.67,-3.37,-18.77,-5.4,-1.51,12.25,22.2,23.43,36.23,48.02,52.14,61,89.28,93.42,91.95,98.72,121.28,121.14,112.69,115.48,133.75,155.35,171.78,193.5,188.94,169.28,177.47,228.6,210.64,241.2,242.83,223.37,242.08,223.06,259.05,270.04,259.38,261.41,312.44,311.2,295.03,292.86,330.28,315.07,279.8,283.48,345.16,332.97,354.24,323.03,315.14,376.28,302.85,375.92,299.1,358.81,367.68,301.65,308.33,332.03,336.26,288.91,340.34,286.58,298.69,289.98,299.26,329.8,267.06,263.56,290.93,267.76,299.74,282,286.67,237.9,262.09,263.11,227.96,230.33,209.86,226.5,235.4,197.91,174.23,206.2,189.96,180.98,191.28,183.33,178.06,163.64,168.96,157.56,136.07,134.12,140.22,134.33,145.44,127.65,126.1,123.08,94.31,134.25,115.48,95.86,106.5,86.11,78.51,89.09,91.66,79.19,77.81,85.15,66.53,82.39,71.58,54.93,68.5,67.66,55.53,43.94,57.22,67.39,59.12,69.64,47.44,54.83,41.35,54.97,48.13,57.86,29.55,52.89,30.47,43.94,42.31,41.62,37.3,34.85,38.72,15.4,29.58,14.93,28.45,15.42,21.32,20.61,20,19.49,18.78,11.96,7.21,12.64,1.72,11.13,-1.87,10.67,-2.33,6.89,-2.83,1.96,-3.75,-1.76,-6.27,-7.13,-3.54,-11.65,-3.98,-14.48,-2.27,-14.13,-7.04,-14.96,-11.21,-14.38,-15.15,-14.08,-17.54,-13.95,-21.24,-12.09,-22.49,-15.18,-26.95,-17.26,-24.48,-16.74,-22.45,-22.25,-21.76,-26.11,-18.36,-26.57,-17.89,-29.69,-20.29,-30.57,-23.3,-27.27,-25.75,-25.68,-25.59,-26.83,-25.72,-26.67,-30.38,-22.97,-32.17,-24.37,-32.2,-24.6,-30.4,-25.58,-32.09,-24.47,-31.89,-29.5,-32.27,-33.62,-24.11,-31.63,-24.13,-35.71,-24.75,-40.12,-21.97,-31.67,-32.62,-31.2,-36.61,-28.33,-40.54,-27.05,-33.12,-34.42,-42.19,-35.09,-33.97,-23.85,-31.89,-37.84,-30.17,-40.85,-30.23,-46.94,-34.83,-37.08,-32.89,-40.89,-39.05,-41.74,-27.14,-41.99,-42.05,-40.6,-38.06,-43.65,-43.04,-32.53,-45.61,-36.24,-41.37,-36.95,-55.09,-41.74,-57.64,-35.25,-55.82,-47.09,-52.45,-41.88,-38.77,-43.73,-36.36,-60.5,-42.04,-50.89,-35.29,-44.31,-46.25,-50.61,-54.96,-50.46,-48.65,-51.12,-43.83,-38.58,-56.89,-49.11,-61.65,-51.16,-59.28,-48.22,-49.96,-43.35,-50,-48.03,-45.9,-43.02,-32.75,-53.6,-50.34,-45.46,-35.95,-42.57,-48.3,-37.52,-46.29,-40.68,-50.38,-38.36,-46.1,-44.48,-39.75,-44.32,-40.02,-40.9,-47.06,-30.14,-48.5,-33.33,-33.94,-46.18,-40.62,-44.58,-28.87,-49.55,-31.28,-45.85,-32.67,-33.38,-32.43,-41.63,-37.77,-29.7,-28.48,-31.55,-30.46,-31.05,-38.18,-21.38,-36.07,-33.09,-32.53,-35.24,-28.57,-26.18,-35.27,-29.46,-30.43,-29.45,-31.8,-35.68,-19.62,-29.78,-25.84,-38.66,-20.96,-32.64,-23.64,-26.74,-28.34,-25.52,-32.04,-24.9,-35.36,-23.82,-30.13,-25.03,-31.41,-18.37,-29.3,-22.26,-26.93,-25.68,-22.18,-28.53,-16.46,-25.72,-17.37,-25.48,-14.84,-27.79,-14.87,-19.61,-13.85,-20.1,-20.24,-14.83,-20.57,-13.75,-19.85,-10.41,-21.68,-8.76,-18.97,-11.23,-15.07,-8.86,-14.52,-11.22,-9.49,-14.67,-9.21,-16.81</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B206" t="str">
+        <v>[L_11_标记]</v>
+      </c>
+      <c r="C206" t="str">
+        <v>a: 32.6ms -90.5uv b: 71.0ms 370.0uv</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B207" t="str">
+        <v>[R_12_名字]</v>
+      </c>
+      <c r="C207" t="str">
+        <v>FERG(12)_dOps</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B208" t="str">
+        <v>[R_12_放大器]</v>
+      </c>
+      <c r="C208" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B209" t="str">
+        <v>[R_12_闪光]</v>
+      </c>
+      <c r="C209" t="str">
+        <v>b白色光:200.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B210" t="str">
+        <v>[R_12_闪光背景]</v>
+      </c>
+      <c r="C210" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B211" t="str">
+        <v>[R_12_采样]</v>
+      </c>
+      <c r="C211" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B212" t="str">
+        <v>[R_12_分析时间]</v>
+      </c>
+      <c r="C212" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B213" t="str">
+        <v>[R_12_数据长度]</v>
+      </c>
+      <c r="C213" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B214" t="str">
+        <v>[R_12_详细数据(uv)]</v>
+      </c>
+      <c r="C214" t="str">
+        <v>-13.22,-0.46,-15.15,0.3,-14.68,-0.88,-11.97,-3.92,-8.33,-7.75,-4.13,-11.55,-1.03,-14.38,0.3,-15.28,-0.53,-14.15,-3.39,-11.08,-7.59,-6.76,-11.1,-2.67,-13.38,0.72,-13.95,2.26,-11.65,2.17,-7.65,0.31,-2.3,-2.5,2.63,-5.03,6.49,-7.77,6.68,-9.15,4.53,-8.86,0.2,-7.03,-6.33,-5.43,-10.59,-2.48,-15.35,0.16,-15.28,1.9,-12.09,1.72,-5.98,1.31,1.36,-0.5,7.16,-2.16,11.69,-3.96,12.27,-3.33,7.72,-6.05,0.68,-7.29,-8.68,-9.43,-17.14,-11.92,-25.56,-13.66,-27.48,-10.65,-23.29,-11.27,-17.59,-10.3,-7.95,-8.45,2.17,-5.17,8.37,-3.24,13.48,0.81,11.44,-1.75,5.74,-4.4,-7.85,-7.36,-20.63,-13.57,-29.52,-18.86,-35.47,-25.15,-36.19,-29.23,-33.4,-24.39,-21.44,-19.58,-6.25,-11.58,8.08,-4.09,14.5,8.62,20.57,10.32,16.29,11.42,10.69,9.37,-4.43,1.05,-18.04,-10.6,-27.37,-16.12,-34.49,-24.83,-33.44,-28.19,-27.97,-26.3,-16.69,-20.79,-1.07,-10.03,11.7,0.94,18.01,17.26,21.02,19.19,13.3,23.78,4.92,16.64,-4.25,5.38,-16.01,-7.89,-24.73,-18.18,-28.77,-29.86,-30.48,-37.9,-19.97,-30.83,-15.16,-25.68,-5.4,-14.41,1.27,0,4.11,9.2,3.63,16.11,2.67,11.39,-5.56,8.4,-12.08,-2.38,-17.71,-15.89,-22.86,-27.33,-21.66,-32.58,-22.25,-35.25,-19.25,-33.24,-15.26,-26.97,-13.2,-16.32,-11.05,-5.48,-9.72,2.49,-9.92,4.39,-10.15,6.4,-10.73,-0.85,-11.74,-8.18,-12.09,-16.53,-11.62,-24.03,-11.39,-25.61,-11.54,-24.95,-12.43,-22.03,-12.19,-15.02,-12.57,-7.92,-13.27,-1.06,-12.8,3.02,-11.49,3.44,-9.86,1.33,-7.66,-4.55,-5.53,-10.25,-3.54,-15.28,-2.72,-18.04,-3.49,-18.19,-5.3,-16.56,-8.59,-12.69,-12.37,-7.67,-15.43,-3.86,-17.24,-1.9,-17.1,-2.53,-15.38,-5.71,-12.66,-10.09,-9.18,-14.96,-6.72,-19.13,-5.69,-21.42,-6.62,-21.55,-9.49,-19.34,-13.64,-15.97,-18.11,-12.43,-21.74,-9.73,-23.96,-8.72,-24.02,-9.86,-21.96,-12.88,-18.51,-17,-14.59,-20.94,-11.2,-23.87,-9.43,-24.83,-9.67,-23.56,-11.87,-20.43,-15.42,-16.23,-19.22,-12.1,-22.29,-9.12,-23.62,-8,-22.8,-8.99,-19.95,-11.7,-15.75,-15.28,-11.26,-18.62,-7.59,-20.72,-5.62,-20.85,-5.83,-18.9,-8.04,-15.32,-11.56,-11,-15.35,-7.07,-18.29,-4.56,-19.55,-4.12,-18.73,-5.85,-16.05,-9.26,-12.25,-13.44,-8.4,-17.24,-5.58,-19.68,-4.64,-20.14,-5.9,-18.58,-9.11,-15.51,-13.47,-11.9,-17.92,-8.86,-21.33,-7.36,-22.92,-7.94,-22.38,-10.6,-20.01,-14.74,-16.61,-19.37,-13.25,-23.37,-11.01,-25.75,-10.64,-26.01,-12.36,-24.19,-15.82,-20.9,-20.17,-17.15,-24.3,-14.05,-27.14,-12.51,-27.98,-13.02,-26.61,-15.46,-23.44,-19.17,-19.34,-23.12,-15.43,-26.21,-12.76,-27.54,-12,-26.69,-13.32,-23.83,-16.27,-19.67,-19.95,-15.25,-23.26,-11.7,-25.18,-9.9,-25.08,-10.23,-22.87,-12.49,-19.07,-15.96,-14.61,-19.58,-10.63,-22.26,-8.12,-23.18,-7.72,-22.01,-9.45,-19.01,-12.79,-14.97,-16.79,-10.97,-20.31,-8.1,-22.4,-7.16,-22.48,-8.43,-20.58,-11.6,-17.25,-15.86,-13.5,-20.11,-10.43,-23.28,-8.99,-24.59,-9.69,-23.8,-12.46,-21.26,-16.67,-17.8,-21.29,-14.53,-25.21,-12.47,-27.48,-12.36,-27.63,-14.35,-25.75,-18.05,-22.51,-22.57,-18.92,-26.79,-16.09,-29.65,-14.91,-30.48,-15.79,-29.12,-18.58,-26.02,-22.55,-22.09,-26.67,-18.45,-29.82,-16.11,-31.15,-15.72,-30.27,-17.36,-27.41,-20.56,-23.3,-24.37,-19.03,-27.68,-15.69,-29.51,-14.12,-29.26,-14.67,-26.9,-17.08,-22.98,-20.58,-18.48,-24.1,-14.52,-26.57,-12.09,-27.2,-11.76,-25.72,-13.53,-22.44,-16.81,-18.19,-20.64,-14.07,-23.89,-11.15,-25.62,-10.21,-25.32,-11.47,-23.05,-14.58,-19.46,-18.69,-15.53,-22.71,-12.4,-25.57,-10.98</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B215" t="str">
+        <v>[R_12_标记]</v>
+      </c>
+      <c r="C215" t="str">
+        <v>63.1uv</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B216" t="str">
+        <v>[L_12_名字]</v>
+      </c>
+      <c r="C216" t="str">
+        <v>FERG(12)_dOps</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B217" t="str">
+        <v>[L_12_放大器]</v>
+      </c>
+      <c r="C217" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B218" t="str">
+        <v>[L_12_闪光]</v>
+      </c>
+      <c r="C218" t="str">
+        <v>b白色光:200.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B219" t="str">
+        <v>[L_12_闪光背景]</v>
+      </c>
+      <c r="C219" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B220" t="str">
+        <v>[L_12_采样]</v>
+      </c>
+      <c r="C220" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B221" t="str">
+        <v>[L_12_分析时间]</v>
+      </c>
+      <c r="C221" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B222" t="str">
+        <v>[L_12_数据长度]</v>
+      </c>
+      <c r="C222" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B223" t="str">
+        <v>[L_12_详细数据(uv)]</v>
+      </c>
+      <c r="C223" t="str">
+        <v>-33.64,-20.81,-32.32,-22.51,-30.63,-24.58,-28.87,-27.1,-27.03,-29.87,-25.52,-32.43,-24.14,-34.49,-22.62,-36.08,-21.44,-36.99,-20.8,-36.62,-19.41,-35.22,-18.67,-32.95,-17.97,-29.98,-17.79,-26.21,-18.88,-23.76,-19.5,-20.76,-22.46,-19.24,-24.82,-18.25,-28.09,-17.71,-31.03,-17.36,-32.87,-18.25,-34.95,-17.87,-32.83,-15.76,-30.9,-14.72,-26.52,-12.46,-21.73,-10.86,-15.44,-9.15,-12.11,-11.15,-8.08,-13.69,-9.18,-17.93,-10.01,-23.78,-13.38,-29.73,-17.15,-36.74,-21.71,-37.99,-25.27,-40.03,-25.28,-37.25,-21.43,-32.48,-18.09,-23.94,-14.82,-15.98,-9.17,-5.97,-10.48,-2.97,-11.61,-3.08,-16.35,-6.49,-22.56,-12.33,-32.49,-20.73,-42.16,-29.33,-47.67,-32.59,-51.27,-34.34,-48.42,-39.19,-41.76,-31.34,-31.86,-22.39,-18.86,-14.99,-6.77,-9.25,-0.34,-2.76,9.67,-10.22,4.91,-14.98,-4.71,-24.85,-13.19,-34.53,-23.04,-44.41,-31.38,-52.16,-42.53,-52.04,-39.03,-41.66,-31.8,-32.9,-25.2,-17.87,-14.37,-1.6,-4.23,9.71,-1.14,19.96,6.53,17.91,-5.86,11.65,-10.06,0.53,-21.67,-11.96,-30.56,-21.09,-41.98,-33.02,-40.47,-34.52,-39.59,-31.33,-29.77,-28.17,-20.38,-21.36,-8.79,-12.14,3.88,-8.59,8.58,-4.68,10.17,-4.04,8.41,-9.12,2.11,-18.8,-8.35,-26.72,-18.96,-34.26,-26.05,-34.15,-31.47,-36.71,-37.17,-32.63,-33.05,-25.44,-30.2,-17.26,-25.93,-8.77,-21.83,-2.81,-17.12,1.48,-14.8,-1.66,-17.95,-5.69,-20.58,-9.55,-23.5,-16.16,-26.42,-22.59,-28.41,-26.64,-26.07,-30.17,-24.64,-28.8,-20.67,-28.82,-14.53,-25.85,-9.51,-23.16,-5.46,-20.23,-2.52,-17.8,-1.9,-17.74,-2.7,-16.03,-5.38,-15.75,-9.25,-15.45,-12.85,-14.63,-16.07,-13.15,-18.81,-10.98,-19.77,-9.13,-20.42,-6.44,-20.72,-4.23,-19.82,-2.71,-18.79,-2.37,-17.62,-2.59,-16.25,-4.01,-15.02,-6.46,-14.04,-9.57,-12.73,-12.64,-11.5,-15.77,-10.33,-18.47,-8.99,-20.52,-8.01,-22.38,-7.13,-23.21,-6.95,-23.56,-7.14,-23.26,-7.93,-22.51,-9.38,-21.3,-11.32,-19.76,-13.55,-18.01,-16.05,-16.21,-18.56,-14.35,-20.85,-12.56,-22.79,-10.97,-24.23,-9.73,-25.06,-8.86,-25.18,-8.49,-24.7,-8.59,-23.53,-9.16,-21.81,-10.16,-19.64,-11.51,-17.13,-13.07,-14.43,-14.71,-11.68,-16.28,-9.06,-17.62,-6.71,-18.61,-4.74,-19.15,-3.27,-19.17,-2.38,-18.63,-2.08,-17.56,-2.38,-15.99,-3.23,-14.02,-4.56,-11.75,-6.24,-9.33,-8.14,-6.9,-10.11,-4.63,-12.01,-2.66,-13.7,-1.13,-15.04,-0.12,-15.95,0.27,-16.37,0.03,-16.27,-0.85,-15.67,-2.31,-14.63,-4.26,-13.24,-6.58,-11.6,-9.14,-9.85,-11.77,-8.14,-14.31,-6.6,-16.6,-5.36,-18.51,-4.52,-19.91,-4.17,-20.74,-4.35,-20.95,-5.05,-20.54,-6.25,-19.54,-7.86,-18.05,-9.79,-16.16,-11.91,-14.02,-14.06,-11.76,-16.1,-9.54,-17.87,-7.52,-19.24,-5.8,-20.11,-4.51,-20.38,-3.7,-20.03,-3.42,-19.06,-3.66,-17.5,-4.36,-15.43,-5.47,-12.98,-6.86,-10.27,-8.41,-7.47,-9.98,-4.74,-11.43,-2.23,-12.62,-0.1,-13.45,1.54,-13.82,2.61,-13.69,3.05,-13.04,2.85,-11.9,2.05,-10.32,0.72,-8.41,-1.04,-6.28,-3.09,-4.08,-5.29,-1.96,-7.49,-0.06,-9.52,1.47,-11.26,2.53,-12.6,3.03,-13.45,2.92,-13.77,2.19,-13.56,0.87,-12.84,-0.95,-11.68,-3.18,-10.2,-5.68,-8.5,-8.29,-6.74,-10.86,-5.04,-13.22,-3.55,-15.23,-2.4,-16.76,-1.66,-17.71,-1.4,-18.04,-1.66,-17.72,-2.41,-16.78,-3.61,-15.29,-5.16,-13.33,-6.97,-11.05,-8.88,-8.59,-10.76,-6.11,-12.45,-3.75,-13.82,-1.67,-14.74,0.02,-15.14,1.23,-14.95,1.9,-14.16,2.01,-12.79,1.6,-10.9,0.71,-8.6,-0.56,-6.01,-2.08,-3.28,-3.72,-0.58,-5.34,1.94,-6.8,4.13,-7.97,5.86,-8.76,7.02,-9.07,7.55,-8.89,7.44,-8.21,6.69,-7.07</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B224" t="str">
+        <v>[L_12_标记]</v>
+      </c>
+      <c r="C224" t="str">
+        <v>58.4uv</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B225" t="str">
+        <v>[R_13_名字]</v>
+      </c>
+      <c r="C225" t="str">
+        <v>FERG(13)_dMax</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B226" t="str">
+        <v>[R_13_放大器]</v>
+      </c>
+      <c r="C226" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B227" t="str">
+        <v>[R_13_闪光]</v>
+      </c>
+      <c r="C227" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B228" t="str">
+        <v>[R_13_闪光背景]</v>
+      </c>
+      <c r="C228" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B229" t="str">
+        <v>[R_13_采样]</v>
+      </c>
+      <c r="C229" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B230" t="str">
+        <v>[R_13_分析时间]</v>
+      </c>
+      <c r="C230" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B231" t="str">
+        <v>[R_13_数据长度]</v>
+      </c>
+      <c r="C231" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B232" t="str">
+        <v>[R_13_详细数据(uv)]</v>
+      </c>
+      <c r="C232" t="str">
+        <v>1.48,10.16,1.01,7.54,6.69,2.07,10.92,1.88,8.19,7.7,2.82,11.82,2.88,8.93,8.8,3.63,12.75,3.9,9.68,9.88,4.42,13.62,4.86,10.33,10.84,5.08,14.34,5.66,10.81,11.61,5.54,14.84,6.24,11.03,12.12,5.74,15.05,6.53,10.98,12.35,5.65,14.96,6.53,10.62,12.26,5.27,14.54,6.19,9.92,11.79,4.49,13.81,5.49,8.84,10.9,3.35,12.36,4.48,7.04,9.5,1.71,10.31,2.21,4.67,7.3,-0.85,6.95,-0.48,1.31,2.47,-6.56,1.78,-6.82,-5.52,-3.31,-12.39,-4.82,-14.08,-11.22,-12.68,-25.19,-17.69,-19.99,-23.96,-24.96,-30.93,-22.91,-29.81,-38.94,-30.57,-46.16,-32.03,-45.75,-46.29,-34.46,-46.97,-31.65,-36.94,-44.12,-34.54,-48,-41.53,-37.87,-31.91,-21.85,-28.62,-14.75,-17.79,-15.99,-11.3,-7.27,7.55,4.67,18.93,14.36,19.95,31.94,43.62,38.97,53.95,54.28,67.69,83,84.11,98.58,106.46,127.45,105.9,129.89,122.26,151.99,153.71,152.6,151.14,174.95,161.3,192.3,211.45,200.45,245.25,240.71,228.7,229.93,263.05,268.02,260.69,260.59,243.62,279.33,294.96,282.87,293.68,317.75,298.24,313.34,331.68,303.78,346.11,292.3,313.05,339.86,340.54,329.3,296.58,357.74,296.86,306.68,312.28,298.31,295.74,282.1,286.15,325.42,306.91,295.01,281.81,276.22,273.33,308.8,303.4,272.64,248.14,269.42,224.28,243.76,258.51,232.69,245.78,221.28,242.07,195.92,194.62,203.94,188.63,204.74,195.88,169.6,164.86,167.25,175.49,156.48,146.19,151.2,139.39,153.56,125.69,129.84,135.84,125.39,113.86,118.02,122.91,122.39,101.2,114.37,109.51,109.61,116.11,104.79,109.42,88.36,99.31,95.63,84.95,83.3,71.62,75.14,86.04,78.9,85.02,67.05,66.34,85.26,68.84,79.14,55.35,66.44,59.7,63.67,76.39,69.98,54.47,72.12,45.09,69.22,50.79,54.74,45.5,37.4,49.04,46.15,49.91,52.81,34.51,45.53,43.35,31.15,46.82,33.9,41.56,27.97,25.77,34.33,20.67,28.76,25.85,23.89,30.71,18.07,25.96,20.18,22.26,25.46,13.36,24.26,16.63,18.07,19.6,12.31,18.15,12.09,13.74,20.1,9.41,19.01,11.16,10.7,16.01,7.27,18.13,10.32,10.33,16.42,4.49,15.59,8.12,8.06,12.58,5.68,12.43,5.45,5.18,12.3,5.13,10.8,4.37,3.24,10.73,-1.3,6.38,2.83,-1.04,10.53,-2.46,6.87,2.22,-1.36,9.19,-4.67,4.51,-1.39,0.56,8,-3.63,5.21,-3.63,-6.5,-1.84,-10.35,-5.74,-3.75,-9.66,-1.92,-13.65,-4.51,-6.08,-13.6,-5.06,-9.16,-0.78,-10.4,-12.06,-8.52,-12.54,-6.21,-6.77,-15.46,-4.63,-10.2,-9.87,-17.08,-17.65,-9.29,-14.87,-5.59,-17.38,-14.71,-5.54,-22.55,-12.84,-10.18,-12.88,-1.56,-11.09,-8.22,-8.65,-19.04,-10.96,-24.8,-8.36,-14.76,-15.15,-7.56,-12.35,-17.31,-12.48,-15.64,-3.22,-23.57,-7.61,-8.79,-11.88,-15.94,-12.37,-17.95,-18.54,-19.92,-12.09,-25.09,-14.76,-7.17,-18.53,-15.95,-19.04,-8.11,-7.5,-16.22,-16.93,-24.48,-23.28,-7.76,-22.79,-16.85,-27.93,-20.83,-8.15,-17.23,-8.96,-16.27,-20.31,-9.12,-21.68,-12.25,-24.25,-11.14,-21.65,-24.1,-4.58,-21.63,-10.76,-6.18,-23.54,-13.03,-23.67,-13.01,-5.89,-28.25,-12.08,-16.81,-9.86,-18.76,-19.92,-14.25,-11.64,-17.63,-7.87,-13.36,-2.55,-23.43,-13.54,-13.23,-15.86,-10.22,-10.57,-8.37,-1.32,-17.33,-4.26,-6.94,-13.29,-4.14,-11.7,-6.43,-2.21,-4.44,-6.55,-6.54,-3.59,-10.56,-5.86,-1.51,-6,-2.19,-5.68,-5.95,2.18,-4.77,3.44,-4.45,-2.77,5.51,-6,8.51,5.65,2.01,11.09,2.22,7.75,7.71,3.23,9,0.56,11,2.31,4.48,8.08,2.11,7.84,8.42,6.04,12.29,5.32,10.17,9.61,3.77,12.47,4.44,10.72,10.43,6.31</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B233" t="str">
+        <v>[R_13_标记]</v>
+      </c>
+      <c r="C233" t="str">
+        <v>a: 36.0ms -76.8uv b: 76.8ms 380.9uv</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B234" t="str">
+        <v>[L_13_名字]</v>
+      </c>
+      <c r="C234" t="str">
+        <v>FERG(13)_dMax</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B235" t="str">
+        <v>[L_13_放大器]</v>
+      </c>
+      <c r="C235" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B236" t="str">
+        <v>[L_13_闪光]</v>
+      </c>
+      <c r="C236" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B237" t="str">
+        <v>[L_13_闪光背景]</v>
+      </c>
+      <c r="C237" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B238" t="str">
+        <v>[L_13_采样]</v>
+      </c>
+      <c r="C238" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B239" t="str">
+        <v>[L_13_分析时间]</v>
+      </c>
+      <c r="C239" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B240" t="str">
+        <v>[L_13_数据长度]</v>
+      </c>
+      <c r="C240" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B241" t="str">
+        <v>[L_13_详细数据(uv)]</v>
+      </c>
+      <c r="C241" t="str">
+        <v>15.64,-6.23,10.99,3.22,0.26,13.96,-6.29,16.38,-2.15,8.7,9.31,-1.45,17.98,-4.09,16.45,3.82,6.71,15.54,-1.55,21.01,0.02,15.56,10.34,4.99,20.69,-0.26,22.05,4.99,12.96,16.46,3.01,23.28,1.34,20.04,9.38,8.9,19.24,-0.09,23.09,1.51,15.24,10.63,2.03,18.18,-4.26,18.23,1.83,4.48,11.84,-4.43,13.72,-7.51,9.04,-4.53,-9.7,2.01,-18.77,0.03,-12.43,-8.8,-8.02,-18.52,-5.92,-23.73,-10.66,-22,-12.32,-16.68,-31.14,-3.37,-30.28,-15.32,-25.4,-31.54,-18.16,-23.29,-13.62,-14.84,-22.64,-17.37,-27.15,4.9,-12.67,3.35,-8.8,6.64,11.72,7.21,26.28,16.43,31.61,32.5,22.05,49.73,46.89,71.49,45.98,59.79,73.69,72.58,98.38,89.89,119.25,120.04,96.05,133.42,130.18,155,127.84,166.51,157.68,165.49,196.28,175.61,219.55,206.71,234.84,215.9,225.39,217.1,253.02,224.35,244.88,256.3,274.65,248.82,297.33,258.72,268.18,310.43,276.87,321.43,281.36,343.71,275.1,313.27,316.04,309.21,315.55,322.73,334.07,323.28,297.91,304.36,339.41,351.51,330.79,345.77,312.51,307.41,339.86,326.27,298.09,319.01,303.42,333.48,311,288.1,304.74,320.47,282.75,294.7,333.29,282.54,278.41,249.09,274.01,284.16,243.5,284.84,244.86,240.28,251.66,263.65,266.1,218.1,233.46,239.7,218.94,203.35,197.37,241.69,189.03,197.01,178.6,198.93,195.66,188.82,175.57,152,172.07,171.67,175.26,165.95,147.32,174.06,143.77,165.25,145.34,121.36,146.92,139.11,135.81,135.38,121.26,124.63,121.3,140.76,113.96,132.19,99.14,104.16,107.52,104.97,109.63,99.1,84.23,108.05,90.38,87.23,72.71,91.08,75.09,69.31,89.28,52.97,76.15,58.42,72.41,75.3,58.92,69.32,44.58,67.37,51.6,48.05,62,37.28,48.9,34.75,42.24,33.18,25.14,48.47,19.39,36.9,20.18,30.28,32.48,16.38,35.12,8.78,25.93,17.6,13.99,22.69,3.41,24.81,3.19,13.22,10.72,3.25,21.86,-1.89,15.77,1.46,4.53,10.33,-3.38,16.62,-7.07,12.5,5.12,-2.41,13.12,-7.22,16.2,-5.07,7.87,5.43,-4.91,16.96,-10.1,10.3,0.55,-0.15,9.75,-6.18,16.84,-3.22,10.75,3.05,-1.75,16.18,-9.29,12.77,-4.64,1.77,9.25,-8.85,11.3,-5.61,9.04,-2.63,-1.32,8.35,-8.06,16.24,-8.15,1.5,3.08,-10.26,14.16,-12.65,9.56,-6.01,-1.49,4.6,-11.87,10.76,-19.34,-2.5,-12.06,-13.91,1.49,-24.94,0.63,-17.62,-10.26,-14.18,-21.57,1.03,-29.83,-11.16,-22.47,-22.74,-10.58,-27.13,-8.58,-27.91,-11.84,-17.93,-21.24,-6.56,-26.76,-7.3,-23.99,-20.77,-21.35,-38.38,-15.87,-28.86,-18.81,-26.73,-22.46,-20.44,-37.66,-4.47,-36.43,-20.18,-24.32,-35.09,-18.26,-39.51,-17.23,-21.5,-30.74,-14.93,-32.23,-8.48,-35.3,-18.3,-28.11,-26.16,-17.05,-27.13,-12.53,-33.93,-24.27,-22.48,-21.51,-6.23,-35.57,-7.42,-16.04,-16.09,-10.45,-22.06,-4.82,-17.53,-9.09,-23.4,-17.86,-3.63,-30.54,-4.77,-28.33,-5.75,-5.6,-21.5,3.84,-22.94,-13.8,-16.91,-25.01,-5.44,-27.3,-0.88,-23.23,-15.01,-21.91,-19.56,-5.77,-20.29,-2.02,-18.95,-18.36,-7.74,-21.25,-4.42,-21.88,-5.1,-24.98,-16.74,-13.12,-26.01,-7.73,-31.66,-9.44,-20.86,-22.41,-9.14,-33.96,-7.61,-26.55,-18.99,-9.63,-24.07,-0.98,-19.98,-7.46,-9.56,-16.32,-4.47,-27.14,-0.66,-18.37,-6.44,-8.73,-19.35,0.47,-16.74,2.49,-12.4,-6.19,-1.91,-14.85,7.28,-17.22,-0.3,-1.31,-11.58,10.55,-7.86,9.34,-8.28,3.5,4.86,-4.39,11.85,-5.5,13.33,3.71,2.67,15.46,-4.75,18.25,-0.2,13.99,12.79,0.25,21.5,0.59,21.36,7.09,8.9,19.24,-1.56,20.45,3.5,16.01,9.33,5.68,22.2,-1.37,20.85,4.04,11.59,14.12,0.03</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B242" t="str">
+        <v>[L_13_标记]</v>
+      </c>
+      <c r="C242" t="str">
+        <v>a: 36.0ms -79.6uv b: 77.0ms 393.4uv</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B243" t="str">
+        <v>[R_14_名字]</v>
+      </c>
+      <c r="C243" t="str">
+        <v>FERG(14)_dOps</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B244" t="str">
+        <v>[R_14_放大器]</v>
+      </c>
+      <c r="C244" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B245" t="str">
+        <v>[R_14_闪光]</v>
+      </c>
+      <c r="C245" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B246" t="str">
+        <v>[R_14_闪光背景]</v>
+      </c>
+      <c r="C246" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B247" t="str">
+        <v>[R_14_采样]</v>
+      </c>
+      <c r="C247" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B248" t="str">
+        <v>[R_14_分析时间]</v>
+      </c>
+      <c r="C248" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B249" t="str">
+        <v>[R_14_数据长度]</v>
+      </c>
+      <c r="C249" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B250" t="str">
+        <v>[R_14_详细数据(uv)]</v>
+      </c>
+      <c r="C250" t="str">
+        <v>-18.36,-28.1,-15.18,-18.55,-27.17,-13.9,-18.9,-26.27,-12.86,-19.38,-25.34,-11.99,-19.94,-24.3,-11.21,-20.39,-23.22,-10.53,-20.74,-21.93,-9.87,-20.97,-20.63,-9.41,-21.27,-19.57,-9.33,-22.23,-18.78,-10.03,-23.48,-18.79,-11.71,-25.4,-19.45,-13.78,-27.5,-20.13,-15.55,-28.72,-20.33,-16.99,-29.27,-18.9,-16.98,-28.46,-16.52,-16.41,-26.79,-14.12,-15.25,-24.92,-13.48,-17.15,-25.5,-13.98,-19.86,-28.92,-17.07,-25.16,-32.8,-22,-30.81,-36.55,-23.66,-34.24,-37.18,-23.5,-31.78,-33.2,-18.22,-27.3,-24.23,-10.25,-21.44,-15.96,-4.33,-16.82,-11.43,-3.28,-14.28,-14.45,-7.67,-23.29,-20.15,-17.36,-35.06,-29.87,-28.24,-45.19,-35.29,-34.6,-46.23,-29.53,-30.62,-37.52,-21.46,-16.02,-21.42,-5.33,-1.86,-7.81,11.37,10.27,0.66,14.83,2.53,-3.93,1.8,-6.45,-19.8,-13.21,-27.53,-38.14,-30.15,-41.01,-48.17,-33.57,-43.87,-47,-32.93,-39.35,-31.91,-13.16,-19.54,-12.42,3.04,-2.4,1.21,9.67,0.78,8.13,14.58,-8.56,-6.7,-4.21,-23.53,-21.37,-21.26,-39.59,-37.6,-38.23,-53.09,-41.83,-39.71,-54.2,-34.37,-31.35,-38.1,-23.06,-18.77,-23.58,-8.67,-6.3,-15.84,-0.7,-2.08,-10.15,2.09,-7.23,-15.3,-8.48,-18.39,-27.66,-18.2,-31.09,-35.27,-24.1,-36.96,-37.88,-27.45,-35.35,-32.45,-19.77,-30.22,-24.42,-11.76,-21.42,-15.7,-4.42,-16.68,-9.36,-1.58,-14.35,-8.8,-3.36,-17.87,-12.12,-8.04,-22.69,-15.03,-12.92,-26.56,-17.18,-14.74,-27.78,-15.29,-15.87,-25.65,-13.02,-14.37,-23.87,-10.39,-12.7,-21.62,-7.8,-12.74,-20.56,-6.87,-13.89,-20.36,-7.58,-15.87,-21.6,-9,-18.54,-22.67,-10.44,-21.01,-23.16,-11.47,-22.64,-23.18,-12.02,-24.03,-22.65,-12.42,-24.9,-21.98,-12.72,-25.71,-21.19,-13.25,-26.52,-20.6,-14.01,-27.44,-20.02,-15,-28.18,-19.46,-15.93,-28.69,-18.73,-16.73,-28.85,-17.79,-17.35,-28.66,-16.67,-17.84,-28.11,-15.45,-18.2,-27.33,-14.17,-18.48,-26.35,-12.92,-18.72,-25.2,-11.72,-18.94,-23.94,-10.59,-19.13,-22.56,-9.59,-19.29,-21.11,-8.71,-19.44,-19.63,-8,-19.6,-18.16,-7.49,-19.78,-16.74,-7.2,-20,-15.42,-7.16,-20.27,-14.21,-7.38,-20.59,-13.16,-7.85,-20.96,-12.27,-8.57,-21.38,-11.56,-9.52,-21.82,-11.02,-10.67,-22.27,-10.66,-12,-22.71,-10.47,-13.47,-23.12,-10.42,-15.04,-23.47,-10.51,-16.66,-23.73,-10.7,-18.28,-23.87,-10.98,-19.86,-23.88,-11.31,-21.35,-23.73,-11.67,-22.7,-23.4,-12.04,-23.89,-22.89,-12.4,-24.88,-22.19,-12.74,-25.65,-21.31,-13.03,-26.17,-20.26,-13.28,-26.44,-19.04,-13.49,-26.47,-17.7,-13.65,-26.26,-16.26,-13.78,-25.82,-14.75,-13.89,-25.17,-13.22,-14,-24.36,-11.71,-14.12,-23.41,-10.27,-14.28,-22.35,-8.93,-14.49,-21.22,-7.74,-14.76,-20.06,-6.73,-15.12,-18.9,-5.95,-15.56,-17.78,-5.4,-16.11,-16.73,-5.12,-16.75,-15.76,-5.1,-17.47,-14.9,-5.36,-18.28,-14.15,-5.87,-19.14,-13.53,-6.64,-20.04,-13.02,-7.62,-20.94,-12.62,-8.8,-21.83,-12.33,-10.13,-22.65,-12.12,-11.57,-23.39,-11.97,-13.08,-24,-11.87,-14.61,-24.45,-11.8,-16.12,-24.72,-11.74,-17.56,-24.79,-11.66,-18.9,-24.63,-11.57,-20.09,-24.24,-11.44,-21.12,-23.61,-11.27,-21.96,-22.76,-11.07,-22.6,-21.69,-10.84,-23.02,-20.42,-10.58,-23.24,-19,-10.32,-23.26,-17.44,-10.07,-23.1,-15.8,-9.86,-22.77,-14.11,-9.7,-22.3,-12.43,-9.62,-21.72,-10.8,-9.64,-21.06,-9.26,-9.79,-20.35,-7.87,-10.07,-19.62,-6.65,-10.49,-18.89,-5.64,-11.08,-18.19,-4.86,-11.81,-17.53,-4.35,-12.69,-16.93,-4.09,-13.7,-16.39,-4.1,-14.83,-15.92,-4.36,-16.04,-15.52,-4.87,-17.3,-15.17,-5.59,-18.58,-14.87,-6.5,-19.84,-14.59,-7.56,-21.04,-14.33,-8.73,-22.13,-14.06,-9.98,-23.08,-13.76,-11.26,-23.85,-13.43,-12.54,-24.41,-13.04</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B251" t="str">
+        <v>[R_14_标记]</v>
+      </c>
+      <c r="C251" t="str">
+        <v>63uv</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B252" t="str">
+        <v>[L_14_名字]</v>
+      </c>
+      <c r="C252" t="str">
+        <v>FERG(14)_dOps</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B253" t="str">
+        <v>[L_14_放大器]</v>
+      </c>
+      <c r="C253" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B254" t="str">
+        <v>[L_14_闪光]</v>
+      </c>
+      <c r="C254" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B255" t="str">
+        <v>[L_14_闪光背景]</v>
+      </c>
+      <c r="C255" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B256" t="str">
+        <v>[L_14_采样]</v>
+      </c>
+      <c r="C256" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B257" t="str">
+        <v>[L_14_分析时间]</v>
+      </c>
+      <c r="C257" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B258" t="str">
+        <v>[L_14_数据长度]</v>
+      </c>
+      <c r="C258" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B259" t="str">
+        <v>[L_14_详细数据(uv)]</v>
+      </c>
+      <c r="C259" t="str">
+        <v>9.17,8.52,1.82,11.58,6.23,3.91,12.79,4.2,6.87,12.53,3.08,10.04,11.04,3.3,12.75,8.82,4.95,14.26,6.46,7.33,14.15,4.53,10.03,12.41,3.64,12.32,9.65,4.12,13.55,6.62,6.03,13.84,4.49,8.74,12.86,3.71,11.81,11.05,4.42,14.08,8.46,6.05,14.63,5.64,8.05,12.94,2.67,9.02,9.03,0.64,9.36,4.1,-0.62,8.75,0.63,0.77,7.32,-1.99,4.05,7.11,-0.77,8.82,7.11,2.74,12.81,6.01,5.81,14.73,5.22,9.09,11.95,1.97,9.16,6.75,-1.45,6.72,-0.46,-5.74,1.42,-7.17,-4.96,1.52,-8.55,-0.16,1.91,-4.85,7.76,6.1,4.96,16.56,11.28,15.7,23.52,15.05,20.36,23.7,11.32,21.7,13.94,6.76,12.1,1.84,-3.83,1.05,-10.15,-10.14,-6.38,-16.93,-9.09,-3.88,-8.23,5.39,2.05,5.33,18.1,15.39,20.79,31.99,21.27,32.01,31.03,25.53,31.85,25.27,17.45,20.91,5.93,0.57,3.13,-15.18,-14.57,-13.08,-19.87,-15.07,-21.2,-18.98,-6.67,-9.49,-4.66,9,6.21,15.02,23.35,22.09,29.11,37.14,28.6,36.83,30.21,16.9,24.7,8.98,5.72,4.65,-9.71,-7.37,-10.26,-24.12,-17.94,-20.01,-22.73,-16.44,-14.86,-9.37,1.11,-4.42,7.26,14.71,12.96,23.39,26.49,22.31,31.15,23.78,17.43,24.01,14.14,12.13,12.05,-1.18,2.12,-1.08,-10.18,-5.03,-12.73,-15.16,-4.35,-10.21,-6.55,1.2,-2.94,6.78,10.39,5.98,17.86,15.14,14.06,24.08,14.03,15.72,20.74,11.97,16.3,14.93,4.6,11.54,6.14,0.38,7.8,-0.43,-0.73,5.3,-2.9,2.17,6.71,-1.41,7.07,7.16,1.84,12.31,7.37,6.19,14.36,5.62,8.51,13.01,4.11,10.42,9.58,1.12,9.89,4.27,0.19,8.57,-0.27,0.81,6.96,-3.26,2.96,4.8,-3.3,5.72,2.9,-1.73,8.09,1.01,1.22,8.7,-0.64,4.28,7.53,-1.57,6.79,5.1,-1.16,8.35,2.13,0.4,8.72,-0.31,3.01,7.9,-1.47,6.01,6.17,-1.04,8.64,4.07,1.03,10.25,2.14,4.05,10.41,1,7.38,9.18,1.02,10.19,6.99,2.37,11.92,4.61,4.75,12.15,2.74,7.67,10.94,1.99,10.4,8.67,2.58,12.21,5.96,4.38,12.64,3.54,6.88,11.54,2.03,9.39,9.18,1.79,11.16,6.12,2.82,11.67,3.12,4.78,10.69,0.91,7.03,8.38,-0.04,8.87,5.25,0.41,9.67,2.02,2.03,9.11,-0.55,4.26,7.22,-1.9,6.39,4.39,-1.75,7.75,1.3,-0.25,7.88,-1.3,2.14,6.7,-2.77,4.72,4.47,-2.75,6.77,1.77,-1.24,7.75,-0.65,1.34,7.4,-2.13,4.36,5.86,-2.21,7.04,3.62,-0.8,8.76,1.36,1.81,9.13,-0.23,5.01,8.16,-0.6,8.05,6.22,0.45,10.22,3.94,2.74,11.04,2.03,5.76,10.39,1.09,8.78,8.52,1.47,11.07,6.01,3.12,12.07,3.58,5.64,11.53,1.91,8.36,9.61,1.45,10.56,6.82,2.29,11.59,3.87,4.18,11.15,1.49,6.52,9.26,0.24,8.62,6.35,0.35,9.79,3.1,1.7,9.62,0.26,3.8,8.02,-1.52,5.97,5.33,-1.89,7.5,2.13,-0.84,7.88,-0.81,1.23,6.91,-2.79,3.68,4.77,-3.36,5.78,1.97,-2.41,6.93,-0.77,-0.24,6.79,-2.73,2.58,5.4,-3.37,5.29,3.16,-2.49,7.21,0.72,-0.27,7.89,-1.2,2.77,7.21,-1.99,5.9,5.46,-1.34,8.37,3.21,0.66,9.63,1.18,3.61,9.45,0.01,6.8,7.98,0.12,9.48,5.71,1.58,11.01,3.33,4.06,11.05,1.55,6.96,9.65,0.89,9.54,7.21,1.55,11.11,4.38,3.35,11.25,1.92,5.78,9.87,0.44,8.13,7.29,0.28,9.71,4.14,1.39,9.99,1.16,3.38,8.81,-0.96,5.6,6.35,-1.75,7.34,3.18,-1.13,8.01,0.01,0.62,7.32</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B260" t="str">
+        <v>[L_14_标记]</v>
+      </c>
+      <c r="C260" t="str">
+        <v>62.6uv</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B261" t="str">
+        <v>[R_15_名字]</v>
+      </c>
+      <c r="C261" t="str">
+        <v>FERG(15)_dMax</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B262" t="str">
+        <v>[R_15_放大器]</v>
+      </c>
+      <c r="C262" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B263" t="str">
+        <v>[R_15_闪光]</v>
+      </c>
+      <c r="C263" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B264" t="str">
+        <v>[R_15_闪光背景]</v>
+      </c>
+      <c r="C264" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B265" t="str">
+        <v>[R_15_采样]</v>
+      </c>
+      <c r="C265" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B266" t="str">
+        <v>[R_15_分析时间]</v>
+      </c>
+      <c r="C266" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B267" t="str">
+        <v>[R_15_数据长度]</v>
+      </c>
+      <c r="C267" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B268" t="str">
+        <v>[R_15_详细数据(uv)]</v>
+      </c>
+      <c r="C268" t="str">
+        <v>-16.19,-6.73,-12.64,-19.6,-10.82,-7.13,-17.25,-16.94,-6.92,-11.12,-19.56,-12.16,-6.71,-16.38,-18.27,-8.09,-10.41,-19.98,-14.27,-7.28,-16.09,-20.09,-10.18,-10.49,-20.79,-16.99,-8.75,-16.36,-22.26,-13,-11.43,-22.03,-20.27,-11.22,-17.23,-24.83,-16.94,-13.13,-23.46,-24.37,-14.84,-19.06,-28.39,-21.79,-16.12,-27.71,-31,-19.52,-24.29,-34.08,-30.33,-23.74,-30.95,-37.23,-28,-32.52,-45.26,-37.51,-32.9,-39.72,-53.38,-46.33,-37.69,-58.03,-55.38,-47.81,-50.49,-62.44,-60.47,-45.25,-58.8,-65.35,-57.61,-63.15,-68.71,-59.09,-63.15,-59.16,-74.24,-54.67,-68.86,-64.62,-56.01,-42.62,-57.01,-64.28,-34.68,-35.13,-34.02,-29.55,-19.54,-29.92,-27.66,-6.32,-11.31,-12.89,14.17,32.07,22.9,25.29,57.95,56.78,42.23,57.49,65.29,91.76,92.49,117.09,133.84,119.46,126.7,161.4,172.03,167.7,177.71,194.65,184.62,179.78,189.06,222.44,237.34,221.33,220.88,259.42,270.24,237.77,297.61,296.88,249.07,299.86,306.28,322.97,297.94,278.46,330.55,278.66,321.94,291.61,291.85,357.48,366.12,315.12,314.8,352.07,331.9,310.13,300.41,340.78,358.66,323.78,293.32,292.54,327.18,306.52,317.41,276.75,269.43,290.03,315.84,257.39,298.37,304.67,270.25,270.08,269.29,280.22,259.45,239.78,273.41,252.33,246.8,229.15,250.51,198.91,212.86,191.64,180.68,189.69,204.22,163.13,183.86,160.85,165.72,160.41,156.58,137.03,142.2,126.86,136.74,132.25,109.64,126.21,107.09,117.81,117.78,118.62,107.35,100.06,83.28,80.15,95.98,89.91,73.84,69.17,87.13,88.98,78.62,88.51,62.73,65.61,70.12,78.07,46.83,53.47,54.19,54.21,54.09,49.33,58.25,42.31,35.46,50.15,56.78,27.41,27.98,28.61,32.08,29.67,20.53,27.62,24.23,19.54,17.75,23.81,7.62,18.43,11.88,12.61,9.39,18.92,6.02,6.38,-1.09,11.21,-1.55,-7.25,4.17,4.52,-6.84,-10.36,-1.41,-2.06,-12.45,-6.01,3.09,-15.19,-16.62,-4.65,-6.37,-18.92,-11.21,-3.54,-15.28,-17.5,-9.46,-9.28,-20.56,-14.77,-11.35,-20.39,-23.93,-13.97,-13.31,-22.32,-19.4,-12.25,-19.45,-28.8,-18.62,-16.23,-26.57,-28.06,-19,-24.01,-29.66,-23.62,-20.79,-32.45,-33.9,-20.16,-24.67,-35.18,-26.64,-24.65,-35.31,-36.7,-29.54,-29.73,-35.2,-36.28,-26.36,-33.04,-38.17,-32.61,-32.62,-39.91,-40.9,-33.91,-34.45,-49.45,-33.49,-35.8,-42.14,-47.74,-34.5,-39.17,-49.8,-44.52,-34.91,-48.76,-52.75,-34.98,-45.8,-56.09,-45.07,-43.16,-50.23,-56.08,-39.75,-47.19,-54.76,-49.94,-39.06,-49.64,-57.41,-35.32,-36.31,-50.93,-42.74,-40.55,-41.55,-53.36,-41.57,-48,-49.58,-52.35,-43.12,-39.35,-53.01,-52.99,-36.03,-47.81,-49.01,-39.46,-39.61,-56.4,-56.72,-50.88,-50.52,-64.15,-39.37,-36.67,-46.98,-59.6,-39.06,-48.25,-55.06,-44.16,-49.5,-59.62,-60.42,-48.74,-45.76,-55.45,-49.61,-40.96,-48.66,-60.95,-44.53,-44.1,-59.92,-59.38,-48.84,-59.41,-56.07,-46.53,-45.16,-69.17,-60.93,-52.15,-53.61,-70.01,-43.46,-56.74,-57.54,-51.68,-58.11,-59.94,-57.6,-43.72,-57.3,-64.23,-59.94,-50.48,-47.32,-68.07,-56,-49.73,-66.16,-62.35,-40.68,-58.42,-56.77,-57.54,-51.79,-54.16,-56.86,-48.32,-42.52,-49.35,-46.39,-49,-51.03,-56.72,-49.57,-50.31,-46.98,-49.56,-44.04,-45.88,-47.13,-35.9,-38.34,-49.7,-46.86,-40.56,-45.72,-51.82,-42.35,-35.34,-48.43,-39.65,-26.4,-31.55,-39.31,-32.27,-33.22,-38.8,-39.41,-35.62,-32.52,-36.64,-32.55,-31.89,-34.78,-39.35,-24.88,-30.27,-39.26,-32.19,-28.24,-30.03,-34.87,-31.39,-27.52,-37.71,-34.75,-27.3,-33.31,-34.81,-30.78,-24.84,-33.17,-35.52,-27.24,-24.2,-36.88,-26.93,-23.73,-31.13,-35.8,-26.18,-22.41,-32.27,-30.91,-22.1,-31.65,-32.92,-23.08,-23.23,-32.64,-27.9,-18.69,-26.85,-34.68,-23.82,-22.75,-29.88,-32.54,-20.01</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B269" t="str">
+        <v>[R_15_标记]</v>
+      </c>
+      <c r="C269" t="str">
+        <v>a: 39.8ms -89.2uv b: 84.4ms 427.4uv</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B270" t="str">
+        <v>[L_15_名字]</v>
+      </c>
+      <c r="C270" t="str">
+        <v>FERG(15)_dMax</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B271" t="str">
+        <v>[L_15_放大器]</v>
+      </c>
+      <c r="C271" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B272" t="str">
+        <v>[L_15_闪光]</v>
+      </c>
+      <c r="C272" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B273" t="str">
+        <v>[L_15_闪光背景]</v>
+      </c>
+      <c r="C273" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B274" t="str">
+        <v>[L_15_采样]</v>
+      </c>
+      <c r="C274" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B275" t="str">
+        <v>[L_15_分析时间]</v>
+      </c>
+      <c r="C275" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B276" t="str">
+        <v>[L_15_数据长度]</v>
+      </c>
+      <c r="C276" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B277" t="str">
+        <v>[L_15_详细数据(uv)]</v>
+      </c>
+      <c r="C277" t="str">
+        <v>-0.12,-2.83,15.19,6.92,-5.16,11.45,13.31,-4.07,5.66,17.08,0.23,-0.13,17.07,6.39,-3.93,13.33,12.37,-4.48,7.08,16.13,-1.67,0.3,16.31,3.44,-4.9,12.67,8.93,-7.01,6.19,12.74,-5.58,-1.25,13.28,-1.43,-7.56,10.04,3.72,-10.94,3.6,7.62,-10.93,-4.04,8.84,-7.4,-11.7,5.73,-3.18,-16.42,-1.22,0.83,-18.34,-9.65,0.45,-17.41,-18.87,-1.87,-13.44,-26.6,-10.35,-10.04,-28.26,-18.99,-14.31,-32.92,-30.6,-15.07,-29.66,-43.2,-23.86,-26.36,-52.51,-31.9,-27.12,-49.37,-44.42,-41.12,-44.38,-58.14,-32.77,-47.59,-59.89,-51.94,-35.5,-55.88,-52.88,-23.44,-42.31,-57.12,-30.7,-44.36,-53.26,-34.34,-18.18,-35.58,-19.25,-3.47,-7.31,-2.18,17.39,7.67,21.11,42.19,31.02,28.6,54.48,66.04,57.11,55.4,82.59,88.26,75.18,107.21,137.1,128.38,135.06,142.3,156.11,147.78,172.16,183.88,169.63,182.29,232.45,227.75,232.74,245.11,216.93,262.71,236.78,248.24,252.2,265.2,292.62,263.71,313,282.63,307.07,273.96,290.06,295.53,314.51,371.86,297.23,315,369.5,378.6,325.25,322.15,324.26,303.06,321.18,381.25,340.32,334.71,351.5,352.93,333.96,365.23,299.4,320.88,296.44,334.6,327.73,283.54,331.83,315.6,236.62,280,280.57,262.03,250.18,249.42,263.1,238.36,269.75,229.46,218.9,231.6,216.95,191.2,192.57,181.24,168.31,155.3,182.71,159.77,142.42,159.86,161.75,138.13,149.82,162.13,133.73,140.12,143.8,118.07,114.53,132.54,121.99,109.89,109.47,108.18,108.07,108.26,113.46,88.67,86.5,99.43,100.9,86.39,90.82,88.07,69.96,80.65,79.96,55.84,49.14,66.18,77.49,52.22,79.11,73.58,36.96,43.32,63.38,45.5,34.89,68.24,52.32,43.78,58.18,57.61,20.13,48.56,39.65,37.7,24.72,48.5,29.11,16.09,32.79,27.9,18.96,27.56,32.57,9.22,20.24,32.63,15.04,5.03,21.94,21.89,1.92,17.07,20.2,2.34,7.8,25.43,6.52,1.76,19.47,12.43,-5.17,13.12,15.44,-4.1,3.88,15.84,-0.08,-3.41,13.3,5.45,-8.87,7.93,9.73,-6.8,0.71,11.38,-4.39,-4.04,8.66,-1.95,-11.96,3.39,2.07,-12.41,-0.99,2.45,-11.69,-13.01,5.32,-11.75,-18.45,3.44,-4.06,-22.05,-8.79,-0.45,-19.55,-13.13,-4.17,-18.82,-22.18,-5.99,-10.46,-27.25,-14.55,-10.49,-28.02,-21.44,-13.72,-25.37,-30.17,-12.15,-25.55,-36.3,-22.2,-14.72,-37.67,-27.6,-18.97,-37.48,-27.34,-10.82,-28.95,-42.1,-18.93,-20.44,-43.46,-27.02,-19.5,-33.2,-36.27,-19.21,-33.98,-32.85,-20.11,-23.81,-35.69,-22.03,-15.46,-39.79,-28.55,-12.02,-36.01,-32.11,-22.2,-23.6,-32.02,-28.61,-16.18,-38.13,-38.91,-13.03,-42.04,-39.69,-15.04,-34.85,-40.8,-29.65,-21.54,-34.5,-37.29,-15.18,-33.57,-41.26,-13.05,-33.61,-45.13,-17.57,-21.23,-46.17,-32.93,-12.62,-39.5,-39.68,-18.04,-36.7,-45.57,-31.78,-30.76,-41.02,-25.8,-30.91,-45.89,-31.84,-23.9,-48.69,-53.99,-34.61,-33.93,-41.82,-34.81,-24.9,-43.78,-49.36,-24.26,-35.41,-43.02,-30.68,-45.14,-42.55,-34.65,-31.4,-59.56,-38.09,-25.9,-48.68,-50.99,-25.75,-42.56,-54.63,-39.21,-34.94,-57.39,-30.8,-21.13,-47.46,-46.51,-26.03,-43.52,-53.08,-18.52,-25.64,-36.88,-27.62,-28.13,-35.3,-40.61,-18.42,-38.92,-37.84,-15.09,-24.5,-31.54,-26.66,-11.02,-31.55,-23.66,-11.68,-27.67,-30.8,-17.94,-24.66,-34.2,-10.66,-6.42,-32.82,-14.17,-8.36,-25.74,-27.64,-4.16,-13.09,-26.75,-10.31,-3.6,-23.1,-16.76,-6.14,-23.1,-13.77,-3.49,-15.42,-18.34,-1.74,-7.79,-22.94,-7.22,-0.81,-20.53,-12.03,-3.54,-16.22,-22.36,-4.43,-8.64,-24.07,-10.94,-4.1,-23.22,-15.59,-2.92,-16.21,-18.88,-3.73,-11.77,-21.11,-7.02,-7.79,-20.32,-13.49,-0.43,-18.15,-19.35,0.91,-10.3,-23.87,-4.3,-5.2</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B278" t="str">
+        <v>[L_15_标记]</v>
+      </c>
+      <c r="C278" t="str">
+        <v>a: 39.8ms -87.1uv b: 84.4ms 473.2uv</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B279" t="str">
+        <v>[R_16_名字]</v>
+      </c>
+      <c r="C279" t="str">
+        <v>FERG(16)_dOps</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B280" t="str">
+        <v>[R_16_放大器]</v>
+      </c>
+      <c r="C280" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B281" t="str">
+        <v>[R_16_闪光]</v>
+      </c>
+      <c r="C281" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B282" t="str">
+        <v>[R_16_闪光背景]</v>
+      </c>
+      <c r="C282" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B283" t="str">
+        <v>[R_16_采样]</v>
+      </c>
+      <c r="C283" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B284" t="str">
+        <v>[R_16_分析时间]</v>
+      </c>
+      <c r="C284" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B285" t="str">
+        <v>[R_16_数据长度]</v>
+      </c>
+      <c r="C285" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B286" t="str">
+        <v>[R_16_详细数据(uv)]</v>
+      </c>
+      <c r="C286" t="str">
+        <v>11.11,18.03,7.63,-3.26,3.01,15.7,13.41,-0.51,-3.53,8.83,15.68,5.13,-5.87,0.3,12.87,10.52,-3.48,-6.58,5.71,12.48,1.92,-9.15,-3.07,9.53,7.26,-6.66,-9.75,2.68,9.62,-0.69,-11.53,-5.15,7.78,5.82,-7.78,-10.4,2.24,9.6,-0.46,-11.37,-4.88,8.16,6.14,-7.48,-10.41,2.05,9.05,-1.13,-12.17,-5.78,7.5,5.62,-7.71,-10.29,2.28,10.68,1.09,-8.88,-1.47,12.51,11.82,-1.07,-2.69,10.26,18.44,9.46,-1.49,4.88,18.09,15.26,0.54,-3.41,8.25,14.02,2.47,-9.05,-3.12,7.93,7.25,-7.35,-10.24,5.12,13.05,5.71,-3.08,5.65,20.96,22.04,11.05,7.33,21.21,31.61,20.36,7.85,12.6,20.42,15.82,-1.3,-8.02,0.03,3.91,-10.23,-22.36,-18.65,-6.13,-11.07,-23.93,-20.02,-7.67,4.92,-0.39,-5.9,3.14,24.31,27.01,13.09,9.56,28.75,30.53,22.3,3.05,9.54,15.1,7.13,-12.18,-23.76,-14.91,-16.77,-30.9,-35.62,-32.52,-25.32,-21.6,-26.41,-28.22,-7.33,5.62,1.95,-0.24,10.39,27.2,29.94,26.4,23.47,36.09,40.13,26.07,5.89,8.01,14.89,7.78,-10.68,-18.42,-11.46,-6.74,-18.07,-36.4,-23.13,-8.5,-6.01,-18.23,-12.88,4.18,17.4,12.45,5.74,18.08,31.37,30.26,18.08,18.18,25.25,33.93,17.67,3.25,5.66,14.55,9.05,-9.85,-16.56,-6.22,-1.27,-10.81,-18.01,-12.1,0.41,2.32,-8.99,-9.94,5.44,15.55,7.71,-1.71,4.76,20.12,15.94,2.19,-2.84,9.88,15.81,3.52,-9.58,-5.72,5.56,2.14,-13.06,-16.89,-4.26,1.85,-7.03,-17.94,-11.89,2.62,1.35,-11.02,-13.35,0,8.27,-1.23,-11.8,-5.27,7.73,6.34,-6.54,-10.57,1.94,9.28,-0.67,-11.79,-5.88,7.08,5.87,-7.62,-10.76,1.97,10.03,0.65,-9.97,-3.56,10.02,9.15,-3.91,-6.77,6.12,14.18,4.65,-5.97,0.09,13.45,12.28,-1.13,-4.41,8.1,15.83,6.11,-4.92,1.02,14.14,12.77,-0.84,-4.24,8.16,15.76,5.93,-5.25,0.52,13.5,11.99,-1.79,-5.39,6.78,14.23,4.23,-7.16,-1.59,11.23,9.58,-4.35,-8.11,3.94,11.32,1.24,-10.21,-4.71,8.09,6.46,-7.46,-11.21,0.87,8.32,-1.67,-13.06,-7.47,5.44,3.95,-9.83,-13.47,-1.25,6.38,-3.42,-14.64,-8.89,4.21,2.95,-10.63,-14.08,-1.66,6.2,-3.37,-14.39,-8.45,4.87,3.83,-9.55,-12.83,-0.23,7.83,-1.55,-12.43,-6.36,7.1,6.22,-7.04,-10.25,2.43,10.58,1.28,-9.57,-3.5,9.99,9.13,-4.14,-7.4,5.23,13.33,3.97,-6.97,-1.02,12.36,11.39,-2.02,-5.45,7.01,14.97,5.44,-5.71,0.03,13.22,12.07,-1.54,-5.21,7.03,14.79,5.07,-6.3,-0.79,12.2,10.88,-2.93,-6.81,5.24,12.85,2.98,-8.55,-3.21,9.65,8.24,-5.67,-9.66,2.29,9.86,-0.04,-11.62,-6.32,6.55,5.17,-8.71,-12.68,-0.68,6.98,-2.82,-14.32,-8.93,4.07,2.85,-10.88,-14.72,-2.56,5.29,-4.3,-15.62,-10.06,3.15,2.16,-11.36,-15.01,-2.65,5.44,-3.93,-15.06,-9.3,4.11,3.34,-9.99,-13.48,-0.95,7.32,-1.88,-12.87,-7.01,6.53,5.89,-7.34,-10.77,1.81,10.15,1.01,-9.97,-4.12,9.41,8.77,-4.49,-7.99,4.51,12.79,3.57,-7.54,-1.83,11.58,10.82,-2.6,-6.29,6.03,14.15,4.76,-6.56,-1.08,12.13,11.19,-2.44,-6.36,5.73,13.65,4.07,-7.46,-2.2,10.81,9.7,-4.11,-8.23,3.68,11.47,1.76,-9.93,-4.81,8.1,6.91,-6.98,-11.2,0.65,8.41,-1.31,-13.02,-7.92,5.02,3.89,-9.95,-14.13,-2.21,5.66,-3.94,-15.54,-10.34,2.74,1.79,-11.88,-15.91,-3.82,4.26,-5.13,-16.55,-11.16,2.13,1.42,-12.04,-15.88,-3.59,4.72,-4.45,-15.67,-10.11,3.39,2.88,-10.4,-14.09,-1.65,6.83,-2.18,-13.29,-7.64</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B287" t="str">
+        <v>[R_16_标记]</v>
+      </c>
+      <c r="C287" t="str">
+        <v>66.8uv</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B288" t="str">
+        <v>[L_16_名字]</v>
+      </c>
+      <c r="C288" t="str">
+        <v>FERG(16)_dOps</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B289" t="str">
+        <v>[L_16_放大器]</v>
+      </c>
+      <c r="C289" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B290" t="str">
+        <v>[L_16_闪光]</v>
+      </c>
+      <c r="C290" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B291" t="str">
+        <v>[L_16_闪光背景]</v>
+      </c>
+      <c r="C291" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B292" t="str">
+        <v>[L_16_采样]</v>
+      </c>
+      <c r="C292" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B293" t="str">
+        <v>[L_16_分析时间]</v>
+      </c>
+      <c r="C293" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B294" t="str">
+        <v>[L_16_数据长度]</v>
+      </c>
+      <c r="C294" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B295" t="str">
+        <v>[L_16_详细数据(uv)]</v>
+      </c>
+      <c r="C295" t="str">
+        <v>16.47,12.5,0.46,3.19,15.16,13.13,0.62,1.31,13.49,13.47,0.9,-0.47,11.66,13.74,1.53,-1.88,9.87,13.95,2.26,-3.09,7.78,13.63,2.54,-4.58,4.81,12.13,2.27,-6.87,1.09,9.71,1.33,-9.13,-2.87,7.72,0.9,-10.08,-4.26,6.97,3.3,-8.02,-4.16,8.62,7.24,-4.42,-2.61,10.61,10.33,-2.14,-3.15,8.82,10.79,-2.13,-6.39,4.46,6.76,-6.5,-12.21,-0.55,3.22,-7.69,-13.23,-2.53,4.59,-3.31,-8.41,2.47,14.15,8.71,1.55,12.01,23.92,18.32,11.01,15.99,27.88,19.4,7.55,7.93,16.96,11.01,-4.42,-8.52,2.28,0.47,-14.82,-16.31,-3.05,-4.1,-13.83,-13.07,2.77,9.86,3.96,4.72,20.64,33.54,26.81,17.78,30.5,37.8,32.22,14.79,19.76,26.07,10.86,-4.27,-4.28,-0.77,-13.25,-27.68,-22.12,-17.76,-17.69,-37.89,-24.78,-10.24,-5.98,-14.74,-5.59,13.94,19.18,10.53,14.49,34.79,36.81,21.8,21.08,27.37,26.29,8.81,-0.21,4.1,2.86,-13.08,-26.3,-20.15,-18.84,-26.75,-32.38,-24.56,-14.67,-19.63,-21.92,-7.31,7.14,5.04,1.76,10.15,24.49,24.96,17.21,19.53,30.23,24.78,12.05,9.47,16.82,11.89,-4.47,-6.98,0.29,0.44,-13.77,-18.11,-5.56,-2.07,-10.33,-12.6,3.28,9.99,1.26,-1.07,11.76,21.73,11.33,4.89,16.2,23.54,14.1,4.01,11.77,19.43,10.27,-1.53,3.44,12.2,5.37,-6.84,-2.7,8.55,3.47,-7.54,-5.64,8.08,5.78,-5.43,-3.94,8.93,9.52,-2.27,-3.22,8.87,11.22,-1.33,-4.75,6.25,9.78,-2.4,-8.13,2.3,7.8,-3.35,-10.63,-0.91,6.57,-3.11,-11.86,-2.87,6.2,-1.58,-11.29,-4,6.71,0.7,-10.08,-4.56,7.06,2.92,-8.74,-5.15,6.98,4.81,-7.32,-5.83,6.72,6.56,-5.62,-6.14,6.42,8.38,-3.53,-6,6.2,10.24,-1.12,-5.54,5.99,11.92,1.41,-4.87,5.61,13.25,3.84,-4.16,4.97,14.08,6.02,-3.48,4.03,14.35,7.86,-2.87,2.82,14.08,9.34,-2.33,1.38,13.27,10.42,-1.87,-0.24,11.95,11.06,-1.51,-2,10.16,11.26,-1.23,-3.82,7.99,11.06,-1,-5.6,5.53,10.51,-0.77,-7.25,2.93,9.69,-0.49,-8.65,0.3,8.67,-0.11,-9.71,-2.22,7.54,0.41,-10.36,-4.51,6.38,1.11,-10.51,-6.47,5.27,2.01,-10.15,-8.02,4.24,3.09,-9.26,-9.1,3.35,4.33,-7.88,-9.68,2.6,5.69,-6.05,-9.79,1.99,7.09,-3.86,-9.44,1.5,8.45,-1.42,-8.7,1.08,9.69,1.14,-7.64,0.7,10.7,3.71,-6.36,0.29,11.41,6.14,-4.95,-0.18,11.72,8.32,-3.51,-0.76,11.59,10.14,-2.11,-1.47,10.98,11.51,-0.82,-2.32,9.89,12.37,0.3,-3.3,8.33,12.71,1.22,-4.36,6.37,12.52,1.94,-5.47,4.08,11.85,2.48,-6.55,1.57,10.75,2.86,-7.52,-1.05,9.31,3.13,-8.31,-3.65,7.62,3.34,-8.82,-6.08,5.79,3.55,-8.99,-8.24,3.93,3.79,-8.77,-10.01,2.13,4.1,-8.12,-11.32,0.47,4.51,-7.04,-12.09,-0.98,5.02,-5.54,-12.31,-2.19,5.6,-3.67,-11.98,-3.13,6.23,-1.51,-11.15,-3.81,6.85,0.84,-9.86,-4.26,7.4,3.27,-8.22,-4.52,7.79,5.65,-6.32,-4.65,7.98,7.86,-4.28,-4.69,7.88,9.77,-2.22,-4.71,7.44,11.29,-0.23,-4.76,6.64,12.32,1.58,-4.86,5.45,12.81,3.14,-5.04,3.91,12.74,4.39,-5.29,2.05,12.1,5.33,-5.6,-0.07,10.94,5.93,-5.92,-2.35,9.33,6.23,-6.22,-4.68,7.36,6.26,-6.42,-6.94,5.13,6.09,-6.46,-9.03,2.77,5.77,-6.29,-10.81,0.4,5.38,-5.86,-12.18,-1.86,4.96,-5.12,-13.08,-3.92,4.57,-4.07,-13.43,-5.68,4.25,-2.72,-13.22,-7.09,4.01,-1.09,-12.45,-8.11,3.84,0.75,-11.17,-8.74,3.73,2.72,-9.43</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B296" t="str">
+        <v>[L_16_标记]</v>
+      </c>
+      <c r="C296" t="str">
+        <v>64.1uv</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B297" t="str">
+        <v>[R_17_名字]</v>
+      </c>
+      <c r="C297" t="str">
+        <v>FERG(17)_dMax</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B298" t="str">
+        <v>[R_17_放大器]</v>
+      </c>
+      <c r="C298" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B299" t="str">
+        <v>[R_17_闪光]</v>
+      </c>
+      <c r="C299" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B300" t="str">
+        <v>[R_17_闪光背景]</v>
+      </c>
+      <c r="C300" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B301" t="str">
+        <v>[R_17_采样]</v>
+      </c>
+      <c r="C301" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B302" t="str">
+        <v>[R_17_分析时间]</v>
+      </c>
+      <c r="C302" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B303" t="str">
+        <v>[R_17_数据长度]</v>
+      </c>
+      <c r="C303" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B304" t="str">
+        <v>[R_17_详细数据(uv)]</v>
+      </c>
+      <c r="C304" t="str">
+        <v>-11.02,-21.42,-24.04,-16.69,-6.79,-4.21,-11.76,-22.49,-26.37,-19.97,-9.74,-5.83,-12.26,-23.1,-28.13,-22.73,-12.3,-7.07,-12.25,-22.99,-29.05,-24.7,-14.22,-7.76,-11.56,-22.03,-29.05,-25.81,-15.49,-7.85,-10.29,-20.33,-28.22,-26.14,-16.06,-7.55,-8.57,-18.12,-27.08,-26.54,-16.7,-7.77,-7.32,-16.35,-26.25,-27.38,-18.32,-8.69,-7.42,-16.81,-25.92,-28.73,-21.09,-13.91,-11.05,-18.86,-29.35,-31.9,-28.65,-18.56,-17.13,-21.6,-36.97,-39.23,-40.32,-29.93,-21.08,-29.39,-38.44,-47.48,-47.27,-31.66,-35.95,-44.31,-52.88,-61.82,-56.2,-54.21,-40.23,-47.99,-54.76,-71.79,-51.33,-52.71,-51.53,-47.32,-49.5,-57.91,-54.05,-35.96,-20.49,-36.79,-25.69,-43.64,-32.77,-12.84,-5.97,9.17,6.31,1.97,-13.26,28.06,26.34,41.88,39.87,23.47,46.46,54.71,82.74,103.96,77.26,71.85,87.19,106.6,137.7,148.3,135.33,156.89,151.02,132.23,154.71,212.03,195.78,192,215.92,219.81,208.57,213.32,244.2,230.68,243.23,261.06,291.38,286.13,314.54,244.78,241.75,250.88,267.63,298.66,277.03,338.56,316.15,283.31,324.7,301.37,331.15,304.65,304.78,293.08,307.63,314.48,309.52,306.35,339.54,339.37,278.76,355.92,314.32,319.48,277.93,255.95,311.81,321.28,294.72,283.61,245.65,295.3,248.7,259.83,294.46,233.22,219.03,216.53,216.7,219.87,254.51,243.23,194.72,174.53,208.48,204.88,214.18,189.05,179.89,166.91,168.87,151.56,174.56,160.05,170.53,131.64,146.31,147.62,135.03,128.51,119.15,112.38,112.37,90.27,111.08,116.47,102.96,91.22,93.78,91.55,100.61,85.52,76.15,67.47,70.38,74.44,79.92,73.71,65.57,75.57,44,49.6,77,79.14,65.93,48.24,36.75,42.36,59.39,61.26,43.19,36.92,26.13,33.23,42.08,57.81,42.08,30.02,22.77,26.12,21.98,45.23,28.91,25.75,11.41,6.94,16.21,27.28,29.3,17.75,-0.84,3.98,12.18,13.46,16.16,12.75,-5.65,-2.83,-3.92,11.31,8.46,2.86,-7.14,-11.2,-9.4,-0.67,2.81,-4.21,-13.67,-21.59,-19.85,-9.89,-5.64,-7.32,-18.2,-28.05,-26.68,-13.34,-8.72,-13.46,-25.63,-34.92,-30.37,-19.73,-15.61,-17.96,-26.78,-37.68,-36.98,-27.17,-21.33,-21.71,-29.34,-37.9,-41.05,-28.74,-21.04,-20.25,-27.78,-42.52,-40.14,-36.67,-25.91,-23.09,-29.33,-41.13,-42.51,-39.32,-22.63,-23,-26.97,-36.71,-46.23,-36.72,-30.92,-25.22,-25.51,-38.29,-43.38,-42.04,-26.97,-18.67,-23.07,-34.18,-48.93,-36.41,-34.29,-24.09,-23.56,-41.47,-44.98,-37.85,-36.26,-29.57,-27.75,-34.34,-49.89,-47,-33.64,-28.33,-31.78,-34.37,-49.76,-42.25,-34.66,-35.58,-30,-41.49,-44.13,-50.48,-38.08,-31.26,-30.01,-36.96,-53.05,-53.55,-54.18,-31.82,-41.98,-40.46,-57.41,-66.5,-61.35,-46.44,-38.45,-51.93,-52.93,-63.12,-63.21,-48.77,-40.5,-42.59,-65.91,-61.25,-53.32,-55.27,-42.66,-44.74,-60.75,-59.12,-73.27,-48.38,-49.4,-55.35,-58.46,-62.56,-74.42,-55.98,-51.57,-53.39,-47.71,-74.74,-56.57,-51.95,-41.75,-39.08,-53.65,-59.11,-61.75,-54.08,-48.99,-38.82,-57.31,-55.38,-68.94,-52.2,-35.65,-41.03,-53.91,-65.42,-67.14,-46.25,-36.86,-39.05,-47.14,-46.77,-62.77,-59.04,-35.91,-39.16,-37.36,-55.58,-55.31,-54.68,-41.05,-35.85,-27.86,-41.86,-49.06,-49.59,-44.06,-25.09,-39.8,-50.87,-52.63,-53.87,-38.5,-37.57,-32.44,-41.43,-56.6,-50.47,-35.07,-30.4,-30.75,-35.27,-51.69,-49.06,-40.98,-30.63,-35.03,-43.94,-44.05,-45.36,-41.33,-31.83,-30.45,-31.84,-51.36,-49.25,-45.12,-29.77,-32.53,-37.66,-47.65,-49.72,-47.58,-38.1,-27.07,-31.69,-45.05,-47.33,-42.25,-30.01,-22.45,-27.45,-38.38,-48.39,-41.49,-31.03,-24.85,-21.61,-35.21,-45.19,-38.85,-28.19,-17.42,-19.4,-31.79,-40.14,-35.72,-25.32,-17.19,-16.52,-23.1,-35.48,-32.36,-26.45,-12.67,-14.24,-20.03,-31.23,-29.27,-22.22</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B305" t="str">
+        <v>[R_17_标记]</v>
+      </c>
+      <c r="C305" t="str">
+        <v>a: 44.3ms -89.0uv b: 91.3ms 414.2uv</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B306" t="str">
+        <v>[L_17_名字]</v>
+      </c>
+      <c r="C306" t="str">
+        <v>FERG(17)_dMax</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B307" t="str">
+        <v>[L_17_放大器]</v>
+      </c>
+      <c r="C307" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B308" t="str">
+        <v>[L_17_闪光]</v>
+      </c>
+      <c r="C308" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B309" t="str">
+        <v>[L_17_闪光背景]</v>
+      </c>
+      <c r="C309" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B310" t="str">
+        <v>[L_17_采样]</v>
+      </c>
+      <c r="C310" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B311" t="str">
+        <v>[L_17_分析时间]</v>
+      </c>
+      <c r="C311" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B312" t="str">
+        <v>[L_17_数据长度]</v>
+      </c>
+      <c r="C312" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B313" t="str">
+        <v>[L_17_详细数据(uv)]</v>
+      </c>
+      <c r="C313" t="str">
+        <v>-17.2,-7.19,-6.52,-16.32,-25.18,-22.82,-12.43,-6.83,-13.1,-24.08,-26.94,-18.6,-9.41,-10.73,-21.3,-28.75,-24.44,-13.82,-9.92,-17.65,-27.99,-28.73,-19.2,-10.99,-14.13,-24.98,-30.64,-24.4,-13.87,-11.67,-20.55,-29.79,-28.37,-17.98,-11.18,-15.89,-26.79,-30.56,-22.59,-12.76,-12.46,-22.48,-30.42,-27.71,-16.46,-12.28,-18.79,-29.43,-31.71,-23.68,-13.79,-18.85,-29.39,-35.14,-32.59,-20.04,-18.71,-30.56,-41.63,-39.91,-34.48,-23.01,-35.29,-48.39,-52.09,-49.22,-33.43,-35.84,-53.06,-53.6,-61.42,-51.09,-38.55,-48.43,-69.47,-58.39,-58.27,-41.3,-55.15,-60.1,-69.22,-60.39,-45.45,-51.65,-46.99,-67.68,-49.8,-49.59,-33.19,-26.25,-39.93,-32.34,-36.37,-13.62,2,4.06,-5.72,-6.08,1.83,25.32,27.84,17.33,35.89,31.86,57.7,61.11,65.43,65.54,98.92,87.08,116.12,121.41,98.86,100.84,120.97,145.92,178.13,139.78,179.34,180.98,181.99,229.91,228.72,204.13,186.15,224.82,244.56,266.19,227.82,241.35,272.46,299.26,285.48,247.73,276.27,271.39,282.48,300.63,273.11,288.56,317.98,277.39,311.65,316.51,275.11,334.3,296.84,312.25,353.71,337.72,298.96,290.21,282.05,287.17,327.24,272.23,299.24,289.31,306.74,297.7,284.15,277,283.52,235.74,294,261.46,237.99,213.85,224.14,252.34,226.89,227.45,210.71,211.46,206.61,202.23,190.63,172.26,173.98,180.28,172.92,160.36,141.17,133.59,146.75,139.96,147.35,132.6,114.69,113.86,98.81,131.58,120.86,100.35,87.71,80.89,123.61,95.35,97.75,81.3,71.67,72.24,93.72,93.16,60.36,53.96,73.8,82.31,68.96,59.25,54.52,54.59,60.03,64.4,54.15,32.74,27.68,50.06,65.29,45.4,35.44,31.52,27.7,39.79,52.2,29.94,25.53,33.99,36.86,33.52,39.08,13.79,13.25,12.62,31.32,38.24,17.79,17.68,15.22,19.37,23.3,13.81,9.35,4.06,7.19,12.95,15.75,2.59,0.94,-3.49,9.94,16.73,4.28,-8.41,-6.2,2.2,10.35,1.25,-5.09,-17.21,-8.37,0.41,2.4,-7.97,-18.18,-16.27,-10.27,-2.58,-6.49,-17.94,-27.34,-18.32,-7.65,-7.71,-19.55,-28.84,-26.14,-14.25,-9.57,-18.82,-28.98,-33.72,-23.28,-17,-14.78,-27.91,-34.58,-29.34,-20.8,-20.55,-22.91,-33.82,-38.49,-26.49,-19.9,-22.77,-36.85,-42.73,-30.93,-26.51,-22.58,-33.84,-39.94,-40.66,-25.06,-22,-23.44,-34.25,-37.5,-30.77,-25.83,-24.02,-31.16,-40.64,-41.7,-27.47,-18.94,-28.26,-41.43,-42.17,-31.8,-27.7,-22.87,-41.46,-42.95,-34.48,-22.69,-23.45,-28.1,-36.05,-44.41,-30.94,-25.5,-30.49,-36.85,-47.7,-35.74,-22.15,-20.56,-42.43,-48.85,-36.98,-34.88,-31.97,-33.51,-47.62,-55.22,-32.62,-31.57,-29.95,-47.26,-56.03,-43.42,-33.46,-28.81,-48.23,-46.32,-49.1,-38.13,-43.04,-31.48,-51.73,-48.93,-52.64,-38.9,-35.12,-51.5,-52.15,-48.31,-52.16,-41.26,-47.64,-58.63,-56.19,-54.51,-41.58,-34.56,-54.54,-52.14,-65.25,-43.23,-36.55,-52.01,-62.19,-60.4,-54.47,-44.82,-52.95,-47.19,-69.53,-62.86,-40.71,-36.02,-49.06,-65.95,-57.5,-50.7,-35.11,-46.71,-54.18,-48.34,-44.97,-35.33,-36.68,-37.88,-52.32,-51.11,-32.16,-38.28,-41.23,-40.46,-52.67,-35.09,-33.32,-31.72,-47.75,-56.18,-51.4,-27.8,-35.75,-35.63,-39.73,-45.27,-36.18,-28.09,-24.16,-45.78,-42.07,-44.14,-23.68,-17.44,-36.12,-36.7,-35.75,-24.37,-19.69,-25.5,-31.73,-38.23,-40.49,-18.41,-26.05,-37.75,-35.44,-35.36,-25.17,-16.08,-24.33,-37.4,-35.49,-28.81,-20.2,-20.21,-33.7,-39.65,-39.02,-29.99,-19.53,-32.04,-42.26,-37,-25.21,-24.14,-20.55,-34.94,-43.28,-35.9,-25.48,-20.87,-27.33,-40.12,-34.03,-22.15,-17.15,-19.9,-30.68,-33.08,-26.71,-17.71,-17.13,-27.43,-32.16,-31.62,-19.01,-10.04,-16.09,-25.91,-30.56,-22.25,-10.04,-9.81,-21.34,-26.46,-23.89,-9.25,-7.09,-12.8,-24.06,-22.42,-13.62</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B314" t="str">
+        <v>[L_17_标记]</v>
+      </c>
+      <c r="C314" t="str">
+        <v>a: 44.4ms -87.5uv b: 91.1ms 447.7uv</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B315" t="str">
+        <v>[R_18_名字]</v>
+      </c>
+      <c r="C315" t="str">
+        <v>FERG(18)_dOps</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B316" t="str">
+        <v>[R_18_放大器]</v>
+      </c>
+      <c r="C316" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B317" t="str">
+        <v>[R_18_闪光]</v>
+      </c>
+      <c r="C317" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B318" t="str">
+        <v>[R_18_闪光背景]</v>
+      </c>
+      <c r="C318" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B319" t="str">
+        <v>[R_18_采样]</v>
+      </c>
+      <c r="C319" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B320" t="str">
+        <v>[R_18_分析时间]</v>
+      </c>
+      <c r="C320" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B321" t="str">
+        <v>[R_18_数据长度]</v>
+      </c>
+      <c r="C321" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B322" t="str">
+        <v>[R_18_详细数据(uv)]</v>
+      </c>
+      <c r="C322" t="str">
+        <v>-2.6,1.57,2.15,-1.2,-7.14,-13.29,-17.15,-17.14,-13.31,-7.28,-1.58,1.41,0.48,-3.98,-10.14,-15.33,-17.43,-15.49,-10.29,-3.92,1.04,2.59,0.12,-5.26,-11.25,-15.31,-15.61,-12.08,-5.93,0.22,3.95,3.95,0.18,-5.54,-10.76,-13.14,-11.5,-6.37,0.37,5.83,8.46,6.49,1.76,-4.23,-9.01,-10.08,-7.25,-1.8,4.13,7.89,7.89,3.69,-2.42,-9.07,-12.58,-12.25,-8.31,-1.7,3.68,6.48,5.56,1.33,-4.31,-8.51,-10.08,-7.29,-0.63,5.7,9.65,11.43,7.46,1.26,-6.3,-11.92,-13.71,-11.66,-7.78,-3.38,-3.04,-6.31,-9.81,-17.36,-24.1,-25.98,-22.89,-17.81,-9.75,-2.89,0.82,1.43,-1.95,-6,-6.23,-5.75,-2.95,4.94,6.71,11.81,6.41,0.4,-8.39,-18.04,-25.04,-27,-27.65,-26.01,-21.45,-19.7,-20.66,-23.8,-27.47,-34.03,-28.44,-20.52,-10.13,2.09,11.27,19.91,17.13,19.04,12.67,12.9,11.94,13.97,12.71,11.77,11.74,3.76,-6.75,-19.56,-32.38,-37.52,-34.75,-32.81,-23.79,-26.33,-23.12,-17.16,-19.53,-17.31,-14.65,-8.04,1.13,15.89,22.66,36.9,29.42,33.48,20.67,12.1,2.83,3.09,1.65,0.45,-1.4,-7.85,-12.9,-24.5,-38.4,-36.97,-44.14,-37.8,-28.73,-21.19,-12.39,-8.84,-6.92,-7.26,-9.25,-7.99,-5.48,4.45,11.21,16.08,17.43,12.5,5.61,-5.56,-14.22,-19.86,-21.65,-19.9,-17.47,-17.68,-17.63,-19.95,-29.38,-35.87,-37.05,-34.98,-25.78,-17.7,-9.17,-3.05,-1.49,-3.73,-8.68,-10.54,-12.9,-11.21,-7.01,-0.53,2.55,2.95,-0.29,-8.15,-15.56,-21.27,-22.63,-20.15,-13.69,-8.21,-5.45,-5.54,-8.67,-13.68,-18.42,-19.49,-16.79,-10.79,-3.42,2.65,5.1,3.68,-1.77,-7.6,-12.19,-13.06,-10.95,-5.41,0.01,3.51,3.03,-1.18,-7.7,-13.68,-17.51,-16.79,-12.9,-6.8,-1.23,1.06,-0.59,-5.6,-11.9,-16.9,-18.66,-16.43,-11.15,-5.3,-1.17,-0.68,-4.28,-10.41,-16.83,-21.04,-21.36,-17.88,-12.21,-6.86,-4.21,-5.52,-10.36,-16.84,-22.43,-24.85,-23.25,-18.35,-12.28,-7.6,-6.3,-9.02,-14.62,-20.84,-25.11,-25.66,-22.29,-16.41,-10.42,-6.84,-7.1,-11.09,-17.11,-22.61,-25.27,-23.92,-19.06,-12.63,-7.22,-4.99,-6.78,-11.75,-17.72,-22.12,-23.01,-19.91,-13.99,-7.59,-3.26,-2.68,-5.98,-11.67,-17.27,-20.37,-19.56,-15.08,-8.7,-2.97,-0.19,-1.43,-6.11,-12.21,-17.15,-18.82,-16.48,-11.08,-4.82,-0.29,0.64,-2.41,-8.19,-14.31,-18.26,-18.44,-14.81,-8.93,-3.31,-0.35,-1.36,-6,-12.43,-18.1,-20.74,-19.38,-14.69,-8.75,-4.14,-2.92,-5.71,-11.51,-18.03,-22.71,-23.74,-20.85,-15.36,-9.69,-6.34,-6.83,-11.08,-17.46,-23.44,-26.66,-25.89,-21.55,-15.56,-10.48,-8.52,-10.57,-15.85,-22.22,-27.11,-28.51,-25.9,-20.38,-14.26,-10.09,-9.61,-13.01,-18.85,-24.7,-28.08,-27.55,-23.28,-16.99,-11.22,-8.29,-9.35,-13.87,-19.87,-24.78,-26.46,-24.1,-18.58,-12.08,-7.19,-5.82,-8.43,-13.83,-19.65,-23.36,-23.32,-19.43,-13.2,-7.12,-3.6,-4.03,-8.12,-14.11,-19.43,-21.79,-20.16,-15.16,-8.81,-3.72,-1.96,-4.25,-9.61,-15.83,-20.31,-21.22,-18.2,-12.53,-6.6,-2.94,-3.11,-7.11,-13.35,-19.32,-22.64,-22.02,-17.81,-11.88,-6.81,-4.81,-6.84,-12.19,-18.77,-23.97,-25.79,-23.59,-18.44,-12.6,-8.66,-8.37,-12,-18.17,-24.46,-28.38,-28.43,-24.7,-18.87,-13.46,-10.82,-12.15,-16.98,-23.39,-28.79,-31.02,-29.19,-24.13,-17.97,-13.3,-12.09,-14.85,-20.45,-26.55,-30.6,-30.92,-27.32,-21.28,-15.25,-11.68,-11.99,-15.99,-21.93,-27.28,-29.72,-28.14,-23.11,-16.61,-11.23,-9.1,-11,-16.01,-21.96,-26.24,-26.98,-23.74,-17.77,-11.43,-7.25,-6.85,-10.31,-16.09,-21.7,-24.72,-23.83,-19.31,-12.98,-7.41,-4.85,-6.34,-11.2,-17.41,-22.36,-23.98,-21.62,-16.24,-10.11,-5.8</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B323" t="str">
+        <v>[R_18_标记]</v>
+      </c>
+      <c r="C323" t="str">
+        <v>61.3uv</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B324" t="str">
+        <v>[L_18_名字]</v>
+      </c>
+      <c r="C324" t="str">
+        <v>FERG(18)_dOps</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B325" t="str">
+        <v>[L_18_放大器]</v>
+      </c>
+      <c r="C325" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B326" t="str">
+        <v>[L_18_闪光]</v>
+      </c>
+      <c r="C326" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B327" t="str">
+        <v>[L_18_闪光背景]</v>
+      </c>
+      <c r="C327" t="str">
+        <v>b背景光_关:0.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B328" t="str">
+        <v>[L_18_采样]</v>
+      </c>
+      <c r="C328" t="str">
+        <v>刺激间隔:15.0S</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B329" t="str">
+        <v>[L_18_分析时间]</v>
+      </c>
+      <c r="C329" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B330" t="str">
+        <v>[L_18_数据长度]</v>
+      </c>
+      <c r="C330" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B331" t="str">
+        <v>[L_18_详细数据(uv)]</v>
+      </c>
+      <c r="C331" t="str">
+        <v>-1.79,7.85,12.54,9.25,-0.23,-10.47,-15.62,-12.69,-3.66,6.09,10.67,7.23,-2.25,-12.26,-16.98,-13.6,-4.26,5.51,10.07,6.54,-2.79,-12.46,-16.46,-12.54,-2.53,7.55,12.17,8.84,-0.2,-9.43,-12.78,-8.31,1.84,12.11,16.22,12.38,3.1,-6.34,-9.92,-5.57,4.27,13.62,17.02,12.49,2.73,-6.61,-9.61,-4.59,5.92,15.39,19.59,15.59,6.7,-1.51,-3.45,2.66,13.22,22.75,27.32,22.49,12.66,3.21,-0.6,3.23,11.44,19.01,20.04,12.68,0.05,-10.19,-13.52,-8.99,0.62,8.82,10.92,5.63,-4.06,-11.08,-11.03,-2.62,9.41,19.7,24.48,22.15,12.44,0.54,1.37,5.92,13.13,17.81,17.11,7.09,-7.83,-20.88,-27.13,-25.55,-14.92,-7.1,-7.6,-18.41,-24.26,-34.58,-27.98,-18,-3.04,9.71,16.75,16.09,7.35,2.78,5.77,13.85,24.34,32.07,32.74,22.1,4.48,-8.28,-15.1,-15.63,-8.42,-4.87,-11.02,-15.41,-33.22,-42.31,-38.16,-28.91,-10.58,2.05,11.47,10.31,8.37,4.48,11.24,21.04,37.08,49.9,46.86,34.61,25.87,11.56,6.25,9.89,13.65,15.01,7.06,-2.66,-22.81,-27.42,-30.13,-21.41,-12.48,-5.06,1.68,-1.26,-7.58,-7.55,-0.79,12.52,26.87,36.03,36.88,31.47,19.73,8.72,7.42,12.69,17.99,19.53,14.28,0.59,-14.26,-23.46,-26.57,-21.14,-12.34,-6.38,-2.7,-13.52,-21.43,-24.72,-19.56,-7.71,5.22,13,14.83,7.53,-2.23,-9.54,-4.84,2.52,10.19,14.57,11.1,0.81,-11.63,-18.56,-17.29,-10.22,0.62,3.85,2.54,-6.54,-16.53,-20.16,-15.96,-5.75,6.03,12.21,10.44,2.35,-6.41,-9.59,-5.89,3.72,13.78,19.1,15.92,6.45,-3.59,-8.15,-4.95,4.39,14.07,18.2,14.61,5.16,-4.47,-8.25,-4.38,5.65,15.61,20.05,16.18,6.76,-2.58,-6.26,-2.02,7.71,17.15,20.81,16.37,6.25,-3.51,-7.38,-3.31,6.1,15.04,18,12.94,2.61,-7.2,-10.9,-6.56,3.01,11.83,14.47,9.17,-1.25,-10.83,-14.15,-9.49,0.16,8.87,11.29,5.72,-4.72,-14.08,-17.01,-12.01,-2.15,6.52,8.75,3.08,-7.26,-16.26,-18.68,-13.17,-3.02,5.73,7.9,2.2,-7.95,-16.52,-18.37,-12.33,-1.87,6.93,9.01,3.28,-6.72,-14.9,-16.24,-9.76,0.93,9.71,11.61,5.75,-4.18,-12.06,-12.99,-6.17,4.62,13.24,14.85,8.74,-1.24,-8.95,-9.6,-2.58,8.16,16.49,17.67,11.18,1.04,-6.62,-7.11,-0.03,10.55,18.46,19.11,12.16,1.77,-5.9,-6.31,0.78,11.13,18.58,18.66,11.24,0.6,-7.08,-7.4,-0.31,9.83,16.85,16.4,8.56,-2.26,-9.88,-10.02,-2.85,7.16,13.83,12.97,4.83,-6.04,-13.47,-13.32,-5.94,4.06,10.51,9.37,1.07,-9.71,-16.8,-16.22,-8.51,1.6,7.96,6.65,-1.68,-12.24,-18.88,-17.78,-9.65,0.65,6.98,5.59,-2.7,-12.98,-19.12,-17.45,-8.89,1.6,7.92,6.44,-1.82,-11.83,-17.5,-15.31,-6.36,4.26,10.47,8.84,0.54,-9.28,-14.57,-11.96,-2.75,7.87,13.86,11.94,3.48,-6.26,-11.3,-8.42,0.91,11.39,17.02,14.68,5.94,-3.86,-8.76,-5.72,3.59,13.8,18.96,16.1,6.99,-2.94,-7.79,-4.67,4.56,14.43,19.06,15.65,6.15,-3.92,-8.72,-5.53,3.62,13.16,17.29,13.37,3.53,-6.61,-11.29,-7.96,1.18,10.48,14.19,9.87,-0.19,-10.29,-14.73,-11.13,-1.88,7.29,10.72,6.13,-4,-13.91,-17.96,-13.97,-4.5,4.67,7.94,3.22,-6.86,-16.45,-20,-15.52,-5.72,3.52,6.71,1.93,-8.01,-17.21,-20.22,-15.2,-5.07,4.27,7.39,2.55,-7.25,-16.08,-18.56,-13.05,-2.63,6.74,9.72,4.77,-4.97,-13.5,-15.54,-9.65,0.94,10.21,12.94,7.75,-2.03,-10.38,-12.12,-5.98,4.63,13.67,16,10.45,0.49,-7.8,-9.36,-3.11,7.39,16.07,17.89,11.88,1.66,-6.67</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B332" t="str">
+        <v>[L_18_标记]</v>
+      </c>
+      <c r="C332" t="str">
+        <v>63uv</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B333" t="str">
+        <v>[R_19_名字]</v>
+      </c>
+      <c r="C333" t="str">
+        <v>FERG(19)_lCone</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B334" t="str">
+        <v>[R_19_放大器]</v>
+      </c>
+      <c r="C334" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B335" t="str">
+        <v>[R_19_闪光]</v>
+      </c>
+      <c r="C335" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B336" t="str">
+        <v>[R_19_闪光背景]</v>
+      </c>
+      <c r="C336" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B337" t="str">
+        <v>[R_19_采样]</v>
+      </c>
+      <c r="C337" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B338" t="str">
+        <v>[R_19_分析时间]</v>
+      </c>
+      <c r="C338" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B339" t="str">
+        <v>[R_19_数据长度]</v>
+      </c>
+      <c r="C339" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B340" t="str">
+        <v>[R_19_详细数据(uv)]</v>
+      </c>
+      <c r="C340" t="str">
+        <v>-6.66,-7.39,-7.42,-6.74,-5.4,-3.5,-1.17,1.41,4.03,6.51,8.66,10.31,11.36,11.73,11.42,10.47,8.97,7.07,4.94,2.78,0.77,-0.89,-2.05,-2.6,-2.48,-1.68,-0.24,1.73,4.1,6.67,9.26,11.66,13.71,15.23,16.11,16.29,15.76,14.57,12.83,10.66,8.24,5.78,3.47,1.5,0.01,-0.9,-1.1,-0.67,0.4,1.98,3.94,6.07,8.24,10.23,11.86,12.84,13.35,13.04,12.11,10.37,8.37,5.64,2.96,-0.31,-2.58,-5.15,-7.01,-8.31,-8.65,-8.52,-7.84,-6.72,-5.61,-4.35,-1.98,-0.4,1.65,1.53,1.76,0.24,-1.39,-3.86,-7.51,-7.1,-10.96,-14.76,-20.64,-20.14,-23.5,-26.86,-25.44,-22.17,-23.81,-22.56,-17.5,-21.15,-15.61,-14.83,-7.51,-11.19,-8.66,-6.06,-5.16,-11.76,-9.33,-9.91,-12.11,-11.07,-11.9,-19.53,-18.14,-18,-12.92,-10.54,-5.14,-1.98,5.24,8.36,10.74,11.55,18.87,25.41,32.76,30.84,29.24,38.48,32.2,36.41,36.9,36.56,35.49,34.1,39.77,41.64,46.34,47.76,51.88,47.39,66.88,59.23,64.94,77.52,75.51,72.3,83.71,77.36,87.69,94.02,93.05,87.35,76.89,90.13,94.74,96.23,85.89,84.64,102.43,84.07,96.2,90.76,100.43,109.17,106.52,104.55,108.79,105.44,133.9,104.81,121.4,110.46,118.29,112.14,119.49,127.23,116.77,104.62,102.45,108.06,111.98,108.98,96.89,95.27,94.72,114.24,104.97,126.78,106.46,123.74,102.72,114.19,95.52,97.04,100.69,108.86,87.57,78.58,79.41,90.92,78.41,84.19,63.94,73.46,76.54,73.36,78.43,65.3,71.99,80.62,69.26,71.47,63.46,64.44,65.96,58.32,53.11,56.74,51.32,39.58,43.03,33.62,32.73,32.8,25.21,28.76,29.02,24.34,28.54,30.14,30.85,30.33,32.64,32.84,29.9,25.74,23.55,21.76,17.73,15.3,14.1,7.88,6,3.69,1.4,0.24,-1.38,-1.27,0.2,0.65,1.97,3.78,5.09,6.46,7.27,7.61,8.12,7.63,7.35,4.79,2.5,0.37,-2.82,-5.62,-7.35,-9.73,-10.64,-11.88,-11.43,-11.65,-10.35,-8.09,-5.81,-2.37,0.03,0.67,2.55,5.06,5.79,3.88,4.27,2.49,0.54,-1.3,-3.01,-5.62,-9.4,-8.65,-11.99,-11.4,-10.02,-10.16,-7.99,-5.09,-3.9,-1.33,-0.21,4.46,3.55,6.65,7.59,7.32,6.53,3.91,0.85,-0.69,-2.1,-8.29,-9.4,-11.34,-11.32,-13.63,-14.07,-11.18,-13.36,-8.79,-6.65,-6.89,-6.6,-2.22,-2.29,-1.81,2.62,0.5,0.01,-5.21,-6.59,-6.63,-11.25,-14.7,-17.71,-21.67,-19.53,-24.23,-22.7,-23.19,-21.57,-18.94,-16.84,-13.85,-14.71,-14.34,-13.56,-12.32,-12.05,-13.83,-14.1,-11.03,-14.69,-19.44,-23.19,-28.19,-25.91,-24.92,-28,-26.55,-26.5,-31.92,-30.27,-28.78,-23.83,-23.76,-18.67,-18.17,-17.89,-8.18,-14.88,-14.33,-10.73,-11.51,-13.81,-17.87,-15.44,-25.08,-26.54,-22.27,-31.57,-30.22,-22.22,-22.93,-18.11,-16.63,-18.57,-11.31,-18.4,-12.56,-9.84,-4.3,-9.37,-6.94,-7.55,-11.43,-12.52,-16.12,-16.13,-23.28,-15.72,-19.59,-21.44,-18.87,-27.39,-26.66,-17.24,-22.64,-12,-18.5,-16.04,-7.58,-9.48,-9.6,-2.03,-7.95,-3.75,-6.49,-8.18,-11.04,-14.6,-19.23,-18.35,-21.23,-22.7,-26.51,-25.26,-26.78,-18.78,-19.62,-21.45,-17.65,-16.36,-10.73,-10.36,-11.18,-8.01,-7.21,-8.49,-11.07,-14.96,-14.42,-19.03,-21.6,-23.17,-25.09,-25.63,-25,-22.87,-21.77,-16.81,-14.35,-15.5,-11.87,-7.41,-5.54,-2.69,-1.84,-3.38,-3.49,-4.86,-2.48,-4.12,-5.81,-9.4,-11.14,-13.25,-13.19,-15.2,-13.4,-14.97,-10.59,-10.32,-8.8,-5.15,-1.19,1.79,2.81,5.18,6.68,6.69,5.93,5.96,3.78,2.15,-0.17,-1.73,-3.78,-5.72,-6.7,-8.29,-8.38,-8.57,-7.32,-6.06,-3.4,-1.86,0.48,3.53,5.65,6.18,7.16,7.53,6.47,5.78,4.26</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B341" t="str">
+        <v>[R_19_标记]</v>
+      </c>
+      <c r="C341" t="str">
+        <v>a: 47.5ms -14.0uv b: 99.4ms 39.7uv</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B342" t="str">
+        <v>[L_19_名字]</v>
+      </c>
+      <c r="C342" t="str">
+        <v>FERG(19)_lCone</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B343" t="str">
+        <v>[L_19_放大器]</v>
+      </c>
+      <c r="C343" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B344" t="str">
+        <v>[L_19_闪光]</v>
+      </c>
+      <c r="C344" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B345" t="str">
+        <v>[L_19_闪光背景]</v>
+      </c>
+      <c r="C345" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B346" t="str">
+        <v>[L_19_采样]</v>
+      </c>
+      <c r="C346" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B347" t="str">
+        <v>[L_19_分析时间]</v>
+      </c>
+      <c r="C347" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B348" t="str">
+        <v>[L_19_数据长度]</v>
+      </c>
+      <c r="C348" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B349" t="str">
+        <v>[L_19_详细数据(uv)]</v>
+      </c>
+      <c r="C349" t="str">
+        <v>-12.78,-15.33,-15.97,-14.6,-11.45,-7.06,-2.18,2.37,5.81,7.57,7.37,5.28,1.7,-2.72,-7.17,-10.84,-13.05,-13.36,-11.68,-8.24,-3.59,1.53,6.27,9.87,11.77,11.68,9.68,6.17,1.8,-2.61,-6.25,-8.46,-8.79,-7.15,-3.78,0.76,5.72,10.27,13.65,15.3,14.94,12.63,8.82,4.12,-0.6,-4.59,-7.19,-7.87,-6.66,-3.71,0.39,4.84,9.06,11.69,12.67,11.62,8.73,4.47,-0.73,-5.95,-11.24,-14.21,-15.13,-15.51,-12.28,-9.7,-6.01,-2.04,-0.24,0.6,-1.22,-7.61,-13.21,-16.23,-22.23,-28.84,-30.47,-32.78,-33.28,-30.05,-29.52,-26.41,-18.31,-17.48,-20.5,-23.15,-19.4,-27.52,-32.3,-31.89,-40.89,-39.53,-43.14,-39.85,-33.94,-29.36,-19.8,-20.3,-10.59,-11.28,-7.25,-5.77,-8.51,-14.79,-17.84,-15.61,-14.3,-15.45,-8.01,-1.15,3.78,7.52,14.71,25.56,29.72,24.34,27.96,26.02,27.05,23.01,19.81,23.14,29.75,24.25,35.93,38.01,56.29,61.84,63.81,71.61,68.18,76.46,64.01,72.91,64.01,64.32,62.42,67.35,72.78,87.4,84.6,95.61,90.67,105.32,100.27,100.98,99.25,99.71,110.07,99.04,86.28,101.87,104.34,95.63,88.76,114.67,96.79,120.83,109.71,113.35,105.57,104.42,101.65,88.01,103.55,104.49,82.82,88.53,77.03,89.63,90.63,88.68,96.01,87.29,83.45,102.11,74.91,88.47,74.61,67.65,67.02,47.71,56.07,53.18,54.65,46.3,60.01,63.94,61.27,59.24,58.33,48.9,41.27,33.4,21.58,24.31,20.07,13.61,15.88,14.54,17.84,21.81,28.66,25.94,26.49,24.29,22.91,13.52,11.71,5.39,-1.43,-4.5,-5.15,-3.87,-1.06,1.89,6.75,9.67,12.87,12.93,11.2,9.25,4.1,-1.14,-6.77,-9.97,-13.16,-13.45,-12.42,-9.5,-5.41,-1.38,2.45,4.73,5.38,4.5,0.92,-3.69,-8.96,-13.65,-18.72,-21.08,-21.25,-19.83,-17.09,-13.68,-9.76,-5.79,-2.69,-2.55,-4.33,-7.24,-12.15,-16.02,-20.92,-26.24,-28.88,-28.1,-27.43,-23.85,-20.46,-16.32,-10.74,-8.68,-9.05,-8.1,-13.05,-16.3,-20.77,-24.9,-29.83,-30.32,-31.01,-29.3,-27.89,-20.79,-18.74,-12.16,-8.9,-8.77,-8.34,-10.58,-16.48,-18.99,-24.95,-29.44,-31.03,-28.61,-28.8,-24.99,-19.86,-16.24,-9.72,-6.56,-9.5,-6.13,-8.27,-16.3,-17.45,-21.61,-25.99,-30.69,-31.36,-27.71,-23.31,-23.1,-14.27,-12.63,-6.39,-6.24,-6.49,-12,-18.13,-22.62,-27.24,-28.55,-34.95,-29.95,-28.45,-25.07,-26.28,-21.75,-18.5,-12.41,-11.99,-19.06,-15.98,-19.48,-25.57,-36,-41.11,-38.86,-40.79,-39.17,-40.58,-31.81,-28.16,-28.9,-26.3,-19.3,-23.76,-30.69,-34.28,-39.41,-37.8,-48.55,-52.79,-48.53,-48.39,-39.48,-37.38,-38.2,-30.36,-26.62,-30.24,-25.19,-30.87,-30.1,-40.72,-45.74,-46.85,-52.55,-47.48,-49.93,-43.42,-41.39,-31.38,-24.6,-31.37,-23.53,-26.5,-32.82,-27.28,-41.01,-42.77,-47.65,-42.59,-47.58,-47.69,-37.53,-29.68,-29.08,-19.16,-22.01,-22.54,-21.7,-25.06,-26.28,-31.82,-31.7,-39.09,-40.1,-43.9,-33.73,-36.33,-25.17,-27.88,-17.04,-20.54,-18.9,-17.47,-23.27,-23.93,-27.93,-36.15,-34.21,-34.17,-36.55,-39.48,-33.61,-25.45,-21.2,-21.57,-15.51,-16.22,-17.65,-20.06,-22.71,-31.43,-34.03,-37.7,-40.58,-38.47,-39.33,-36.42,-31.87,-24.27,-22.37,-16.49,-18.88,-17.79,-22.07,-25.85,-32.96,-34.25,-39.95,-41.74,-40.68,-38.89,-37.49,-30.14,-25.25,-22.45,-17.86,-16.81,-18.89,-20.39,-27.47,-29.08,-35.6,-37.49,-40.29,-39.06,-35.73,-33.39,-27.68,-22.8,-18.11,-13.54,-14.06,-13.46,-16.61,-20.22,-24.13,-28.07,-32.16,-32.78,-33,-30.59,-26.47,-21.33,-15.9,-10.43,-8.1,-7.52,-8.01,-10.23,-14.38,-18.6,-23.62,-26.06,-27.78,-27.19,-25.16,-21.5,-17.12,-12.15,-8.15,-5.13,-4.35,-5.57,-9.46,-13.14,-18.79,-22.86,-26.49,-28.35,-28.54,-26.6,-23.67</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B350" t="str">
+        <v>[L_19_标记]</v>
+      </c>
+      <c r="C350" t="str">
+        <v>a: 47.5ms -10.5uv b: 99.3ms 54.4uv</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B351" t="str">
+        <v>[R_20_名字]</v>
+      </c>
+      <c r="C351" t="str">
+        <v>FERG(20)_lFlicker</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B352" t="str">
+        <v>[R_20_放大器]</v>
+      </c>
+      <c r="C352" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B353" t="str">
+        <v>[R_20_闪光]</v>
+      </c>
+      <c r="C353" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B354" t="str">
+        <v>[R_20_闪光背景]</v>
+      </c>
+      <c r="C354" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B355" t="str">
+        <v>[R_20_采样]</v>
+      </c>
+      <c r="C355" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B356" t="str">
+        <v>[R_20_分析时间]</v>
+      </c>
+      <c r="C356" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B357" t="str">
+        <v>[R_20_数据长度]</v>
+      </c>
+      <c r="C357" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B358" t="str">
+        <v>[R_20_详细数据(uv)]</v>
+      </c>
+      <c r="C358" t="str">
+        <v>12.33,13.17,11.75,11.61,11.62,12.92,11.11,13.42,11.38,11.26,11.94,10.13,16.01,13.04,13.28,14.77,13.86,15.22,13.89,17.94,15.88,17.59,20.46,18.67,24.39,24.99,20.32,23.17,22.33,26.9,29.36,29.45,26.61,29.34,29.82,30.5,29.68,29.95,29.24,29.38,27.9,28.29,28.55,29.59,28.02,27.54,27.13,26.41,23.15,21.98,21.22,18.34,16.91,15.42,13.9,11.92,9.67,6.93,5.98,3.28,-0.35,-3.06,-4.92,-6.11,-8.37,-13.32,-13.89,-16.85,-19.72,-20.38,-23.63,-23.57,-25.16,-27.83,-25.31,-30.78,-29.56,-31.74,-31.85,-32.17,-32.35,-35.03,-37.75,-31.57,-36.64,-32.23,-35.06,-33.08,-33.96,-29.99,-28.68,-27.78,-28.66,-27.32,-26.49,-25.65,-18.8,-18.51,-18.35,-16,-13.26,-10.24,-9.77,-7.74,-4.69,-6.39,-3.91,-2.02,3.09,3.12,6.11,7.97,6.74,9.9,11.29,11.75,14.32,14.56,15.42,16.51,17.22,18.52,19.1,18.58,20.47,20.14,20.04,18.25,18.9,18.35,20.62,20.77,21.17,20.65,22.08,16.3,22.31,19.84,21.92,18.17,16.26,17.17,18.11,17.87,17.72,17.81,17.06,18.24,17.69,13.24,12.4,13.03,17.14,15,11.2,15.18,9.91,12.68,13.98,12,13.85,7.99,7.81,10.11,11.64,8.65,8.58,5.66,8.84,7.18,8.37,5.68,2.79,3.56,3.58,3.26,1.75,-0.44,-0.28,-1.32,-3.08,-4.32,-4.83,-5.45,-7.41,-7.83,-9.06,-10.61,-11.06,-12.34,-13.5,-12.56,-15.52,-16.06,-16.87,-14.7,-17.71,-15.19,-18.23,-17.3,-21.87,-16.02,-19.85,-22.26,-22.86,-19.18,-24.01,-20.09,-18.74,-18.9,-22.27,-20.4,-20.77,-19.46,-18.79,-18.82,-21.92,-18.84,-18.2,-18.02,-19.99,-16.13,-19.01,-19.65,-18.85,-17.94,-15.07,-15.81,-16.59,-13.55,-13.8,-12.74,-13.1,-13.03,-11.33,-12.36,-12.21,-11.21,-11.66,-10.02,-10.62,-9.27,-9.98,-9.54,-8.57,-8.48,-8.06,-7.16,-4.67,-4.36,-2.89,-2.3,-1.41,-2.01,0.13,0.91,3.53,4.01,2.41,6.37,9,7.7,8.36,12.23,14.1,11.64,15.21,17.14,16.21,17.16,16.54,22.78,18.83,19.53,23.25,22.64,22.42,27.52,27.94,24.99,27.97,28.91,25.12,28.47,24.44,25.37,24.55,25.7,22.1,20.45,22.29,19.74,18.31,17.22,15.54,14.88,11.7,9.89,7.18,6.52,4.89,1.67,-1.34,-2.99,-5.67,-8.27,-10.94,-13.98,-16.15,-17.95,-22.07,-22.9,-24.6,-28.66,-29.87,-32.56,-34.9,-33.01,-36.37,-38.43,-38.46,-43,-42.99,-41.53,-43.1,-45.75,-43.96,-45.81,-45.84,-42.13,-40.22,-43.79,-43.42,-40.81,-42.04,-40.15,-36.86,-34.99,-34.32,-32.37,-28.95,-29.53,-28.78,-27.94,-26.2,-19.8,-17.96,-17.31,-18.7,-12.09,-12.58,-8.81,-10.29,-8.92,-6.91,-5.63,-6.61,-3.64,-1.37,0.31,-0.7,0.4,-0.41,1.67,2.12,0.44,2.22,1.97,1.89,2.66,1.95,2.15,1.38,1.56,1.62,1.01,0.9,0.4,0.13,-1.33,0.09,0.56,1.56,-1.8,0.09,-0.26,-1.29,0.6,-0.38,-3.26,3.7,0.96,3.14,3.71,1.37,1.57,3.79,3.99,0.32,5.51,4.74,7.16,9.13,7.81,4.93,5.08,6.15,7.14,7.96,10.97,11.23,8.01,8.83,12.72,10.66,9.49,10.59,9.11,9.41,8.37,8.5,7.62,5.97,3.88,3.14,0.98,0.72,-1.3,-2.1,-4.92,-6.51,-7.68,-10.73,-12.27,-14.25,-15.86,-18.3,-19.42,-22.77,-25.85,-25.98,-28.8,-27.73,-34.18,-34.87,-38.36,-36,-36.08,-40.43,-41.53,-45.1,-44.26,-45.51,-45.61,-47.41,-44.15,-43.61,-46.28,-46.75,-44.44,-42.62,-41.92,-45.61,-40.84,-42.39,-37.62,-42.28,-36.37,-39.57,-37.07,-32.25,-33.13,-29.77,-29.12,-29.86,-26.24,-22.81,-21.66,-20.25,-21.16,-18.44,-15.79,-14.47,-13.09,-10.79,-10.14,-8.25,-7.85,-6.85,-7.45,-4.97,-4.64,-3.37,-2.64,-2.5,-2.61,-0.6,-0.82,0.31,1.16</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B359" t="str">
+        <v>[R_20_标记]</v>
+      </c>
+      <c r="C359" t="str">
+        <v>幅值: 23uv 相位: 48°</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B360" t="str">
+        <v>[L_20_名字]</v>
+      </c>
+      <c r="C360" t="str">
+        <v>FERG(20)_lFlicker</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B361" t="str">
+        <v>[L_20_放大器]</v>
+      </c>
+      <c r="C361" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B362" t="str">
+        <v>[L_20_闪光]</v>
+      </c>
+      <c r="C362" t="str">
+        <v>b白色光:600.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B363" t="str">
+        <v>[L_20_闪光背景]</v>
+      </c>
+      <c r="C363" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B364" t="str">
+        <v>[L_20_采样]</v>
+      </c>
+      <c r="C364" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B365" t="str">
+        <v>[L_20_分析时间]</v>
+      </c>
+      <c r="C365" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B366" t="str">
+        <v>[L_20_数据长度]</v>
+      </c>
+      <c r="C366" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B367" t="str">
+        <v>[L_20_详细数据(uv)]</v>
+      </c>
+      <c r="C367" t="str">
+        <v>1.14,4.54,3.56,5.66,9.2,11.6,9.76,13.39,15.45,14.71,18.49,17.89,19.42,18.75,23.71,24.4,21.78,27.26,21.54,26.99,21.86,25.29,29.65,30.27,26.43,25.1,25.91,26.22,25.85,25.2,20.69,23.81,18.72,21.7,21.28,15.97,16.49,15.13,14.19,10.84,9.55,9.69,7.3,6.15,2.61,2.14,0.74,-0.2,-3.83,-5.32,-6.74,-6.84,-9.71,-8.65,-10.33,-13.05,-13.07,-13.9,-13.93,-14.85,-15.49,-15.7,-18.63,-20.11,-16.92,-17.94,-20.71,-17.6,-20.08,-16.9,-18.51,-21.11,-16.52,-18.45,-20.3,-17.92,-18.39,-17.4,-14.24,-15.76,-16.04,-15.8,-15.2,-11.62,-9.7,-14,-14.41,-13.75,-14.26,-6.51,-9.28,-8.35,-7.16,-9.17,-5.8,-4.76,-9.33,-8.37,-8.59,-5.15,-7.3,-4.84,-4.96,-5.66,-5.12,-4.2,-4.1,-3.9,-3,-3.84,-3.29,-1.63,-1.4,-0.51,-1.1,1.34,2.99,1.19,4.03,6.32,4.05,6.04,7.44,7.06,11.65,11.1,13.47,13.77,14.8,14.91,17.76,19.32,17.52,18.42,23.29,22.4,22.58,22.96,23.07,25.16,27.99,29.9,27.62,29.66,30.82,30.32,27.75,30.48,27.94,29.11,26.47,30.37,27.95,23.6,27.74,23.76,20.36,20.76,22.53,20.67,16.76,17.67,15.5,15.6,12.64,11.7,9.3,8.15,6.35,4.97,4.11,2.19,0.44,-0.84,-0.74,-3.36,-4.03,-6.45,-5.67,-8.43,-7.47,-10.17,-8.89,-10.27,-7.72,-10.77,-11.85,-14.67,-13.51,-10.06,-13.15,-11.96,-12.77,-11.03,-9.66,-11.13,-11.72,-12.39,-8.51,-7.94,-6.8,-8.28,-9.53,-9.88,-7.57,-3.55,-3.28,-6.54,-3.56,-4.67,-3.65,-3.89,-1.71,-2.33,0.26,-2.27,-3.99,-3.17,0.48,-1.9,0.66,-2.69,-1.8,-1.87,-0.49,-1.06,-1.17,-1.24,0.71,0.49,-0.38,0.03,0.19,1.03,1.43,0.6,1.36,3.02,1.28,2.48,5.57,5.15,3.99,4.32,7.14,8.37,7.55,10.39,11.87,9.12,12.05,16.23,17.76,17.79,19.46,22.82,21.88,22.79,24.16,25.04,28.05,24.99,30.75,28.58,28.62,33.43,32.21,32.1,29.3,35.88,30.22,33,35.28,31.04,34.34,32.63,33.69,36.03,34.34,32.79,30.54,29.75,32.43,28.65,28.32,24.97,26.36,24.11,21.67,22.01,18.63,18.09,15.63,15.02,13.18,12,9.37,8.09,6.83,4.76,3,3.79,0.69,1.6,-0.19,-0.18,-3.96,-2.51,-4.6,-4.3,-7.69,-7.95,-6.9,-5.35,-9.1,-8.03,-7.11,-5.84,-5.9,-6.55,-5.21,-5.91,-3.74,-6.69,-2.33,-3.68,-6.12,-2.32,-2.97,-6.13,-5.28,-2.98,-2.88,-1.45,-0.34,-1.13,-3.46,1.94,1.49,-2.58,3.74,4,-0.41,1.41,3,1.2,3.67,2.72,1.27,3.02,1.85,4.26,2.53,3.92,5.57,5.39,5.32,5.71,5.65,7.43,6.56,7.85,10.03,10.59,9.81,9.52,12.7,12.43,14.16,15.91,15.12,18.03,18.54,21.77,21.8,23.59,23.04,26.85,28.68,27.32,26.49,31.9,28.89,33.54,32.71,35.42,37.69,39.78,36.3,41.53,37.01,41.31,39.08,40.8,38.51,39.65,44.32,42.27,38.57,41.33,41.98,37.02,37.48,36.3,34.41,37.08,32.78,31.63,29.31,28.36,28.69,28.67,27.19,23,21.45,21.42,20,16.85,15.88,14.83,12.72,11.66,8.26,8.59,7,5.99,3.28,2.43,2.43,-1.65,0.45,-0.69,-2.01,0.12,-3.69,-1.6,-4.75,-4.59,-5.77,-2.07,-3.36,-2.71,-4.25,-2.99,-3.97,-2.08,-4.76,-3.58,1.33,-0.04,-0.96,-0.57,1.03,-0.4,2.2,3.77,1.58,3.73,8.95,7.27,3.76,6.81,12.17,8.3,7.62,7.51,12.56,10.52,8.55,9.28,11.43,10.96,9.03,12.21,13.8,11.92,11.67,13.36,13.66,13.5,12.77,13.33,13.29,14.1,13.51,13.98,15.06,15.5,16.34,16.82,17.09,20.25,18.74,19.56,18.84,19.51,22.84,24.91,22.59,24.72</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B368" t="str">
+        <v>[L_20_标记]</v>
+      </c>
+      <c r="C368" t="str">
+        <v>幅值: 23.5uv 相位: 49.6°</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B369" t="str">
+        <v>[R_21_名字]</v>
+      </c>
+      <c r="C369" t="str">
+        <v>FERG(21)_lCone</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B370" t="str">
+        <v>[R_21_放大器]</v>
+      </c>
+      <c r="C370" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B371" t="str">
+        <v>[R_21_闪光]</v>
+      </c>
+      <c r="C371" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B372" t="str">
+        <v>[R_21_闪光背景]</v>
+      </c>
+      <c r="C372" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B373" t="str">
+        <v>[R_21_采样]</v>
+      </c>
+      <c r="C373" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B374" t="str">
+        <v>[R_21_分析时间]</v>
+      </c>
+      <c r="C374" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B375" t="str">
+        <v>[R_21_数据长度]</v>
+      </c>
+      <c r="C375" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B376" t="str">
+        <v>[R_21_详细数据(uv)]</v>
+      </c>
+      <c r="C376" t="str">
+        <v>12.83,8.53,2.93,-2.79,-7.39,-9.91,-9.79,-7,-2.09,3.98,10,14.77,17.34,17.18,14.33,9.36,3.25,-2.77,-7.51,-10.04,-9.89,-7.13,-2.36,3.4,8.92,13.03,14.83,13.89,10.33,4.8,-1.66,-7.81,-12.5,-14.84,-14.44,-11.47,-6.61,-0.91,4.38,8.13,9.49,8.12,4.23,-1.47,-7.87,-13.74,-17.95,-19.7,-18.67,-15.12,-9.8,-3.82,1.59,5.3,6.57,5.11,1.22,-4.31,-10.33,-15.65,-19.13,-20.04,-18.22,-13.98,-8.08,-1.82,3.85,7.55,8.69,7.12,3.02,-2.26,-8.18,-13.39,-15.95,-16.59,-13.97,-10.05,-4.22,2.09,7.63,11.16,11.58,9.03,4.55,-2.11,-8.68,-12.92,-16.89,-18.43,-16.46,-11.1,-3.44,0.48,3.8,7.18,7.98,1.61,-1.59,-6.87,-17.01,-19.75,-23.73,-23.88,-23.3,-20.61,-9.58,-9.43,0.44,-2.43,-0.49,-2.57,-8.98,-15.31,-18.27,-27.2,-25.38,-24.27,-17.41,-13.32,-3.49,1.1,1.8,6.64,11.13,4.89,4.56,-2.7,-4.96,-7.82,-10.12,-1.91,2.32,9.73,20.74,26.6,29.65,32.7,34.13,34.61,25.45,30.79,23.36,21.32,21.54,22.39,35.94,44.54,59.61,67.22,63.1,63.91,64.71,65.41,58.2,55.99,66.77,68.87,66.42,72.74,73.27,76.81,94.93,105.66,91.73,96.63,115.05,92.71,96.92,84.91,90.59,81.4,91.34,109.96,95.07,123.55,125.36,137.27,136.64,136.97,126.16,125.46,128.16,119.33,115.47,97.56,95.27,93.18,114.69,111.17,118.76,108.6,127.7,115.04,116.85,110.62,94.99,85.58,80.24,89.17,80.08,88.07,92.22,97.03,91.22,84.29,99.35,82.31,84.86,81.93,66.03,52.81,44.98,49.19,54.52,55.77,44.34,61.31,52.63,63.31,57.61,54.68,46.57,43.06,30.08,26.24,21.7,16.28,12.75,16.87,22.56,26.64,30.07,31.09,33.9,29.01,23.23,19.64,10.33,3.83,0.01,-2.67,0.96,3.4,8.38,14.85,19.51,22.23,21.31,19.69,15.62,9.69,3.55,-1.71,-4.3,-6.26,-2.79,1.84,7.25,13.67,18.9,21.4,21.55,19.17,14.94,9.54,3.07,-1.31,-4.01,-4.42,-1.73,3.36,9.15,14.78,20.1,22.52,22.56,19.3,14.44,7.99,1.15,-2.77,-6.07,-6.02,-2.36,2.11,8.33,12.79,18.02,19.14,17.81,14.73,8.78,0.79,-3.57,-9.03,-10.81,-11.48,-7.9,-3.39,1.44,7.19,9.13,10.28,10.82,5.92,0.11,-7.65,-13.37,-18.88,-20.35,-19.73,-14.03,-9.07,-4.76,2.52,2.63,2.96,1.32,1.64,-5.69,-12.45,-16.51,-19.77,-25.61,-20.77,-16.47,-13.73,-4.44,-1.49,4.13,3.93,4.88,-0.94,-5.11,-12.9,-16.68,-19.16,-18.91,-20.93,-12.05,-7.11,-2.78,5.52,4.14,3.61,3.86,3.69,-1.72,-11.42,-13.19,-14.23,-16.57,-15.23,-13.04,-0.06,-1.26,8.24,9.58,9.1,7.59,4,-2.2,-11.43,-14.97,-17.84,-12.78,-12.54,-8.22,-4.89,5.9,8.97,9.63,9.75,0.37,2.14,-4.39,-11.96,-16.73,-23.7,-15.54,-22.12,-12.67,-7.34,2.91,2.5,1.6,1.17,1.1,-6.35,-17.46,-23.25,-21.74,-24.31,-20.69,-23.8,-14.63,-10.9,-5.18,-0.1,-4.18,-3.99,-4.02,-9.82,-14.16,-27.16,-30.09,-26.49,-25.29,-24.53,-17.94,-10.97,-2.11,-0.11,0.51,-5.25,-0.76,-8.82,-15.12,-17.98,-21.79,-24.88,-24.93,-16.6,-7.53,-2.44,3.65,9.07,4.76,5.67,3.88,-2.72,-5.7,-12.49,-13.16,-16.13,-9.88,-3.69,-3.75,7.95,10.98,16.75,16.59,13.27,7.63,2.27,-2.18,-4.82,-10.52,-4.96,-3.62,3.32,7.16,13.13,17.6,22.34,20.27,18.31,12.14,7.2,0.59,-4.97,-3.9,-4.4,-2.63,4.73,8.92,13.5,19.3,19.24,19.13,16.94,11.35,5.21,-1.72,-5.25,-8.27,-7.75,-5.44,1.25,7.41,11.19,16.61,17.84,15.23,11.69,5.4,-0.64,-5.42,-9.53,-11.89,-10.13,-5.68,0.06,5.5,10.79,14.23,15.73,14.29,11.27</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B377" t="str">
+        <v>[R_21_标记]</v>
+      </c>
+      <c r="C377" t="str">
+        <v>a: 50.4ms -9.4uv b: 105.8ms 79.1uv</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B378" t="str">
+        <v>[L_21_名字]</v>
+      </c>
+      <c r="C378" t="str">
+        <v>FERG(21)_lCone</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B379" t="str">
+        <v>[L_21_放大器]</v>
+      </c>
+      <c r="C379" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B380" t="str">
+        <v>[L_21_闪光]</v>
+      </c>
+      <c r="C380" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B381" t="str">
+        <v>[L_21_闪光背景]</v>
+      </c>
+      <c r="C381" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B382" t="str">
+        <v>[L_21_采样]</v>
+      </c>
+      <c r="C382" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B383" t="str">
+        <v>[L_21_分析时间]</v>
+      </c>
+      <c r="C383" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B384" t="str">
+        <v>[L_21_数据长度]</v>
+      </c>
+      <c r="C384" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B385" t="str">
+        <v>[L_21_详细数据(uv)]</v>
+      </c>
+      <c r="C385" t="str">
+        <v>9.88,14.73,19.65,24.17,27.87,30.41,31.57,31.25,29.51,26.56,22.73,18.41,14.08,10.19,7.14,5.26,4.75,5.65,7.87,11.19,15.27,19.66,23.92,27.59,30.28,31.69,31.66,30.15,27.31,23.38,18.72,13.79,9.04,4.92,1.81,-0.02,-0.41,0.6,2.91,6.2,10.09,14.15,17.93,20.94,22.94,23.56,22.75,20.65,17.1,12.73,8.04,3.12,-1.43,-5.28,-7.99,-8.97,-8.95,-7.13,-4.41,-0.63,3.58,8.36,11.4,14.03,16.35,16.7,15.13,12.39,7.73,2.66,-2.34,-6,-9.47,-13.82,-16.15,-14.74,-14.02,-10.27,-9.96,-3.29,0.18,1.99,7.84,7.67,8.52,10.51,11.81,5.58,4.64,-1.08,-1.7,-12.63,-8.64,-11.56,-13.66,-15.99,-8.98,-7.75,0.38,5.62,5.04,15.13,20.8,22.73,24.75,26.31,23.71,22.1,22.36,17.17,19.82,16.66,11.32,16.76,12.17,23.88,24.45,27.37,40.28,36.18,45.56,54.51,59.29,59.22,62.52,63.93,62.7,60.11,55.7,57.89,53.76,57,59.01,55.36,61.83,68.9,62.83,73.44,76.13,92.16,94.98,100.88,96.53,105.28,99.02,96.51,111.13,89.1,96.73,91.08,98.39,90.26,91.37,81.24,96.22,112.54,98.18,112.1,109.15,126.35,118.69,125.04,140.55,120.53,119.48,144.75,133.42,126.33,130.25,121.86,99.56,119.99,107.94,109.77,103.49,107.93,114.4,124.22,112.07,119.32,123.87,118.4,134.89,125.84,120.72,115.1,120.83,100.04,92.88,102.58,82.94,76.83,74.28,77.41,76.58,68.29,74.07,86.15,87.44,78.19,80.82,88.39,88.51,77.4,79.66,67.33,63.55,59.57,51.35,46.37,42.77,36.85,31.69,35.25,35,29.13,38.47,36.83,42.35,41.85,45.91,42.02,41.66,39.32,33.62,29.84,21.94,17.44,13.84,9.61,3.7,1.42,1.15,0.91,5.01,7.01,10.01,14.78,18.92,21.58,23.93,23.8,23.29,20.75,17.64,13.1,9.12,4.08,0.44,-3.33,-4.73,-6.08,-4.14,-1.57,1.05,5.71,10.16,15.03,18.89,22.92,23.72,24.46,24.11,21.71,19.31,15.34,11.25,6.03,3.59,-0.51,-0.52,-1.28,0.23,2.47,6.37,11.87,16.16,19.31,25.3,28.01,28.8,26.96,24.19,22.23,18.03,12.74,10.59,6,0.46,-3.31,-1.53,-4.42,-0.7,1.48,5.66,8.18,13.44,13.92,16.55,19.7,19.31,16.04,17.64,10.2,8.75,0.58,-3.46,-9.57,-11.78,-14.67,-17.64,-14.81,-13.88,-9.83,-4.62,-1.39,2,5.1,9.37,6.93,10.98,9.61,5.5,-2.02,-4.63,-9.99,-12.89,-16.13,-17.87,-24.75,-21.44,-19.8,-16.21,-12.3,-6.3,-5.17,-1.91,5.65,1.38,5.89,3.79,5.45,1.36,-0.89,-7.51,-13.34,-11.05,-20.27,-21.88,-21.79,-20.45,-17.08,-8.79,-11.13,-3.79,3.68,9.72,14.83,12.64,8.19,11,11.83,1.32,-2.47,1.26,-9.17,-5.11,-8.27,-10.32,-17.02,-11.46,-12.04,-7.95,3.06,6.92,1.93,14.24,15.23,13.3,10.41,11.12,10.56,5.81,-4.12,-8.35,-9.71,-10.79,-13.23,-21.43,-20.22,-16.75,-9.52,-7.83,-3.16,1.85,0.88,8.47,6.34,4.9,10.49,2.03,1.95,-2.41,-9.6,-16.44,-13.41,-19.12,-19.85,-22.83,-17.4,-18.36,-17.5,-13.41,-8.2,-2.8,4.14,2.47,9.72,5.54,5.02,6.17,2.08,-1.11,-10.68,-14.49,-17.17,-17.33,-14.85,-15.36,-15.94,-11.86,-7.36,-2.23,6.68,7.79,14.1,16.17,18.37,19.55,18.06,14.27,9.29,6.58,0.58,0.54,-3.77,-6.73,-4.43,-1.7,0.19,2.34,8.1,13.91,16.47,22.94,26.06,27.38,26.92,27.63,23.09,20.4,15.3,12.69,6.91,4.6,1.77,-0.88,-0.7,-0.07,3.66,6.7,10.94,16.28,19.78,22.2,24.3,24.94,24.64,22.82,19.36,15.21,9.95,5.6,0.69,-2.75,-5.75,-6.31,-6.02,-3.94,-1.51,2.29,7.14,10.42,14.86,17.81,19.26,19.67,18.16,16.11,12.3</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B386" t="str">
+        <v>[L_21_标记]</v>
+      </c>
+      <c r="C386" t="str">
+        <v>a: 50.4ms -12.9uv b: 105.7ms 32.9uv</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B387" t="str">
+        <v>[R_22_名字]</v>
+      </c>
+      <c r="C387" t="str">
+        <v>FERG(22)_lFlicker</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B388" t="str">
+        <v>[R_22_放大器]</v>
+      </c>
+      <c r="C388" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B389" t="str">
+        <v>[R_22_闪光]</v>
+      </c>
+      <c r="C389" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B390" t="str">
+        <v>[R_22_闪光背景]</v>
+      </c>
+      <c r="C390" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B391" t="str">
+        <v>[R_22_采样]</v>
+      </c>
+      <c r="C391" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B392" t="str">
+        <v>[R_22_分析时间]</v>
+      </c>
+      <c r="C392" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B393" t="str">
+        <v>[R_22_数据长度]</v>
+      </c>
+      <c r="C393" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B394" t="str">
+        <v>[R_22_详细数据(uv)]</v>
+      </c>
+      <c r="C394" t="str">
+        <v>23.13,21.77,24.46,30.58,37.99,35.36,26.74,24.05,22.06,19.35,31.17,34.57,35.78,28.57,27.38,16.89,18.13,26.39,33.47,36.7,36.49,31.25,22.08,21.35,18.67,29.06,32.62,34.35,33.73,25.59,19.63,18.54,23.17,26.36,33.68,30.67,28.04,20.49,13.96,13.59,16.54,21.38,24.97,23.06,14.28,6.97,5.14,4.23,8.46,13.39,14.06,8.92,-0.26,-5.17,-6.79,-4.33,-1.9,3.78,1.73,-5.44,-12.24,-18.55,-19.66,-13.88,-12.21,-8.74,-9.29,-15.28,-22.07,-27.92,-25.89,-20.29,-10.46,-12.84,-10.54,-24.79,-28.55,-23.18,-22.64,-9.61,-9.12,-11,-10.71,-16.93,-21.37,-14.76,-12.1,-1.8,1.46,-0.14,-2.71,-7.47,-6.83,-1.84,2.45,11.77,11.43,12.06,7.34,4.07,4.24,11.07,17.54,24.04,21.47,16.92,12.1,8.94,14.86,19.13,25.92,29.44,25.7,19.97,15.27,13.3,18.92,25.6,30.76,29.04,26.42,19.3,14.82,16.29,20.54,26.18,30.9,29.38,21.59,18.85,14.83,19.2,24.18,32.39,31.75,26.04,21.11,15.11,18.86,23.48,31.7,35.39,36.45,27.57,25.75,20.08,20.65,25.36,35.88,39.05,33.08,29.03,23.25,25.3,26.53,32.11,38.1,37.57,34.06,27.94,24.27,22.3,28.97,32.77,34.43,33.58,28.24,19.98,15.22,17.47,19.66,26.08,26.2,21.19,12.8,8.42,4.45,5.43,11.97,14.04,11.35,5.05,-5.17,-9.82,-11.81,-6.3,-0.43,0.43,-4.07,-7.85,-16.9,-23.07,-21.97,-14.54,-14.76,-8.36,-14.11,-23.52,-24,-25.51,-23.12,-19.2,-15.4,-14.68,-19.35,-26.85,-25,-26.69,-19.1,-12.29,-5.59,-9.34,-15.41,-16.55,-18.41,-14.74,-4.42,-0.6,4.81,0.81,-5.07,-6.35,-4.86,2.5,10.76,14.49,16.96,12.33,7.22,6.1,8.38,15.42,23,26.28,23.61,18.68,16.28,14.62,19.62,26.12,32.5,32.15,30.14,23.2,20.09,21.13,26.22,35.4,35.74,33.76,31.66,26.92,19.3,25.15,31.22,41.65,40.89,34.14,31.54,27.85,24.28,30.32,36.79,38.96,40.58,35.74,29.33,23.84,27.36,31.21,42.08,42.37,39.47,31.9,29.52,27.8,30.78,34.47,37.88,41.48,37.25,29.49,26.14,23.29,27.81,33.54,35.93,34.65,27.35,20.83,16.54,17.62,20.13,23.51,26.36,20.28,12.14,7.85,4.05,4.14,9.91,12.06,12.39,5.13,-2.01,-7.93,-9.53,-6.62,-1.07,-0.95,-6.1,-11.42,-20.46,-21.02,-21.88,-17.58,-12.91,-9.18,-13.02,-20.99,-25.76,-27.06,-20.5,-18.7,-12.88,-15.52,-16.28,-24.13,-25.92,-24.13,-19.66,-10.88,-4.88,-3.54,-11.6,-16.83,-13.92,-8.16,-0.57,3.81,5.82,4.02,-0.29,-2.38,-2.37,3.16,14.73,20.52,20.69,15.9,11.26,8.61,11.15,18.89,28.7,30.48,28.77,21.58,18.03,17.78,23.9,29.5,33.71,36.66,30.85,26.63,20.93,20.56,28.34,34.51,37.42,34.68,29,20.69,19.68,23.2,30.54,31.16,38.97,31.78,25.99,20.16,19.05,24.44,29.61,31.68,30.07,29.62,25.56,18.27,22.33,25.61,30.05,35.47,30.89,24.98,23.6,21.49,22.19,27.92,37.17,37.62,35.81,25.38,20.48,22.52,28.21,32.27,35.34,34.88,30.62,22.98,19.82,19.16,26.65,29.33,31.68,28.99,20.63,14.47,11.96,14.81,19.57,24.27,21.41,14.94,7.07,3.31,1.98,5.12,10.51,9.94,9.89,0.21,-7.76,-10.52,-11.25,-5.76,-2.66,-2.38,-4.79,-9.5,-16.24,-20.3,-13.61,-7.54,-10.42,-11.36,-11.32,-20.24,-24.28,-25.2,-12.84,-12.65,-9.55,-4.51,-15.78,-14.59,-19.74,-14.79,-5.23,-3.77,-1.66,-1.05,-8.27,-8.02,-10.32,-1.99,6.55,10.26,9.62,9.02,0.42,2.73,3.45,11.88,17.32,22.11,21.63,13.49,11.67,9.2,14.57,21.76,29.24,28.84,24.53,20.38,14.44,16.36,24.32,28.17,34.42,31.55,27.84,21.19,17.74,22.12,28.85,36.56</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B395" t="str">
+        <v>[R_22_标记]</v>
+      </c>
+      <c r="C395" t="str">
+        <v>幅值: 25.2uv 相位: 48.5°</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B396" t="str">
+        <v>[L_22_名字]</v>
+      </c>
+      <c r="C396" t="str">
+        <v>FERG(22)_lFlicker</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B397" t="str">
+        <v>[L_22_放大器]</v>
+      </c>
+      <c r="C397" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B398" t="str">
+        <v>[L_22_闪光]</v>
+      </c>
+      <c r="C398" t="str">
+        <v>f白色光:1000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B399" t="str">
+        <v>[L_22_闪光背景]</v>
+      </c>
+      <c r="C399" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B400" t="str">
+        <v>[L_22_采样]</v>
+      </c>
+      <c r="C400" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B401" t="str">
+        <v>[L_22_分析时间]</v>
+      </c>
+      <c r="C401" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B402" t="str">
+        <v>[L_22_数据长度]</v>
+      </c>
+      <c r="C402" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B403" t="str">
+        <v>[L_22_详细数据(uv)]</v>
+      </c>
+      <c r="C403" t="str">
+        <v>8.02,10.77,22.09,21.8,18.82,15.4,9.32,8.94,12.11,16.48,18.79,22.8,25.77,24.3,20.07,14.27,13.81,14.57,18.6,24.46,28.23,25.31,28.05,22.29,12.87,9.6,10.14,11.6,16.87,18.07,17.35,17,9.76,3.64,-2.15,-5.91,-4.73,-0.2,2.46,3.67,0.51,-5.56,-13.14,-19.41,-22.45,-22.6,-20.27,-15.62,-13.86,-16.31,-22.37,-27.4,-36.32,-38.37,-34.13,-35.17,-30.97,-28.29,-28.5,-30.86,-34.84,-41.28,-46.15,-44.12,-36.09,-33.51,-26.72,-27.31,-30.15,-36.6,-40.75,-41.98,-37.46,-32.65,-26.51,-17.97,-21.22,-21.2,-25.58,-28.24,-31.93,-29.38,-23.36,-16.9,-12.48,-8.04,-12.22,-12.42,-16.86,-19.3,-17.09,-10.96,-5.73,0.32,3.2,0.72,-6.31,-9.5,-13.14,-11.82,-7.26,-1.63,2.84,5.18,3.26,-1.26,-6.51,-10.39,-9.73,-5.64,-0.17,3.38,9.03,6.96,3.99,-1.89,-6.94,-4.01,-1.31,1.6,6.01,9.03,11.72,5.08,3.82,-0.71,-1.8,5.85,6,14.28,17.32,19.49,15.35,10.65,4.78,6.51,7.58,16.94,18.27,26.57,26.19,22.24,16.84,13.69,9.58,16.26,16.66,20.88,27.55,23.83,23.9,16.36,10.99,8.32,8.76,12.81,16.99,20.25,17.59,14.54,6.95,0.77,-2.45,-2.85,-0.3,3.36,5.54,4.31,-0.49,-6.97,-14.18,-18.13,-18.56,-16.14,-12.8,-10.93,-10.95,-14.26,-21.85,-29.15,-34.17,-32.58,-29.71,-25.49,-21.76,-21.91,-22.5,-26.95,-32.9,-35.05,-34.43,-29.78,-24.63,-23.02,-19.78,-26.27,-25.15,-29.56,-35.69,-33.82,-29.95,-25.62,-21.28,-15.21,-14.74,-21.63,-23.45,-30.57,-27.35,-23.65,-17.8,-9.65,-11.97,-11.72,-10.56,-15.16,-21.95,-20.34,-18.33,-10.86,-5.4,-3.31,-3.13,-7.03,-12.26,-15.97,-16.64,-13.32,-7.51,-1.53,1.89,2.12,-1.24,-5.86,-10.43,-10.96,-8.01,-3.28,5.5,9.78,7.13,3.82,3.22,1.03,-2.07,-0.99,8.18,10.84,16.44,18.15,16.95,13.48,8.16,8.9,12.86,20.17,26.34,31.1,30.2,24.79,20.16,20.39,16.58,16.94,26.3,29.88,34.61,35.4,30.66,27.84,18.99,18.48,20.83,19.23,27.36,31.82,29.94,27.81,20.23,12.94,10.48,11.45,10.89,16.07,17.47,17.99,14.11,6.11,-1.18,-5.65,-8.21,-6.86,-3.43,-0.94,-1.85,-5.08,-11.84,-19.11,-24.23,-28.19,-26.69,-22.63,-16.96,-18.08,-23.69,-29.81,-33.4,-36.52,-39.36,-39.89,-29.27,-29.75,-30.32,-28.49,-33.26,-38.5,-40.4,-44.61,-35.97,-31.44,-28.3,-24.36,-24.61,-25.97,-31.04,-33.97,-37.13,-33.39,-27.28,-16.24,-13.16,-11.05,-14.69,-21.03,-22.06,-22.39,-19.71,-11.98,-5.09,-3.99,-0.26,-4.98,-8.34,-9.85,-13.69,-10.23,-4.68,1.36,5.54,8.72,4.44,0.02,-4.37,-6.06,-4.17,0.7,6.37,11.02,13.52,10.85,4.14,0.69,-2.8,1.09,5.59,11.37,17.41,18.31,16.39,9.3,7.33,2.14,1.4,9.35,18.27,24.03,24.93,21.08,13.63,9.1,7.29,11.4,16,18.98,26.04,27.17,28.08,20.73,20.8,12.36,12.56,19.13,22.51,29.67,31.54,30.57,22.28,18.08,10.62,12.96,13.58,18.04,19.9,24.17,22.35,17.65,10.84,4.36,0.86,4.06,6.98,11.29,12.36,9.44,2.96,-3.29,-9.79,-12.36,-11.86,-8.46,-4.99,-3.75,-4.98,-10.74,-17.47,-23.93,-26.5,-24,-23.82,-17.49,-16.91,-15.47,-20.05,-26.82,-30.23,-34.13,-30.24,-25.39,-22.86,-20.93,-14.6,-22.45,-26.48,-31.15,-31.62,-27.93,-27.73,-21.87,-15.82,-9.61,-13.9,-21.21,-25.56,-26.22,-20.14,-14.2,-14.22,-7.3,-1.73,-2.8,-12.11,-15.22,-14.38,-15.5,-10.42,-5.64,-0.25,0.97,-1.14,-5.19,-10.03,-11.77,-11.47,-5.99,-2.01,2.85,5.59,3.54,-1.04,-5.99,-9.41,-8.26,-4.84,0.35,7.36,8.59,8.51,3.49,-0.71,-3.7,-5.07,0.11,5.41,10.61,16.07,15.08,9.81,7.06,0.55,5.5</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B404" t="str">
+        <v>[L_22_标记]</v>
+      </c>
+      <c r="C404" t="str">
+        <v>幅值: 23.1uv 相位: 49.4°</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B405" t="str">
+        <v>[R_23_名字]</v>
+      </c>
+      <c r="C405" t="str">
+        <v>FERG(23)_lCone</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B406" t="str">
+        <v>[R_23_放大器]</v>
+      </c>
+      <c r="C406" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B407" t="str">
+        <v>[R_23_闪光]</v>
+      </c>
+      <c r="C407" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B408" t="str">
+        <v>[R_23_闪光背景]</v>
+      </c>
+      <c r="C408" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B409" t="str">
+        <v>[R_23_采样]</v>
+      </c>
+      <c r="C409" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B410" t="str">
+        <v>[R_23_分析时间]</v>
+      </c>
+      <c r="C410" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B411" t="str">
+        <v>[R_23_数据长度]</v>
+      </c>
+      <c r="C411" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B412" t="str">
+        <v>[R_23_详细数据(uv)]</v>
+      </c>
+      <c r="C412" t="str">
+        <v>25.41,12.34,-1.52,0.76,15.71,23.83,14.25,-1.52,-4.16,9.08,20.87,15.72,-0.41,-7.69,2.55,16.86,16.67,1.75,-9.47,-3.21,12.24,17.02,4.78,-9.27,-7.61,7.48,16.76,8.39,-7.12,-10.21,3.04,15.93,12.24,-3.23,-10.77,-0.66,14.57,15.92,1.99,-9.28,-3.3,12.77,19.02,7.98,-5.95,-4.69,10.64,21.15,14.05,-1.18,-4.78,8.26,22.02,19.54,4.47,-3.73,5.81,21.27,23.6,10.18,-1.83,3.08,19,25.83,15.25,0.55,0.5,14.92,25.72,18.39,2.66,-2.62,8.57,21.46,19.52,2.79,-5.33,0.3,15.86,18.34,3.55,-9.46,-6.35,8.28,13.94,0.09,-15.34,-14.93,-1.46,7.11,0.5,-20.09,-25.98,-11.87,-0.26,0.03,-21.57,-31.96,-19.66,-7.87,-4.02,-21.57,-26.96,-27.42,-14.8,-5.79,-8.55,-25.54,-28.98,-15.7,-0.71,-2.44,-17.81,-24.84,-11.1,9.94,5.58,-4.3,-15.01,-8,14.44,23.96,13.38,-0.52,7.13,20.37,33.49,25.51,22.1,17.01,28.15,48.18,46.85,32,24.28,41.1,55.71,71.86,61.34,43.16,47.98,67.6,85.48,75.95,67.17,70.39,93.97,92.65,100.64,91.04,89.43,105.6,120.33,96.9,91.02,93.28,94.65,108.5,125.24,124.8,91.86,98.39,113.34,127.12,108.67,118.48,122.67,137.6,120.85,131.97,122.16,97.72,104.12,134.19,131.7,126.37,91.31,113.02,123.22,140.88,122.83,86.38,96.88,122.12,125.18,97.35,87.45,86.54,111.96,109.56,104.17,92.24,65.75,76.74,90.47,85.07,64.45,66.46,63.23,88.75,89.93,59.78,45.07,46.52,63.15,71.56,50.4,42.83,30.72,52.92,56.57,53.98,36.74,25.5,35.62,41.33,45.6,28.95,18.95,23.85,33.59,35,24.93,12.47,10.29,23.48,36.01,25.86,7.39,3.82,17.29,31.09,25.42,9.56,2.32,10.69,25.71,24.97,11.75,-0.25,4.29,20.4,25.72,13.6,-1.05,-0.42,14.41,24.01,16.11,-0.4,-4.4,8.58,20.98,17.43,0.77,-7.9,1.45,16.29,17.04,2.96,-9.34,-4.92,10.54,16.74,4.51,-10.8,-11.29,2.89,12.91,5.78,-10.74,-15.33,-4.6,9.66,5.17,-10.73,-20.15,-12.18,2.97,5.21,-7.36,-20.42,-16.91,-2.29,3.36,-6.49,-22.05,-21.8,-8.32,2.87,-3.29,-21.5,-27.38,-14.49,-0.31,-2.12,-18.02,-27.43,-18.18,-3.77,1.5,-14.6,-26.45,-24.73,-6.67,1.68,-10.32,-24.72,-25.99,-11.12,-0.24,-1.43,-21.54,-26.96,-16.23,-0.09,-1.89,-14.22,-26.05,-20.16,-3.25,1.03,-6.32,-25.59,-18.97,-3.15,1.03,-5.22,-17.87,-25.02,-6.6,2.89,1.86,-15.24,-20.55,-10.89,-0.62,3.42,-12.61,-21.42,-19.19,0.73,-1.49,-9.22,-28.76,-20.67,-12.17,-2.63,-3.93,-27.08,-25.33,-14.98,-3.68,-11.83,-24.74,-30.28,-23,-4.81,-8.94,-19.62,-36.33,-29.98,-17.77,-4.94,-19.65,-39.6,-37.49,-19.9,-7.68,-23.63,-40.14,-40.38,-29.19,-18.97,-19.69,-31.29,-43.54,-30.87,-17.11,-15.3,-29.92,-39.74,-32.94,-19.96,-16.92,-23.78,-41.46,-42.45,-28.8,-13.77,-17.26,-33.38,-44.99,-26.66,-12,-12.67,-30.27,-41.98,-29.13,-15.04,-10.54,-26.69,-39.23,-31.13,-18.71,-4.26,-15.18,-32.74,-32.15,-18.19,-4.4,-11.43,-22.33,-29.01,-16.15,-6.56,-1.44,-18.63,-26.78,-18.53,-1.65,2.07,-14.16,-23.25,-24.29,-3.41,5.16,-9.41,-18.51,-20.41,-8.83,0.75,-1.86,-17.02,-22.28,-16.34,2.67,-2.68,-12.26,-23.88,-17.86,-5.23,1.67,-9.15,-24.72,-25.11,-9.02,-0.93,-8.41,-24.26,-27.89,-16.61,-0.62,-6.16,-23.5,-31.7,-21.98,-3.88,-5.9,-20.29,-31.84,-23.74,-8.82,-4.89,-14.72,-30.21,-28.44,-12.43,-3.92,-11.98,-27.1,-29.12,-18.55,-3.5,-7.34,-20.58,-29.66,-19.99,-4.28,-1.99,-14.96,-27.05,-23.29,-6.22,1.08,-8.63,-22.95,-23.51,-8.7,3.89,-2.12,-18.25,-22.94,-10.08,4.11,3.56,-11.29,-20.48,-11.29,4.59</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B413" t="str">
+        <v>[R_23_标记]</v>
+      </c>
+      <c r="C413" t="str">
+        <v>a: 54.7ms -12.6uv b: 114.1ms 111.7uv</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B414" t="str">
+        <v>[L_23_名字]</v>
+      </c>
+      <c r="C414" t="str">
+        <v>FERG(23)_lCone</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B415" t="str">
+        <v>[L_23_放大器]</v>
+      </c>
+      <c r="C415" t="str">
+        <v>1-75 Hz</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B416" t="str">
+        <v>[L_23_闪光]</v>
+      </c>
+      <c r="C416" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B417" t="str">
+        <v>[L_23_闪光背景]</v>
+      </c>
+      <c r="C417" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B418" t="str">
+        <v>[L_23_采样]</v>
+      </c>
+      <c r="C418" t="str">
+        <v>刺激间隔:1.0S</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B419" t="str">
+        <v>[L_23_分析时间]</v>
+      </c>
+      <c r="C419" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B420" t="str">
+        <v>[L_23_数据长度]</v>
+      </c>
+      <c r="C420" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B421" t="str">
+        <v>[L_23_详细数据(uv)]</v>
+      </c>
+      <c r="C421" t="str">
+        <v>11.22,18.33,19.4,13.13,5.74,4.57,10.61,17.44,17.84,11.16,4,3.45,9.82,16.36,16.13,9.14,2.3,2.4,9.11,15.36,14.55,7.31,0.89,1.68,8.72,14.67,13.31,5.93,-0.02,1.48,8.83,14.47,12.59,5.12,-0.3,1.92,9.54,14.83,12.45,4.94,0.09,3,10.83,15.72,12.84,5.31,1.03,4.59,12.55,16.98,13.56,6.02,2.31,6.44,14.45,18.31,14.35,6.83,3.54,8.26,16.04,19.32,14.86,7.01,4.38,9.35,17.01,19.21,14.08,6.78,4.01,9.06,17,18.23,12.51,4.35,2.51,7.27,15.06,15.61,8.81,-0.4,-1.75,5.71,9.59,10.25,1.5,-3.31,-8.32,-0.06,7,1.53,-0.48,-10.37,-11.68,-4.52,3.94,-1.84,-5.91,-18.36,-19.47,-7.02,-4.4,-2.71,-13.64,-20.37,-11.76,-4.76,-2.71,-0.38,-11.6,-14.76,-3.92,0.82,2.46,3.01,3.42,-2.49,-2.18,10.07,16.84,17.79,10.78,10.68,14.32,24.61,30.14,27.93,27.1,24.77,33.73,44.56,47.33,43.95,38.46,42.37,53.24,59.43,60.17,62.84,57.47,49.76,60.78,75.07,90.06,76.24,72.61,82.21,84.9,102.89,108.24,96.08,93.92,80.85,91.75,113.27,116.88,100.55,95.71,93.9,101.15,132.95,125.93,129.49,107.34,120.15,133,122.46,144.26,112.82,122.11,129.4,134.09,127.29,137.22,116.35,123.05,120.16,130.61,124.98,123.81,135.16,110.39,129.95,122.07,119.29,120.6,126.99,105.73,98.2,119,116.11,120.99,107.5,102.48,94.49,99.24,96.51,91.4,86.69,71.3,78.48,86.65,85.41,85.41,74.95,70.36,72.38,68.76,82.05,71.72,52.94,46.77,50.12,59.86,61.32,54,45.67,37.66,40.71,51.22,54.97,43.04,38.68,30.32,33.58,40.3,40.84,33.3,29.41,25.89,30,35.38,35.87,26.88,21.24,18.44,22.76,29.04,30.76,24.39,14.75,14.02,20.45,28.2,28.48,20.45,13.57,13.62,18.96,25.81,24.17,16.83,10.77,11.12,17.47,23.73,21.91,14.81,8.23,9.01,15.78,21.69,19.15,12.26,6.01,7.23,14.4,19.83,16.4,9.05,3.06,6.18,13.13,16.61,14.48,5.99,1.95,4.74,11.04,14.91,10.93,3.1,-0.67,1.68,9.28,13.71,7.71,0.09,-3.31,0.98,6.86,12.29,6.52,-2.13,-4.72,-0.28,9.1,10.08,3.09,-2.68,-7.42,-1.96,5.73,8.7,2.5,-4.03,-5.39,1.7,8.88,6.27,0.36,-5.83,-6.3,-0.87,9.14,6.46,-0.07,-4.74,-3.84,-0.05,8.92,8.81,3.81,-6.07,-4.89,0.64,5.83,6.66,2.82,-6.31,-3.6,0.54,8.15,6.25,-2.18,-7.58,-4.61,1.27,6.26,9.94,-4.67,-4.29,-7.16,1.08,3.32,7.45,-2.67,-12.44,-7.86,-1.6,6.1,-1.02,-8.97,-6.52,-5.07,-0.78,0.12,5.28,-6.04,-9.28,-10.15,-1.99,3.96,-5.72,-11.76,-18.28,-10.64,0.53,3.22,-1.39,-9.88,-14.66,-11.8,0.13,1.09,-7,-11.2,-21.61,-15.81,-5.97,2.44,-9.11,-16.23,-16.48,-15.39,-0.11,-0.85,-3.96,-13.38,-21.39,-9.43,-2.72,2.82,-11.27,-14.3,-17.46,-12.37,-5.63,-3.61,-4.08,-8.48,-9.16,-7.72,4.69,2.17,-4.67,-15.14,-14.8,-3.69,7.18,6.49,-2,-7.95,-4.22,-2.13,2.7,4.14,-1.6,-5.81,-8.02,3.03,6.25,8.46,0.37,-6.35,-0.22,6.16,8.18,11.74,0.21,-4.09,-0.37,6.81,11.16,9.58,-0.87,-2.3,0.21,11.66,12.24,6.3,-1.35,-0.35,2.65,11.62,11.61,8.08,3.24,-2.89,1.95,8.61,14.37,8.5,1.49,-4.42,3.09,9.87,13.85,8.77,0.16,-3.66,4.48,11.06,10.77,6.3,-1.85,-0.81,4.7,10.59,13.05,5.05,-0.67,-0.41,4.88,12.62,12.99,5.84,0.24,-1.24,7.45,12.74,14.43,6.01,1.35,0.91,9.58,15.08,14.77,7.81,1.47,3.8,11.23,17.22,16.83,9.4,3.47,6.57,13.67,20.33</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B422" t="str">
+        <v>[L_23_标记]</v>
+      </c>
+      <c r="C422" t="str">
+        <v>a: 54.7ms -16.0uv b: 114.1ms 63.1uv</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B423" t="str">
+        <v>[R_24_名字]</v>
+      </c>
+      <c r="C423" t="str">
+        <v>FERG(24)_lFlicker</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B424" t="str">
+        <v>[R_24_放大器]</v>
+      </c>
+      <c r="C424" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B425" t="str">
+        <v>[R_24_闪光]</v>
+      </c>
+      <c r="C425" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B426" t="str">
+        <v>[R_24_闪光背景]</v>
+      </c>
+      <c r="C426" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B427" t="str">
+        <v>[R_24_采样]</v>
+      </c>
+      <c r="C427" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B428" t="str">
+        <v>[R_24_分析时间]</v>
+      </c>
+      <c r="C428" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B429" t="str">
+        <v>[R_24_数据长度]</v>
+      </c>
+      <c r="C429" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B430" t="str">
+        <v>[R_24_详细数据(uv)]</v>
+      </c>
+      <c r="C430" t="str">
+        <v>10.97,34.89,30.58,10.02,7.29,30.24,30.29,10.28,8.27,25.53,30.04,9.71,2.15,22.78,27.66,10.51,2.94,25.44,30.73,10.7,4.45,22.85,30.87,10.02,2.39,25.16,28.41,8.33,3.43,23.04,28.72,9.09,2.19,24.35,27.66,7.55,2.71,20.55,27.5,7.54,-1.06,19.22,24.38,3.1,-3.41,13.22,20.08,1.35,-8,8.74,15.25,-4.4,-16.69,2.12,12.91,-9.97,-18.81,-4.8,7.78,-12.81,-26.01,-5.21,4.41,-17.05,-26.68,-13.56,-2.57,-20.87,-32.73,-15.51,-6.74,-19.61,-35.2,-15.16,-1.69,-23.38,-29.64,-12.74,-4.36,-19.64,-27.9,-12.73,2.45,-15.93,-27.67,-8.3,4.4,-11.26,-22.71,-3.57,11.35,-5.36,-15.77,0.57,15.34,2.49,-9.98,5.22,21.39,6.78,-4.39,10.73,24.63,11.58,-1.46,14.4,30.59,14.99,3.05,15.98,33.01,19.66,6.12,20.76,34.21,21.09,5.91,22.5,37.22,24.35,8.98,23.43,36.88,23.8,8.69,23.69,41.16,26.72,11.2,24.25,36.24,25.23,7.89,18.94,39.88,29.68,8.18,21.46,41.18,32.34,11.04,19.24,41.2,29.88,11.43,20.55,38.23,28.36,10.88,18.48,37.29,27.46,9.67,18.89,35.35,27.16,5.66,15.09,31.2,23.21,2.08,7.96,27.83,18.8,-4.83,4.06,20.47,10.82,-8.24,-2.91,12.96,3.28,-16.96,-13.58,6.2,-0.85,-27.04,-20.56,-2.95,-8.69,-29.86,-30.55,-9.85,-16.31,-37.7,-36.43,-15.48,-20.2,-43.09,-39.38,-20.26,-24.01,-40.45,-42.4,-22.75,-20.3,-41.02,-37.38,-16.25,-20.15,-41.67,-36.67,-17,-14.6,-33.71,-31.59,-7.55,-10.66,-27.57,-24.58,0.14,0.3,-17.52,-14.38,8.42,10.37,-10.16,-6.71,15.91,18.02,0.16,-0.53,23.47,25.96,5.89,7.26,28.48,33.14,13.34,11.06,34.06,35.3,16.95,15.3,35.68,40.09,18.03,15.97,36.4,37.82,18.75,15.47,36.1,41.54,16.88,13.07,33.06,38.74,17.93,10.29,32.72,36.81,14.53,8.58,27.62,33.2,13.29,1.76,26.82,30.64,6.96,1.13,19.95,24.22,8.6,0.59,17.43,24.82,7.06,-3.42,16.98,24.16,4.17,-4.75,13.07,20.73,3.61,-5.74,12.38,19.68,1.8,-8.25,10.57,18.04,-1.75,-9.99,8.37,15.94,-4.96,-12.72,3.03,11.73,-8.48,-17.42,0.79,8.5,-8.72,-20.39,-3.38,4.85,-11.86,-25.5,-10.82,-0.23,-15.61,-30.61,-15.73,-1.47,-20.5,-34.67,-18.04,-5.42,-19.88,-32.58,-19.44,-5.21,-27.14,-38.83,-22.49,-3.09,-23.51,-38.14,-19.79,-4.5,-18.48,-33.83,-14.48,-1.74,-15.55,-29.74,-17.32,-0.02,-11.38,-26.2,-9.74,5.96,-7.47,-20.21,-6.4,11.68,-1.07,-16.37,-1.72,16.71,4.15,-9.99,2.22,19.05,8.06,-7.51,7.56,24.54,11.65,-4.67,7.71,27.19,12.67,-3.37,9.54,29.06,13.76,-1.34,9.15,28.67,18.11,-1.54,10.68,29.45,14.74,-4.29,7.64,28.84,18.79,-1.5,10.62,25.42,19.01,-2.53,8.66,23.79,17.19,-2.23,5.28,24.84,16.28,-0.83,7.62,30.94,18.56,3.11,9.21,25.9,20.76,3.06,8.77,28.4,24.19,1.13,8.19,29.34,22.68,3.9,9.05,29.13,22.72,1.68,7.12,27.82,21.86,0.01,4.11,24.31,19.46,-4.57,1.81,19.34,12.13,-7.02,-6.82,12.71,10.1,-12.59,-11.12,7.02,1.47,-23.42,-19.37,-1.99,-8.62,-26.99,-29.28,-11.46,-15.35,-34.08,-33.55,-15.31,-19.03,-40.39,-41.95,-21.53,-22.33,-43.92,-43.9,-21.34,-27.11,-43.89,-46,-25.94,-26.96,-48.76,-46,-22.43,-20.29,-40.63,-41.23,-18.54,-15.64,-35.4,-38.4,-13.6,-10.27,-30.63,-30.84,-6.85,-1.69,-20.59,-22.36,-0.41,5.46,-14.39,-14.51,8.29,12.56,-5.98,-6.4,15.36,18.99,0.48,-3.58,19.36,26.76,6.18,4.84,22.45,29.59,12.99,4.99,27.83,31.86,14.27,10.79,26.69,36.9,15.68,9.64,29,33.05,18.33,8.44,24.19</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B431" t="str">
+        <v>[R_24_标记]</v>
+      </c>
+      <c r="C431" t="str">
+        <v>幅值: 21.6uv 相位: 49.5°</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B432" t="str">
+        <v>[L_24_名字]</v>
+      </c>
+      <c r="C432" t="str">
+        <v>FERG(24)_lFlicker</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B433" t="str">
+        <v>[L_24_放大器]</v>
+      </c>
+      <c r="C433" t="str">
+        <v>1-300 Hz</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B434" t="str">
+        <v>[L_24_闪光]</v>
+      </c>
+      <c r="C434" t="str">
+        <v>f白色光:2000.0cd.m-2,5ms</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B435" t="str">
+        <v>[L_24_闪光背景]</v>
+      </c>
+      <c r="C435" t="str">
+        <v>b白色光:30.0cd.m-2</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B436" t="str">
+        <v>[L_24_采样]</v>
+      </c>
+      <c r="C436" t="str">
+        <v>刺激频率:20.0Hz</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B437" t="str">
+        <v>[L_24_分析时间]</v>
+      </c>
+      <c r="C437" t="str">
+        <v>200ms</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B438" t="str">
+        <v>[L_24_数据长度]</v>
+      </c>
+      <c r="C438" t="str">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B439" t="str">
+        <v>[L_24_详细数据(uv)]</v>
+      </c>
+      <c r="C439" t="str">
+        <v>16.26,9.89,-3.43,-3.9,12.63,15.24,6.33,-6.27,3.53,14.61,10.62,-6.85,-0.11,13.99,17.3,-1.81,-7.04,4.4,11.34,0.49,-9.8,-4.11,7.81,4.71,-10.31,-11.94,0.45,3.32,-9.88,-20.21,-11.83,-2.35,-10.75,-25.89,-24.42,-11.25,-11.55,-27.99,-34.15,-21.65,-14.95,-26.75,-40.95,-31.47,-19.27,-27.26,-42.19,-41.49,-31,-22.78,-37.61,-44.64,-37.37,-27.18,-33.99,-50.61,-41.51,-25.56,-28.16,-42.33,-45.98,-31.03,-23.73,-35.25,-44.22,-33.18,-23.89,-25.56,-37.24,-35.18,-21.05,-14.66,-28.16,-37.14,-21.85,-14.62,-22.18,-32.32,-26.79,-12.99,-11.79,-26.67,-29.04,-14.35,-7.61,-19.06,-27.98,-17.11,-4.39,-8.89,-24.52,-22.12,-7.22,-4.02,-17.96,-24.82,-12.39,-2.64,-10.61,-24.08,-16.65,-2.3,-4.32,-17.32,-22.29,-5.73,0.31,-11.06,-19.56,-10.57,2.39,-3.72,-19.36,-12.45,0.9,3.8,-5.63,-11.93,-2.04,13.12,2.18,-8.96,-4.42,12.66,11.61,-5.38,-1.42,13.28,19.07,3.9,-2.23,10.73,19.03,16.88,2.1,5.88,17.61,20.78,4.88,3.36,14.44,23.18,11.94,0.72,5.1,17.12,16.05,-0.14,-1.14,9.71,13.57,-1.76,-9.11,-0.52,8.73,-0.74,-15.47,-13.51,-1.59,-3.69,-19.46,-26.48,-14.39,-8.54,-21.58,-34.62,-28.46,-17.62,-24.35,-40.35,-42.77,-28.31,-29.28,-42.08,-49.87,-39.47,-27.9,-38.48,-53.94,-49.78,-33.45,-36.63,-49.17,-56.42,-37.73,-33.19,-46.02,-51.83,-47.03,-34.08,-37.64,-51.71,-47.54,-30.3,-30.55,-43.47,-48.5,-35.89,-20.24,-31.36,-40.78,-33.94,-19.34,-19.54,-33.31,-34.96,-20.04,-11.09,-22.96,-34.04,-21.55,-7.46,-12.34,-25.97,-22.43,-5.85,-3.72,-16.25,-22.28,-9.15,2.04,-7.27,-18.62,-11.96,3.36,1.32,-11.57,-12.96,1.49,7.6,-5.31,-13.7,-3.39,12.26,7.01,-10.28,-4.94,11.12,9.91,-3,-8.73,9.6,18.18,8.47,-3.8,2.47,16.23,17.82,2.31,0.81,13.93,20.82,6.03,-1.98,8.83,21.46,12.12,-0.39,1.56,17.45,21.53,4.74,-0.22,11.26,16.68,5.33,-1.7,3.13,13.81,9.23,-8.4,-6.78,3.54,7.3,-8.89,-16.45,-5.98,1.66,-7.96,-22.74,-19.18,-7.1,-9.8,-26.81,-31.71,-19.89,-14.93,-28.59,-39.72,-34.35,-22.18,-28.76,-44.8,-44.44,-31.65,-28.93,-43.39,-52.72,-41.26,-29.82,-39.23,-50.47,-48.35,-32.85,-35,-46.77,-52.66,-35.32,-29.09,-41.76,-48.6,-39.56,-25.62,-33.15,-47.66,-42.65,-27.11,-19.85,-38.6,-37.78,-28.12,-15.47,-22.97,-37.88,-28.5,-14.44,-15.82,-25.55,-28.8,-12.9,-8.14,-17.21,-27.38,-13.9,-3.55,-7.1,-21.21,-18.45,-3.3,-1.24,-14.15,-20.97,-7.34,2.43,-8.44,-19.4,-12.87,1.36,-2.23,-16.35,-18.3,-4.04,1.33,-10.24,-20.91,-8.36,2.61,-6.54,-17.84,-16.22,2.89,0.64,-11.39,-17.27,-3.66,5.52,-3.89,-15.52,-6.03,7.91,4.97,-13.87,-9.81,3.5,9.4,-2.36,-12.04,4.14,14.94,7.8,-5.31,1.31,11.33,15.43,-0.45,-4.75,11.89,19.13,3.71,-3.34,4.79,13.92,11.34,-4.29,-5.47,10.43,11.25,-0.79,-8.46,-0.11,10.71,2.36,-13,-9.84,3.78,0.46,-15.33,-19.69,-7.15,-2.72,-15.46,-28.14,-20.2,-9.13,-17.25,-33.61,-32.24,-17.61,-16.83,-31.61,-40.87,-29.26,-21.01,-33.5,-43.6,-41.04,-26.26,-32.13,-44.61,-47.86,-34.67,-25.42,-44.11,-49.72,-39.59,-32.01,-32.63,-46.47,-43.71,-30.23,-26.28,-40.54,-45.5,-35.42,-23.27,-34.38,-43.47,-33.81,-21.67,-22.83,-38.68,-39.45,-23.51,-17.86,-29.43,-38.04,-26.27,-15.03,-18.48,-32.45,-26.92,-12.14,-12.79,-24.71,-27.82,-15.6,-5.67,-16.93,-27.11,-19.02,-4.32,-8.11,-21.21,-21.13,-5.07,-1.09,-14.91,-20.57,-9.02,1.05,-5,-18.26,-11.53,0.99,3.88,-7.76,-13.46,4.16,13.69,-3.23,-10.52,0.58,16.62,10.37,-1.48,0.81,16.25,20.74,2.18,-0.6</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>FERG</v>
+      </c>
+      <c r="B440" t="str">
+        <v>[L_24_标记]</v>
+      </c>
+      <c r="C440" t="str">
+        <v>幅值: 21.5uv 相位: 47.9°</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C440"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>